<commit_message>
climate data: 2026-05-06 23:44 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1117,6 +1117,320 @@
       </c>
       <c r="J21" s="5" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-06T14:00</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>1012.9</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>1522.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06T15:00</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>1012.1</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>2562.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-06T16:00</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>1011.5</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>717.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06T17:00</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>1011.2</v>
+      </c>
+      <c r="J25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-06T18:00</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>1011.2</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>752.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06T19:00</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>1011.2</v>
+      </c>
+      <c r="J27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-06T20:00</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>1011.6</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06T21:00</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>1012</v>
+      </c>
+      <c r="J29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-06T22:00</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>1012</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06T23:00</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>1011.9</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-07 03:53 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1431,130 @@
         <v>0</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T00:00</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>1011.8</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T01:00</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>1011.6</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T02:00</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>1011.3</v>
+      </c>
+      <c r="J34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T03:00</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>1011</v>
+      </c>
+      <c r="J35" s="5" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-07 23:49 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,14 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +79,12 @@
         <bgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+        <bgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -94,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -109,6 +121,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -476,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1555,6 +1570,678 @@
       </c>
       <c r="J35" s="5" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T09:00</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T10:00</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>1010</v>
+      </c>
+      <c r="K36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T10:00</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T11:00</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>2546.6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T11:00</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T12:00</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="K38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T12:00</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T13:00</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>1009.9</v>
+      </c>
+      <c r="K39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T13:00</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T14:00</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>1009.7</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>2575.6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T14:00</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T15:00</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>1009.4</v>
+      </c>
+      <c r="K41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T15:00</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T16:00</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>1009</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>2993.8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T16:00</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T17:00</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>1008.8</v>
+      </c>
+      <c r="K43" s="5" t="n">
+        <v>2433.1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T17:00</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T18:00</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>1009.1</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>1737.7</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T18:00</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T19:00</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>1009.4</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T19:00</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T20:00</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>1009.7</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>271.7</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T20:00</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T21:00</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="n">
+        <v>1010.5</v>
+      </c>
+      <c r="K47" s="5" t="n">
+        <v>32.3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T21:00</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T22:00</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>1011.3</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T22:00</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:00</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="n">
+        <v>1011.5</v>
+      </c>
+      <c r="K49" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:00</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T00:00</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="n">
+        <v>1011.1</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07T04:00</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="6" t="n"/>
+      <c r="K51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07T05:00</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="6" t="n"/>
+      <c r="K52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07T06:00</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="6" t="n"/>
+      <c r="K53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07T07:00</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="6" t="n"/>
+      <c r="K54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07T08:00</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="6" t="n"/>
+      <c r="J55" s="6" t="n"/>
+      <c r="K55" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-08 03:43 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2242,6 +2242,154 @@
       <c r="J55" s="6" t="n"/>
       <c r="K55" s="6" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T00:00</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T01:00</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>1010.6</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T01:00</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T02:00</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E57" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="5" t="n"/>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="n">
+        <v>1010.3</v>
+      </c>
+      <c r="K57" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T02:00</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T03:00</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T03:00</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T04:00</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="5" t="n"/>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="K59" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-08 23:52 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2390,6 +2390,606 @@
         <v>0</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T04:00</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>1008.9</v>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T09:00</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D61" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>1009.6</v>
+      </c>
+      <c r="J61" s="5" t="n">
+        <v>1473.4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T10:00</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>1009.6</v>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>1467.1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:00</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D63" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>1018.9</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:00</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>1010.1</v>
+      </c>
+      <c r="J64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:00</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D65" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="E65" s="5" t="n"/>
+      <c r="F65" s="5" t="n"/>
+      <c r="G65" s="5" t="n"/>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="J65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T14:00</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>1354.2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T15:00</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D67" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="E67" s="5" t="n"/>
+      <c r="F67" s="5" t="n"/>
+      <c r="G67" s="5" t="n"/>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>1009.2</v>
+      </c>
+      <c r="J67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T16:00</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>1008.1</v>
+      </c>
+      <c r="J68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T17:00</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="E69" s="5" t="n"/>
+      <c r="F69" s="5" t="n"/>
+      <c r="G69" s="5" t="n"/>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="n">
+        <v>1007.9</v>
+      </c>
+      <c r="J69" s="5" t="n">
+        <v>499.3</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T18:00</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>1007.4</v>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>851.2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T19:00</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D71" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="E71" s="5" t="n"/>
+      <c r="F71" s="5" t="n"/>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>1007.2</v>
+      </c>
+      <c r="J71" s="5" t="n">
+        <v>323.8</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T20:00</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>1007.1</v>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T21:00</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="D73" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="E73" s="5" t="n"/>
+      <c r="F73" s="5" t="n"/>
+      <c r="G73" s="5" t="n"/>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>1007.2</v>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08T22:00</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>1006.7</v>
+      </c>
+      <c r="J74" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-08T23:00</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D75" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="E75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
+      <c r="G75" s="5" t="n"/>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>1006</v>
+      </c>
+      <c r="J75" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08T05:00</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08T06:00</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
+      <c r="I77" s="6" t="n"/>
+      <c r="J77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08T07:00</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08T08:00</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-09 03:46 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2990,6 +2990,134 @@
       <c r="I79" s="6" t="n"/>
       <c r="J79" s="6" t="n"/>
     </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T00:00</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>1005.8</v>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T01:00</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D81" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E81" s="5" t="n"/>
+      <c r="F81" s="5" t="n"/>
+      <c r="G81" s="5" t="n"/>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="n">
+        <v>1006.4</v>
+      </c>
+      <c r="J81" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T02:00</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="n">
+        <v>1005.7</v>
+      </c>
+      <c r="J82" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T03:00</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D83" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="E83" s="5" t="n"/>
+      <c r="F83" s="5" t="n"/>
+      <c r="G83" s="5" t="n"/>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>1005.5</v>
+      </c>
+      <c r="J83" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-09 23:41 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3118,6 +3118,574 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T08:00</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="n"/>
+      <c r="J84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T09:00</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D85" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="E85" s="5" t="n"/>
+      <c r="F85" s="5" t="n"/>
+      <c r="G85" s="5" t="n"/>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="n">
+        <v>1003.8</v>
+      </c>
+      <c r="J85" s="5" t="n">
+        <v>910.8</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T10:00</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="E86" s="4" t="n"/>
+      <c r="F86" s="4" t="n"/>
+      <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="n">
+        <v>1004</v>
+      </c>
+      <c r="J86" s="4" t="n">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T12:00</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D87" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="E87" s="5" t="n"/>
+      <c r="F87" s="5" t="n"/>
+      <c r="G87" s="5" t="n"/>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="n">
+        <v>1004.3</v>
+      </c>
+      <c r="J87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T13:00</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I88" s="4" t="n">
+        <v>1003.7</v>
+      </c>
+      <c r="J88" s="4" t="n">
+        <v>1350.3</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T14:00</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D89" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="E89" s="5" t="n"/>
+      <c r="F89" s="5" t="n"/>
+      <c r="G89" s="5" t="n"/>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="n">
+        <v>1003.5</v>
+      </c>
+      <c r="J89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T15:00</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D90" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="E90" s="4" t="n"/>
+      <c r="F90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>1004.8</v>
+      </c>
+      <c r="J90" s="4" t="n">
+        <v>126.2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T16:00</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D91" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="E91" s="5" t="n"/>
+      <c r="F91" s="5" t="n"/>
+      <c r="G91" s="5" t="n"/>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="n">
+        <v>1005.2</v>
+      </c>
+      <c r="J91" s="5" t="n">
+        <v>680.7</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T17:00</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I92" s="4" t="n">
+        <v>1005.5</v>
+      </c>
+      <c r="J92" s="4" t="n">
+        <v>140.6</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T18:00</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D93" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="E93" s="5" t="n"/>
+      <c r="F93" s="5" t="n"/>
+      <c r="G93" s="5" t="n"/>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="n">
+        <v>1005.9</v>
+      </c>
+      <c r="J93" s="5" t="n">
+        <v>679.2</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-09T19:00</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D94" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="E94" s="4" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I94" s="4" t="n">
+        <v>1006.5</v>
+      </c>
+      <c r="J94" s="4" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-09T20:00</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D95" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="E95" s="5" t="n"/>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="n"/>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="n">
+        <v>1007.6</v>
+      </c>
+      <c r="J95" s="5" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T04:00</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="6" t="n"/>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="6" t="n"/>
+      <c r="I96" s="6" t="n"/>
+      <c r="J96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T05:00</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
+      <c r="I97" s="6" t="n"/>
+      <c r="J97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T06:00</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
+      <c r="F98" s="6" t="n"/>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="6" t="n"/>
+      <c r="I98" s="6" t="n"/>
+      <c r="J98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T07:00</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n"/>
+      <c r="I99" s="6" t="n"/>
+      <c r="J99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T11:00</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
+      <c r="F100" s="6" t="n"/>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="6" t="n"/>
+      <c r="I100" s="6" t="n"/>
+      <c r="J100" s="6" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T21:00</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n"/>
+      <c r="I101" s="6" t="n"/>
+      <c r="J101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T22:00</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="n"/>
+      <c r="E102" s="6" t="n"/>
+      <c r="F102" s="6" t="n"/>
+      <c r="G102" s="6" t="n"/>
+      <c r="H102" s="6" t="n"/>
+      <c r="I102" s="6" t="n"/>
+      <c r="J102" s="6" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-09T23:00</t>
+        </is>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="n"/>
+      <c r="E103" s="6" t="n"/>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="6" t="n"/>
+      <c r="H103" s="6" t="n"/>
+      <c r="I103" s="6" t="n"/>
+      <c r="J103" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-10 04:02 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3686,6 +3686,102 @@
       <c r="I103" s="6" t="n"/>
       <c r="J103" s="6" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T00:00</t>
+        </is>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="n"/>
+      <c r="E104" s="6" t="n"/>
+      <c r="F104" s="6" t="n"/>
+      <c r="G104" s="6" t="n"/>
+      <c r="H104" s="6" t="n"/>
+      <c r="I104" s="6" t="n"/>
+      <c r="J104" s="6" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T01:00</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="6" t="n"/>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T02:00</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="n"/>
+      <c r="E106" s="6" t="n"/>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="6" t="n"/>
+      <c r="H106" s="6" t="n"/>
+      <c r="I106" s="6" t="n"/>
+      <c r="J106" s="6" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T03:00</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="n"/>
+      <c r="E107" s="6" t="n"/>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="6" t="n"/>
+      <c r="H107" s="6" t="n"/>
+      <c r="I107" s="6" t="n"/>
+      <c r="J107" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-10 13:03 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3782,6 +3782,256 @@
       <c r="I107" s="6" t="n"/>
       <c r="J107" s="6" t="n"/>
     </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T09:00</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D108" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="n">
+        <v>1009.1</v>
+      </c>
+      <c r="J108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T10:00</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D109" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="E109" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="5" t="n"/>
+      <c r="G109" s="5" t="n"/>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I109" s="5" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="J109" s="5" t="n">
+        <v>1801.3</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T11:00</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D110" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>1009.2</v>
+      </c>
+      <c r="J110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T12:00</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D111" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="E111" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="5" t="n"/>
+      <c r="G111" s="5" t="n"/>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="n">
+        <v>1009.4</v>
+      </c>
+      <c r="J111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T04:00</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="n"/>
+      <c r="E112" s="6" t="n"/>
+      <c r="F112" s="6" t="n"/>
+      <c r="G112" s="6" t="n"/>
+      <c r="H112" s="6" t="n"/>
+      <c r="I112" s="6" t="n"/>
+      <c r="J112" s="6" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T05:00</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="n"/>
+      <c r="E113" s="6" t="n"/>
+      <c r="F113" s="6" t="n"/>
+      <c r="G113" s="6" t="n"/>
+      <c r="H113" s="6" t="n"/>
+      <c r="I113" s="6" t="n"/>
+      <c r="J113" s="6" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T06:00</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="n"/>
+      <c r="E114" s="6" t="n"/>
+      <c r="F114" s="6" t="n"/>
+      <c r="G114" s="6" t="n"/>
+      <c r="H114" s="6" t="n"/>
+      <c r="I114" s="6" t="n"/>
+      <c r="J114" s="6" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T07:00</t>
+        </is>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="n"/>
+      <c r="E115" s="6" t="n"/>
+      <c r="F115" s="6" t="n"/>
+      <c r="G115" s="6" t="n"/>
+      <c r="H115" s="6" t="n"/>
+      <c r="I115" s="6" t="n"/>
+      <c r="J115" s="6" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-10T08:00</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="n"/>
+      <c r="E116" s="6" t="n"/>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="H116" s="6" t="n"/>
+      <c r="I116" s="6" t="n"/>
+      <c r="J116" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-10 23:45 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4032,6 +4032,376 @@
       <c r="I116" s="6" t="n"/>
       <c r="J116" s="6" t="n"/>
     </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T13:00</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D117" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="E117" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F117" s="5" t="n"/>
+      <c r="G117" s="5" t="n"/>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I117" s="5" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="J117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T14:00</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D118" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="J118" s="4" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T15:00</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D119" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" s="5" t="n"/>
+      <c r="G119" s="5" t="n"/>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="n">
+        <v>1009</v>
+      </c>
+      <c r="J119" s="5" t="n">
+        <v>915.3</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T16:00</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="D120" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="n">
+        <v>1009.3</v>
+      </c>
+      <c r="J120" s="4" t="n">
+        <v>432.2</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T17:00</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="D121" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="E121" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F121" s="5" t="n"/>
+      <c r="G121" s="5" t="n"/>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I121" s="5" t="n">
+        <v>1008.9</v>
+      </c>
+      <c r="J121" s="5" t="n">
+        <v>457.2</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T18:00</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="D122" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F122" s="4" t="n"/>
+      <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="n">
+        <v>1009</v>
+      </c>
+      <c r="J122" s="4" t="n">
+        <v>235.9</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T19:00</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D123" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="E123" s="5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F123" s="5" t="n"/>
+      <c r="G123" s="5" t="n"/>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I123" s="5" t="n">
+        <v>1008.9</v>
+      </c>
+      <c r="J123" s="5" t="n">
+        <v>41.6</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T20:00</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D124" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F124" s="4" t="n"/>
+      <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="n">
+        <v>1009.1</v>
+      </c>
+      <c r="J124" s="4" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T21:00</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D125" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="E125" s="5" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F125" s="5" t="n"/>
+      <c r="G125" s="5" t="n"/>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I125" s="5" t="n">
+        <v>1009.8</v>
+      </c>
+      <c r="J125" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-10T22:00</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D126" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="n">
+        <v>1010.4</v>
+      </c>
+      <c r="J126" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-10T23:00</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="D127" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="E127" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" s="5" t="n"/>
+      <c r="G127" s="5" t="n"/>
+      <c r="H127" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I127" s="5" t="n">
+        <v>1010.6</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-11 04:13 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4402,6 +4402,112 @@
         <v>0</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T00:00</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D128" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="n">
+        <v>1010.7</v>
+      </c>
+      <c r="J128" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T01:00</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="n"/>
+      <c r="E129" s="6" t="n"/>
+      <c r="F129" s="6" t="n"/>
+      <c r="G129" s="6" t="n"/>
+      <c r="H129" s="6" t="n"/>
+      <c r="I129" s="6" t="n"/>
+      <c r="J129" s="6" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T02:00</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="n"/>
+      <c r="E130" s="6" t="n"/>
+      <c r="F130" s="6" t="n"/>
+      <c r="G130" s="6" t="n"/>
+      <c r="H130" s="6" t="n"/>
+      <c r="I130" s="6" t="n"/>
+      <c r="J130" s="6" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T03:00</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="n"/>
+      <c r="E131" s="6" t="n"/>
+      <c r="F131" s="6" t="n"/>
+      <c r="G131" s="6" t="n"/>
+      <c r="H131" s="6" t="n"/>
+      <c r="I131" s="6" t="n"/>
+      <c r="J131" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-11 23:53 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4508,6 +4508,628 @@
       <c r="I131" s="6" t="n"/>
       <c r="J131" s="6" t="n"/>
     </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T09:00</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D132" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" s="4" t="n"/>
+      <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I132" s="4" t="n">
+        <v>1012.7</v>
+      </c>
+      <c r="J132" s="4" t="n">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T10:00</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D133" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="E133" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" s="5" t="n"/>
+      <c r="G133" s="5" t="n"/>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I133" s="5" t="n">
+        <v>1013.1</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>999.9</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T11:00</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D134" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I134" s="4" t="n">
+        <v>1013.4</v>
+      </c>
+      <c r="J134" s="4" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T12:00</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D135" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="E135" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F135" s="5" t="n"/>
+      <c r="G135" s="5" t="n"/>
+      <c r="H135" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I135" s="5" t="n">
+        <v>1013.1</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>984.3</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T13:00</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D136" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I136" s="4" t="n">
+        <v>1013.3</v>
+      </c>
+      <c r="J136" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T14:00</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D137" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="5" t="n"/>
+      <c r="G137" s="5" t="n"/>
+      <c r="H137" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="J137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T15:00</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D138" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E138" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I138" s="4" t="n">
+        <v>1013</v>
+      </c>
+      <c r="J138" s="4" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T16:00</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D139" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="5" t="n"/>
+      <c r="G139" s="5" t="n"/>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>1012.8</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>2265</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T17:00</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D140" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I140" s="4" t="n">
+        <v>1013</v>
+      </c>
+      <c r="J140" s="4" t="n">
+        <v>1471.8</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T18:00</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D141" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" s="5" t="n"/>
+      <c r="G141" s="5" t="n"/>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>1013.2</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T19:00</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D142" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" s="4" t="n"/>
+      <c r="G142" s="4" t="n"/>
+      <c r="H142" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I142" s="4" t="n">
+        <v>1013.6</v>
+      </c>
+      <c r="J142" s="4" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T20:00</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="5" t="n"/>
+      <c r="G143" s="5" t="n"/>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>1014.2</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>75.2</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T21:00</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D144" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" s="4" t="n"/>
+      <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I144" s="4" t="n">
+        <v>1015</v>
+      </c>
+      <c r="J144" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11T22:00</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D145" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" s="5" t="n"/>
+      <c r="G145" s="5" t="n"/>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>1015.8</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11T23:00</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D146" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E146" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" s="4" t="n"/>
+      <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I146" s="4" t="n">
+        <v>1016.1</v>
+      </c>
+      <c r="J146" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T04:00</t>
+        </is>
+      </c>
+      <c r="B147" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="n"/>
+      <c r="E147" s="6" t="n"/>
+      <c r="F147" s="6" t="n"/>
+      <c r="G147" s="6" t="n"/>
+      <c r="H147" s="6" t="n"/>
+      <c r="I147" s="6" t="n"/>
+      <c r="J147" s="6" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T05:00</t>
+        </is>
+      </c>
+      <c r="B148" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C148" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D148" s="6" t="n"/>
+      <c r="E148" s="6" t="n"/>
+      <c r="F148" s="6" t="n"/>
+      <c r="G148" s="6" t="n"/>
+      <c r="H148" s="6" t="n"/>
+      <c r="I148" s="6" t="n"/>
+      <c r="J148" s="6" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T06:00</t>
+        </is>
+      </c>
+      <c r="B149" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D149" s="6" t="n"/>
+      <c r="E149" s="6" t="n"/>
+      <c r="F149" s="6" t="n"/>
+      <c r="G149" s="6" t="n"/>
+      <c r="H149" s="6" t="n"/>
+      <c r="I149" s="6" t="n"/>
+      <c r="J149" s="6" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T07:00</t>
+        </is>
+      </c>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D150" s="6" t="n"/>
+      <c r="E150" s="6" t="n"/>
+      <c r="F150" s="6" t="n"/>
+      <c r="G150" s="6" t="n"/>
+      <c r="H150" s="6" t="n"/>
+      <c r="I150" s="6" t="n"/>
+      <c r="J150" s="6" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-11T08:00</t>
+        </is>
+      </c>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="n"/>
+      <c r="E151" s="6" t="n"/>
+      <c r="F151" s="6" t="n"/>
+      <c r="G151" s="6" t="n"/>
+      <c r="H151" s="6" t="n"/>
+      <c r="I151" s="6" t="n"/>
+      <c r="J151" s="6" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-12 03:57 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K151"/>
+  <dimension ref="A1:K155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5130,6 +5130,142 @@
       <c r="I151" s="6" t="n"/>
       <c r="J151" s="6" t="n"/>
     </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-12T00:00</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="D152" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E152" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" s="4" t="n"/>
+      <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I152" s="4" t="n">
+        <v>1016.2</v>
+      </c>
+      <c r="J152" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12T01:00</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="D153" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="E153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="5" t="n"/>
+      <c r="G153" s="5" t="n"/>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I153" s="5" t="n">
+        <v>1016.2</v>
+      </c>
+      <c r="J153" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-12T02:00</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D154" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="E154" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" s="4" t="n"/>
+      <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I154" s="4" t="n">
+        <v>1016.3</v>
+      </c>
+      <c r="J154" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12T03:00</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D155" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="E155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" s="5" t="n"/>
+      <c r="G155" s="5" t="n"/>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="n">
+        <v>1016</v>
+      </c>
+      <c r="J155" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-12 23:55 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J155"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -5239,6 +5239,346 @@
         <v>671</v>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12T14:00</t>
+        </is>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D156" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E156" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F156" s="8" t="n"/>
+      <c r="G156" s="8" t="n"/>
+      <c r="H156" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I156" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J156" s="8" t="n">
+        <v>568.7</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-12T15:00</t>
+        </is>
+      </c>
+      <c r="B157" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D157" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="E157" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F157" s="9" t="n"/>
+      <c r="G157" s="9" t="n"/>
+      <c r="H157" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I157" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J157" s="9" t="n">
+        <v>647.7</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12T16:00</t>
+        </is>
+      </c>
+      <c r="B158" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D158" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E158" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="8" t="n"/>
+      <c r="G158" s="8" t="n"/>
+      <c r="H158" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I158" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J158" s="8" t="n">
+        <v>1653.1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-12T17:00</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D159" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E159" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" s="9" t="n"/>
+      <c r="G159" s="9" t="n"/>
+      <c r="H159" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I159" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J159" s="9" t="n">
+        <v>1057.7</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12T18:00</t>
+        </is>
+      </c>
+      <c r="B160" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D160" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E160" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="8" t="n"/>
+      <c r="G160" s="8" t="n"/>
+      <c r="H160" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I160" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J160" s="8" t="n">
+        <v>329.5</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-12T19:00</t>
+        </is>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C161" s="9" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D161" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E161" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" s="9" t="n"/>
+      <c r="G161" s="9" t="n"/>
+      <c r="H161" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I161" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J161" s="9" t="n">
+        <v>346.1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12T20:00</t>
+        </is>
+      </c>
+      <c r="B162" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D162" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E162" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" s="8" t="n"/>
+      <c r="G162" s="8" t="n"/>
+      <c r="H162" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I162" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J162" s="8" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-12T21:00</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C163" s="9" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D163" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E163" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" s="9" t="n"/>
+      <c r="G163" s="9" t="n"/>
+      <c r="H163" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I163" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J163" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12T22:00</t>
+        </is>
+      </c>
+      <c r="B164" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D164" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E164" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F164" s="8" t="n"/>
+      <c r="G164" s="8" t="n"/>
+      <c r="H164" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I164" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J164" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-12T23:00</t>
+        </is>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C165" s="9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D165" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E165" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" s="9" t="n"/>
+      <c r="G165" s="9" t="n"/>
+      <c r="H165" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I165" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J165" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-13 04:05 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J165"/>
+  <dimension ref="A1:J169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -5579,6 +5579,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00</t>
+        </is>
+      </c>
+      <c r="B166" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C166" s="8" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D166" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E166" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F166" s="8" t="n"/>
+      <c r="G166" s="8" t="n"/>
+      <c r="H166" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I166" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J166" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T01:00</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D167" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E167" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F167" s="9" t="n"/>
+      <c r="G167" s="9" t="n"/>
+      <c r="H167" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J167" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T02:00</t>
+        </is>
+      </c>
+      <c r="B168" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C168" s="8" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D168" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E168" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" s="8" t="n"/>
+      <c r="G168" s="8" t="n"/>
+      <c r="H168" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I168" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J168" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T03:00</t>
+        </is>
+      </c>
+      <c r="B169" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D169" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E169" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" s="9" t="n"/>
+      <c r="G169" s="9" t="n"/>
+      <c r="H169" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I169" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J169" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-13 23:52 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -5715,6 +5715,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T04:00</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D170" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="E170" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" s="8" t="n"/>
+      <c r="G170" s="8" t="n"/>
+      <c r="H170" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I170" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J170" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T05:00</t>
+        </is>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C171" s="9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D171" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="E171" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" s="9" t="n"/>
+      <c r="G171" s="9" t="n"/>
+      <c r="H171" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I171" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J171" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T06:00</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D172" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E172" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" s="8" t="n"/>
+      <c r="G172" s="8" t="n"/>
+      <c r="H172" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I172" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J172" s="8" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T07:00</t>
+        </is>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C173" s="9" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="D173" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E173" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" s="9" t="n"/>
+      <c r="G173" s="9" t="n"/>
+      <c r="H173" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I173" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J173" s="9" t="n">
+        <v>210.2</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T08:00</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D174" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E174" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" s="8" t="n"/>
+      <c r="G174" s="8" t="n"/>
+      <c r="H174" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I174" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J174" s="8" t="n">
+        <v>372.9</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T09:00</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C175" s="9" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D175" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E175" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" s="9" t="n"/>
+      <c r="G175" s="9" t="n"/>
+      <c r="H175" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I175" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J175" s="9" t="n">
+        <v>775.4</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T10:00</t>
+        </is>
+      </c>
+      <c r="B176" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C176" s="8" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D176" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E176" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" s="8" t="n"/>
+      <c r="G176" s="8" t="n"/>
+      <c r="H176" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I176" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J176" s="8" t="n">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T11:00</t>
+        </is>
+      </c>
+      <c r="B177" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D177" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E177" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" s="9" t="n"/>
+      <c r="G177" s="9" t="n"/>
+      <c r="H177" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I177" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J177" s="9" t="n">
+        <v>2551.2</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T12:00</t>
+        </is>
+      </c>
+      <c r="B178" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C178" s="8" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D178" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E178" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" s="8" t="n"/>
+      <c r="G178" s="8" t="n"/>
+      <c r="H178" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I178" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J178" s="8" t="n">
+        <v>3096.2</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T13:00</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D179" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E179" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" s="9" t="n"/>
+      <c r="G179" s="9" t="n"/>
+      <c r="H179" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I179" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J179" s="9" t="n">
+        <v>2274.3</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T14:00</t>
+        </is>
+      </c>
+      <c r="B180" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C180" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D180" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E180" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" s="8" t="n"/>
+      <c r="G180" s="8" t="n"/>
+      <c r="H180" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I180" s="8" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J180" s="8" t="n">
+        <v>2668.2</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T15:00</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D181" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E181" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" s="9" t="n"/>
+      <c r="G181" s="9" t="n"/>
+      <c r="H181" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I181" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J181" s="9" t="n">
+        <v>2308.6</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T16:00</t>
+        </is>
+      </c>
+      <c r="B182" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D182" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E182" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" s="8" t="n"/>
+      <c r="G182" s="8" t="n"/>
+      <c r="H182" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I182" s="8" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J182" s="8" t="n">
+        <v>1030.4</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T17:00</t>
+        </is>
+      </c>
+      <c r="B183" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C183" s="9" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D183" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E183" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" s="9" t="n"/>
+      <c r="G183" s="9" t="n"/>
+      <c r="H183" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I183" s="9" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J183" s="9" t="n">
+        <v>1550.4</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T18:00</t>
+        </is>
+      </c>
+      <c r="B184" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D184" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E184" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" s="8" t="n"/>
+      <c r="G184" s="8" t="n"/>
+      <c r="H184" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="J184" s="8" t="n">
+        <v>1058.5</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:00</t>
+        </is>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C185" s="9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D185" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E185" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" s="9" t="n"/>
+      <c r="G185" s="9" t="n"/>
+      <c r="H185" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I185" s="9" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J185" s="9" t="n">
+        <v>462.3</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T20:00</t>
+        </is>
+      </c>
+      <c r="B186" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D186" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E186" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" s="8" t="n"/>
+      <c r="G186" s="8" t="n"/>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I186" s="8" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J186" s="8" t="n">
+        <v>82.40000000000001</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T21:00</t>
+        </is>
+      </c>
+      <c r="B187" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="D187" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E187" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" s="9" t="n"/>
+      <c r="G187" s="9" t="n"/>
+      <c r="H187" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I187" s="9" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J187" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13T22:00</t>
+        </is>
+      </c>
+      <c r="B188" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C188" s="8" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D188" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E188" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" s="8" t="n"/>
+      <c r="G188" s="8" t="n"/>
+      <c r="H188" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I188" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J188" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-13T23:00</t>
+        </is>
+      </c>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D189" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E189" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" s="9" t="n"/>
+      <c r="G189" s="9" t="n"/>
+      <c r="H189" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I189" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J189" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-14 04:04 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J189"/>
+  <dimension ref="A1:J193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -6395,6 +6395,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00</t>
+        </is>
+      </c>
+      <c r="B190" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C190" s="8" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D190" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E190" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" s="8" t="n"/>
+      <c r="G190" s="8" t="n"/>
+      <c r="H190" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I190" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J190" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T01:00</t>
+        </is>
+      </c>
+      <c r="B191" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C191" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D191" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E191" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" s="9" t="n"/>
+      <c r="G191" s="9" t="n"/>
+      <c r="H191" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I191" s="9" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J191" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T02:00</t>
+        </is>
+      </c>
+      <c r="B192" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C192" s="8" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="D192" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E192" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" s="8" t="n"/>
+      <c r="G192" s="8" t="n"/>
+      <c r="H192" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I192" s="8" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="J192" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T03:00</t>
+        </is>
+      </c>
+      <c r="B193" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C193" s="9" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D193" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="E193" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" s="9" t="n"/>
+      <c r="G193" s="9" t="n"/>
+      <c r="H193" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I193" s="9" t="n">
+        <v>1017.4</v>
+      </c>
+      <c r="J193" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-14 23:46 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J193"/>
+  <dimension ref="A1:J213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -6531,6 +6531,676 @@
         <v>0</v>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T04:00</t>
+        </is>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C194" s="8" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D194" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E194" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" s="8" t="n"/>
+      <c r="G194" s="8" t="n"/>
+      <c r="H194" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I194" s="8" t="n">
+        <v>1017.4</v>
+      </c>
+      <c r="J194" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T05:00</t>
+        </is>
+      </c>
+      <c r="B195" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C195" s="9" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D195" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="E195" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" s="9" t="n"/>
+      <c r="G195" s="9" t="n"/>
+      <c r="H195" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I195" s="9" t="n">
+        <v>1017.2</v>
+      </c>
+      <c r="J195" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T06:00</t>
+        </is>
+      </c>
+      <c r="B196" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C196" s="8" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D196" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E196" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F196" s="8" t="n"/>
+      <c r="G196" s="8" t="n"/>
+      <c r="H196" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I196" s="8" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J196" s="8" t="n">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T07:00</t>
+        </is>
+      </c>
+      <c r="B197" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C197" s="9" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D197" s="9" t="n">
+        <v>96</v>
+      </c>
+      <c r="E197" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F197" s="9" t="n"/>
+      <c r="G197" s="9" t="n"/>
+      <c r="H197" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I197" s="9" t="n">
+        <v>1017.6</v>
+      </c>
+      <c r="J197" s="9" t="n">
+        <v>409.4</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T08:00</t>
+        </is>
+      </c>
+      <c r="B198" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C198" s="8" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D198" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E198" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" s="8" t="n"/>
+      <c r="G198" s="8" t="n"/>
+      <c r="H198" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I198" s="8" t="n">
+        <v>1017.4</v>
+      </c>
+      <c r="J198" s="8" t="n">
+        <v>1293.5</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T09:00</t>
+        </is>
+      </c>
+      <c r="B199" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C199" s="9" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D199" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E199" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" s="9" t="n"/>
+      <c r="G199" s="9" t="n"/>
+      <c r="H199" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I199" s="9" t="n">
+        <v>1017.2</v>
+      </c>
+      <c r="J199" s="9" t="n">
+        <v>1969</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T10:00</t>
+        </is>
+      </c>
+      <c r="B200" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C200" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D200" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E200" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="8" t="n"/>
+      <c r="G200" s="8" t="n"/>
+      <c r="H200" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I200" s="8" t="n">
+        <v>1016.6</v>
+      </c>
+      <c r="J200" s="8" t="n">
+        <v>2629.7</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T11:00</t>
+        </is>
+      </c>
+      <c r="B201" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C201" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D201" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E201" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" s="9" t="n"/>
+      <c r="G201" s="9" t="n"/>
+      <c r="H201" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I201" s="9" t="n">
+        <v>1016.1</v>
+      </c>
+      <c r="J201" s="9" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T12:00</t>
+        </is>
+      </c>
+      <c r="B202" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C202" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D202" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E202" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F202" s="8" t="n"/>
+      <c r="G202" s="8" t="n"/>
+      <c r="H202" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I202" s="8" t="n">
+        <v>1015.8</v>
+      </c>
+      <c r="J202" s="8" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T13:00</t>
+        </is>
+      </c>
+      <c r="B203" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C203" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D203" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E203" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" s="9" t="n"/>
+      <c r="G203" s="9" t="n"/>
+      <c r="H203" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I203" s="9" t="n">
+        <v>1015.6</v>
+      </c>
+      <c r="J203" s="9" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T14:00</t>
+        </is>
+      </c>
+      <c r="B204" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C204" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D204" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E204" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F204" s="8" t="n"/>
+      <c r="G204" s="8" t="n"/>
+      <c r="H204" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I204" s="8" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="J204" s="8" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T15:00</t>
+        </is>
+      </c>
+      <c r="B205" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C205" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D205" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E205" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F205" s="9" t="n"/>
+      <c r="G205" s="9" t="n"/>
+      <c r="H205" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I205" s="9" t="n">
+        <v>1014.5</v>
+      </c>
+      <c r="J205" s="9" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T16:00</t>
+        </is>
+      </c>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C206" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D206" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E206" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F206" s="8" t="n"/>
+      <c r="G206" s="8" t="n"/>
+      <c r="H206" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I206" s="8" t="n">
+        <v>1013.8</v>
+      </c>
+      <c r="J206" s="8" t="n">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T17:00</t>
+        </is>
+      </c>
+      <c r="B207" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C207" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D207" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E207" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F207" s="9" t="n"/>
+      <c r="G207" s="9" t="n"/>
+      <c r="H207" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I207" s="9" t="n">
+        <v>1013.6</v>
+      </c>
+      <c r="J207" s="9" t="n">
+        <v>1935.2</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T18:00</t>
+        </is>
+      </c>
+      <c r="B208" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C208" s="8" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D208" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="E208" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F208" s="8" t="n"/>
+      <c r="G208" s="8" t="n"/>
+      <c r="H208" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I208" s="8" t="n">
+        <v>1013.7</v>
+      </c>
+      <c r="J208" s="8" t="n">
+        <v>1149.7</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T19:00</t>
+        </is>
+      </c>
+      <c r="B209" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C209" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D209" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="E209" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F209" s="9" t="n"/>
+      <c r="G209" s="9" t="n"/>
+      <c r="H209" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I209" s="9" t="n">
+        <v>1014</v>
+      </c>
+      <c r="J209" s="9" t="n">
+        <v>365.2</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T20:00</t>
+        </is>
+      </c>
+      <c r="B210" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C210" s="8" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D210" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E210" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F210" s="8" t="n"/>
+      <c r="G210" s="8" t="n"/>
+      <c r="H210" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I210" s="8" t="n">
+        <v>1014.3</v>
+      </c>
+      <c r="J210" s="8" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T21:00</t>
+        </is>
+      </c>
+      <c r="B211" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C211" s="9" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D211" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E211" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F211" s="9" t="n"/>
+      <c r="G211" s="9" t="n"/>
+      <c r="H211" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I211" s="9" t="n">
+        <v>1014.6</v>
+      </c>
+      <c r="J211" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14T22:00</t>
+        </is>
+      </c>
+      <c r="B212" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C212" s="8" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D212" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E212" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F212" s="8" t="n"/>
+      <c r="G212" s="8" t="n"/>
+      <c r="H212" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I212" s="8" t="n">
+        <v>1015.2</v>
+      </c>
+      <c r="J212" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14T23:00</t>
+        </is>
+      </c>
+      <c r="B213" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C213" s="9" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D213" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="E213" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F213" s="9" t="n"/>
+      <c r="G213" s="9" t="n"/>
+      <c r="H213" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I213" s="9" t="n">
+        <v>1015.4</v>
+      </c>
+      <c r="J213" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-15 04:09 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,14 @@
       <color rgb="FF7F6000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +96,12 @@
         <bgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+        <bgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -122,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -147,6 +159,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -514,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J213"/>
+  <dimension ref="A1:J217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -7201,6 +7216,112 @@
         <v>0</v>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T00:00</t>
+        </is>
+      </c>
+      <c r="B214" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C214" s="8" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="D214" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="E214" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F214" s="8" t="n"/>
+      <c r="G214" s="8" t="n"/>
+      <c r="H214" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I214" s="8" t="n">
+        <v>1015.4</v>
+      </c>
+      <c r="J214" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-15T01:00</t>
+        </is>
+      </c>
+      <c r="B215" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C215" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D215" s="10" t="n"/>
+      <c r="E215" s="10" t="n"/>
+      <c r="F215" s="10" t="n"/>
+      <c r="G215" s="10" t="n"/>
+      <c r="H215" s="10" t="n"/>
+      <c r="I215" s="10" t="n"/>
+      <c r="J215" s="10" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-15T02:00</t>
+        </is>
+      </c>
+      <c r="B216" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C216" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D216" s="10" t="n"/>
+      <c r="E216" s="10" t="n"/>
+      <c r="F216" s="10" t="n"/>
+      <c r="G216" s="10" t="n"/>
+      <c r="H216" s="10" t="n"/>
+      <c r="I216" s="10" t="n"/>
+      <c r="J216" s="10" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-15T03:00</t>
+        </is>
+      </c>
+      <c r="B217" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C217" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D217" s="10" t="n"/>
+      <c r="E217" s="10" t="n"/>
+      <c r="F217" s="10" t="n"/>
+      <c r="G217" s="10" t="n"/>
+      <c r="H217" s="10" t="n"/>
+      <c r="I217" s="10" t="n"/>
+      <c r="J217" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-15 23:51 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J217"/>
+  <dimension ref="A1:J237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -7322,6 +7322,674 @@
       <c r="I217" s="10" t="n"/>
       <c r="J217" s="10" t="n"/>
     </row>
+    <row r="218">
+      <c r="A218" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T04:00</t>
+        </is>
+      </c>
+      <c r="B218" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C218" s="8" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D218" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="E218" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F218" s="8" t="n"/>
+      <c r="G218" s="8" t="n"/>
+      <c r="H218" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I218" s="8" t="n">
+        <v>1014.6</v>
+      </c>
+      <c r="J218" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T05:00</t>
+        </is>
+      </c>
+      <c r="B219" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C219" s="9" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D219" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E219" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F219" s="9" t="n"/>
+      <c r="G219" s="9" t="n"/>
+      <c r="H219" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I219" s="9" t="n">
+        <v>1014.5</v>
+      </c>
+      <c r="J219" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T06:00</t>
+        </is>
+      </c>
+      <c r="B220" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C220" s="8" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D220" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E220" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F220" s="8" t="n"/>
+      <c r="G220" s="8" t="n"/>
+      <c r="H220" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I220" s="8" t="n">
+        <v>1014.8</v>
+      </c>
+      <c r="J220" s="8" t="n">
+        <v>57.2</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T07:00</t>
+        </is>
+      </c>
+      <c r="B221" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C221" s="9" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D221" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E221" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F221" s="9" t="n"/>
+      <c r="G221" s="9" t="n"/>
+      <c r="H221" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I221" s="9" t="n">
+        <v>1015</v>
+      </c>
+      <c r="J221" s="9" t="n">
+        <v>601.7</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T08:00</t>
+        </is>
+      </c>
+      <c r="B222" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C222" s="8" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D222" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E222" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F222" s="8" t="n"/>
+      <c r="G222" s="8" t="n"/>
+      <c r="H222" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I222" s="8" t="n">
+        <v>1015.2</v>
+      </c>
+      <c r="J222" s="8" t="n">
+        <v>869.2</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T09:00</t>
+        </is>
+      </c>
+      <c r="B223" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C223" s="9" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D223" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E223" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F223" s="9" t="n"/>
+      <c r="G223" s="9" t="n"/>
+      <c r="H223" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I223" s="9" t="n">
+        <v>1015.2</v>
+      </c>
+      <c r="J223" s="9" t="n">
+        <v>964.4</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T10:00</t>
+        </is>
+      </c>
+      <c r="B224" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C224" s="8" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D224" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E224" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F224" s="8" t="n"/>
+      <c r="G224" s="8" t="n"/>
+      <c r="H224" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I224" s="8" t="n">
+        <v>1015.2</v>
+      </c>
+      <c r="J224" s="8" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T11:00</t>
+        </is>
+      </c>
+      <c r="B225" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C225" s="9" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D225" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E225" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F225" s="9" t="n"/>
+      <c r="G225" s="9" t="n"/>
+      <c r="H225" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I225" s="9" t="n">
+        <v>1015.3</v>
+      </c>
+      <c r="J225" s="9" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T12:00</t>
+        </is>
+      </c>
+      <c r="B226" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C226" s="8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D226" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E226" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F226" s="8" t="n"/>
+      <c r="G226" s="8" t="n"/>
+      <c r="H226" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I226" s="8" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="J226" s="8" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T13:00</t>
+        </is>
+      </c>
+      <c r="B227" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C227" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="D227" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E227" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F227" s="9" t="n"/>
+      <c r="G227" s="9" t="n"/>
+      <c r="H227" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I227" s="9" t="n">
+        <v>1014.7</v>
+      </c>
+      <c r="J227" s="9" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T14:00</t>
+        </is>
+      </c>
+      <c r="B228" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C228" s="8" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D228" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E228" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F228" s="8" t="n"/>
+      <c r="G228" s="8" t="n"/>
+      <c r="H228" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I228" s="8" t="n">
+        <v>1014.5</v>
+      </c>
+      <c r="J228" s="8" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T15:00</t>
+        </is>
+      </c>
+      <c r="B229" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C229" s="9" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D229" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E229" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F229" s="9" t="n"/>
+      <c r="G229" s="9" t="n"/>
+      <c r="H229" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I229" s="9" t="n">
+        <v>1014.4</v>
+      </c>
+      <c r="J229" s="9" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T16:00</t>
+        </is>
+      </c>
+      <c r="B230" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C230" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D230" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E230" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" s="8" t="n"/>
+      <c r="G230" s="8" t="n"/>
+      <c r="H230" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I230" s="8" t="n">
+        <v>1014.1</v>
+      </c>
+      <c r="J230" s="8" t="n">
+        <v>2140.3</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T17:00</t>
+        </is>
+      </c>
+      <c r="B231" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C231" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="D231" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E231" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F231" s="9" t="n"/>
+      <c r="G231" s="9" t="n"/>
+      <c r="H231" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I231" s="9" t="n">
+        <v>1014.3</v>
+      </c>
+      <c r="J231" s="9" t="n">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T18:00</t>
+        </is>
+      </c>
+      <c r="B232" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C232" s="8" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="D232" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E232" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F232" s="8" t="n"/>
+      <c r="G232" s="8" t="n"/>
+      <c r="H232" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I232" s="8" t="n">
+        <v>1014.5</v>
+      </c>
+      <c r="J232" s="8" t="n">
+        <v>1200.7</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T19:00</t>
+        </is>
+      </c>
+      <c r="B233" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C233" s="9" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D233" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E233" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" s="9" t="n"/>
+      <c r="G233" s="9" t="n"/>
+      <c r="H233" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I233" s="9" t="n">
+        <v>1014.9</v>
+      </c>
+      <c r="J233" s="9" t="n">
+        <v>646.8</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T20:00</t>
+        </is>
+      </c>
+      <c r="B234" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C234" s="8" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D234" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E234" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F234" s="8" t="n"/>
+      <c r="G234" s="8" t="n"/>
+      <c r="H234" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I234" s="8" t="n">
+        <v>1015.9</v>
+      </c>
+      <c r="J234" s="8" t="n">
+        <v>77.3</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T21:00</t>
+        </is>
+      </c>
+      <c r="B235" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C235" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D235" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="E235" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F235" s="9" t="n"/>
+      <c r="G235" s="9" t="n"/>
+      <c r="H235" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I235" s="9" t="n">
+        <v>1016.7</v>
+      </c>
+      <c r="J235" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-15T22:00</t>
+        </is>
+      </c>
+      <c r="B236" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C236" s="8" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D236" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E236" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F236" s="8" t="n"/>
+      <c r="G236" s="8" t="n"/>
+      <c r="H236" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I236" s="8" t="n">
+        <v>1017.7</v>
+      </c>
+      <c r="J236" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-15T23:00</t>
+        </is>
+      </c>
+      <c r="B237" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C237" s="9" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D237" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E237" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F237" s="9" t="n"/>
+      <c r="G237" s="9" t="n"/>
+      <c r="H237" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I237" s="9" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J237" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-16 03:51 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J237"/>
+  <dimension ref="A1:J241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -7990,6 +7990,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T00:00</t>
+        </is>
+      </c>
+      <c r="B238" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C238" s="8" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D238" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="E238" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F238" s="8" t="n"/>
+      <c r="G238" s="8" t="n"/>
+      <c r="H238" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I238" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J238" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T01:00</t>
+        </is>
+      </c>
+      <c r="B239" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C239" s="9" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D239" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E239" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F239" s="9" t="n"/>
+      <c r="G239" s="9" t="n"/>
+      <c r="H239" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I239" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J239" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T02:00</t>
+        </is>
+      </c>
+      <c r="B240" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C240" s="8" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="D240" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E240" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" s="8" t="n"/>
+      <c r="G240" s="8" t="n"/>
+      <c r="H240" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I240" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J240" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T03:00</t>
+        </is>
+      </c>
+      <c r="B241" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C241" s="9" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="D241" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E241" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" s="9" t="n"/>
+      <c r="G241" s="9" t="n"/>
+      <c r="H241" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I241" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J241" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-16 23:45 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J241"/>
+  <dimension ref="A1:J261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -8126,6 +8126,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T04:00</t>
+        </is>
+      </c>
+      <c r="B242" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C242" s="8" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D242" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E242" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" s="8" t="n"/>
+      <c r="G242" s="8" t="n"/>
+      <c r="H242" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I242" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J242" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T05:00</t>
+        </is>
+      </c>
+      <c r="B243" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C243" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D243" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E243" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" s="9" t="n"/>
+      <c r="G243" s="9" t="n"/>
+      <c r="H243" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I243" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J243" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T06:00</t>
+        </is>
+      </c>
+      <c r="B244" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C244" s="8" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D244" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E244" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F244" s="8" t="n"/>
+      <c r="G244" s="8" t="n"/>
+      <c r="H244" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I244" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J244" s="8" t="n">
+        <v>63.2</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T07:00</t>
+        </is>
+      </c>
+      <c r="B245" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C245" s="9" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="D245" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E245" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F245" s="9" t="n"/>
+      <c r="G245" s="9" t="n"/>
+      <c r="H245" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I245" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J245" s="9" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T08:00</t>
+        </is>
+      </c>
+      <c r="B246" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C246" s="8" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D246" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E246" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F246" s="8" t="n"/>
+      <c r="G246" s="8" t="n"/>
+      <c r="H246" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I246" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J246" s="8" t="n">
+        <v>1312.6</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T09:00</t>
+        </is>
+      </c>
+      <c r="B247" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C247" s="9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D247" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E247" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F247" s="9" t="n"/>
+      <c r="G247" s="9" t="n"/>
+      <c r="H247" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I247" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J247" s="9" t="n">
+        <v>2021.1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T10:00</t>
+        </is>
+      </c>
+      <c r="B248" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C248" s="8" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D248" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E248" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F248" s="8" t="n"/>
+      <c r="G248" s="8" t="n"/>
+      <c r="H248" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I248" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J248" s="8" t="n">
+        <v>2642.1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T11:00</t>
+        </is>
+      </c>
+      <c r="B249" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C249" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D249" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E249" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F249" s="9" t="n"/>
+      <c r="G249" s="9" t="n"/>
+      <c r="H249" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I249" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J249" s="9" t="n">
+        <v>3121.8</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T12:00</t>
+        </is>
+      </c>
+      <c r="B250" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C250" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D250" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="E250" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" s="8" t="n"/>
+      <c r="G250" s="8" t="n"/>
+      <c r="H250" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I250" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J250" s="8" t="n">
+        <v>3420.3</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T13:00</t>
+        </is>
+      </c>
+      <c r="B251" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C251" s="9" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D251" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E251" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" s="9" t="n"/>
+      <c r="G251" s="9" t="n"/>
+      <c r="H251" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I251" s="9" t="n">
+        <v>1018</v>
+      </c>
+      <c r="J251" s="9" t="n">
+        <v>3510.5</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T14:00</t>
+        </is>
+      </c>
+      <c r="B252" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C252" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D252" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="E252" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F252" s="8" t="n"/>
+      <c r="G252" s="8" t="n"/>
+      <c r="H252" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I252" s="8" t="n">
+        <v>1017.6</v>
+      </c>
+      <c r="J252" s="8" t="n">
+        <v>3400.8</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T15:00</t>
+        </is>
+      </c>
+      <c r="B253" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C253" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D253" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E253" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F253" s="9" t="n"/>
+      <c r="G253" s="9" t="n"/>
+      <c r="H253" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I253" s="9" t="n">
+        <v>1017.4</v>
+      </c>
+      <c r="J253" s="9" t="n">
+        <v>2403</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T16:00</t>
+        </is>
+      </c>
+      <c r="B254" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C254" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D254" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E254" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F254" s="8" t="n"/>
+      <c r="G254" s="8" t="n"/>
+      <c r="H254" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I254" s="8" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J254" s="8" t="n">
+        <v>1203.3</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T17:00</t>
+        </is>
+      </c>
+      <c r="B255" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C255" s="9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D255" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E255" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F255" s="9" t="n"/>
+      <c r="G255" s="9" t="n"/>
+      <c r="H255" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I255" s="9" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J255" s="9" t="n">
+        <v>2054.3</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T18:00</t>
+        </is>
+      </c>
+      <c r="B256" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C256" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D256" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E256" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F256" s="8" t="n"/>
+      <c r="G256" s="8" t="n"/>
+      <c r="H256" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I256" s="8" t="n">
+        <v>1017.1</v>
+      </c>
+      <c r="J256" s="8" t="n">
+        <v>1370.1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T19:00</t>
+        </is>
+      </c>
+      <c r="B257" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C257" s="9" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D257" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E257" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F257" s="9" t="n"/>
+      <c r="G257" s="9" t="n"/>
+      <c r="H257" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I257" s="9" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J257" s="9" t="n">
+        <v>587.2</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T20:00</t>
+        </is>
+      </c>
+      <c r="B258" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C258" s="8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D258" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E258" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F258" s="8" t="n"/>
+      <c r="G258" s="8" t="n"/>
+      <c r="H258" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I258" s="8" t="n">
+        <v>1017.7</v>
+      </c>
+      <c r="J258" s="8" t="n">
+        <v>58.6</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T21:00</t>
+        </is>
+      </c>
+      <c r="B259" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C259" s="9" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D259" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E259" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F259" s="9" t="n"/>
+      <c r="G259" s="9" t="n"/>
+      <c r="H259" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I259" s="9" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J259" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16T22:00</t>
+        </is>
+      </c>
+      <c r="B260" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C260" s="8" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D260" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E260" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F260" s="8" t="n"/>
+      <c r="G260" s="8" t="n"/>
+      <c r="H260" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I260" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J260" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-16T23:00</t>
+        </is>
+      </c>
+      <c r="B261" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C261" s="9" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="D261" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E261" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F261" s="9" t="n"/>
+      <c r="G261" s="9" t="n"/>
+      <c r="H261" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I261" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J261" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-17 04:10 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J261"/>
+  <dimension ref="A1:J265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -8806,6 +8806,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T00:00</t>
+        </is>
+      </c>
+      <c r="B262" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C262" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D262" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E262" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F262" s="8" t="n"/>
+      <c r="G262" s="8" t="n"/>
+      <c r="H262" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I262" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J262" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T01:00</t>
+        </is>
+      </c>
+      <c r="B263" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C263" s="9" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="D263" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E263" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F263" s="9" t="n"/>
+      <c r="G263" s="9" t="n"/>
+      <c r="H263" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I263" s="9" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J263" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T02:00</t>
+        </is>
+      </c>
+      <c r="B264" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C264" s="8" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D264" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E264" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F264" s="8" t="n"/>
+      <c r="G264" s="8" t="n"/>
+      <c r="H264" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I264" s="8" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J264" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T03:00</t>
+        </is>
+      </c>
+      <c r="B265" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C265" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D265" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E265" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F265" s="9" t="n"/>
+      <c r="G265" s="9" t="n"/>
+      <c r="H265" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I265" s="9" t="n">
+        <v>1018.3</v>
+      </c>
+      <c r="J265" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-17 23:54 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J265"/>
+  <dimension ref="A1:J285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -8942,6 +8942,676 @@
         <v>0</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T04:00</t>
+        </is>
+      </c>
+      <c r="B266" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C266" s="8" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D266" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E266" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F266" s="8" t="n"/>
+      <c r="G266" s="8" t="n"/>
+      <c r="H266" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I266" s="8" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J266" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T05:00</t>
+        </is>
+      </c>
+      <c r="B267" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C267" s="9" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D267" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E267" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F267" s="9" t="n"/>
+      <c r="G267" s="9" t="n"/>
+      <c r="H267" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I267" s="9" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="J267" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T06:00</t>
+        </is>
+      </c>
+      <c r="B268" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C268" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D268" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E268" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F268" s="8" t="n"/>
+      <c r="G268" s="8" t="n"/>
+      <c r="H268" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I268" s="8" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J268" s="8" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T07:00</t>
+        </is>
+      </c>
+      <c r="B269" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C269" s="9" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="D269" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E269" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F269" s="9" t="n"/>
+      <c r="G269" s="9" t="n"/>
+      <c r="H269" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I269" s="9" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J269" s="9" t="n">
+        <v>562.3</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T08:00</t>
+        </is>
+      </c>
+      <c r="B270" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C270" s="8" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D270" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="E270" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F270" s="8" t="n"/>
+      <c r="G270" s="8" t="n"/>
+      <c r="H270" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I270" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J270" s="8" t="n">
+        <v>1256.8</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T09:00</t>
+        </is>
+      </c>
+      <c r="B271" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C271" s="9" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D271" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E271" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F271" s="9" t="n"/>
+      <c r="G271" s="9" t="n"/>
+      <c r="H271" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I271" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J271" s="9" t="n">
+        <v>2000.7</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T10:00</t>
+        </is>
+      </c>
+      <c r="B272" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C272" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D272" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E272" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" s="8" t="n"/>
+      <c r="G272" s="8" t="n"/>
+      <c r="H272" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I272" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J272" s="8" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T11:00</t>
+        </is>
+      </c>
+      <c r="B273" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C273" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D273" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E273" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F273" s="9" t="n"/>
+      <c r="G273" s="9" t="n"/>
+      <c r="H273" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I273" s="9" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J273" s="9" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T12:00</t>
+        </is>
+      </c>
+      <c r="B274" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C274" s="8" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="D274" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E274" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F274" s="8" t="n"/>
+      <c r="G274" s="8" t="n"/>
+      <c r="H274" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I274" s="8" t="n">
+        <v>1017.7</v>
+      </c>
+      <c r="J274" s="8" t="n">
+        <v>3426.1</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T13:00</t>
+        </is>
+      </c>
+      <c r="B275" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C275" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D275" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E275" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F275" s="9" t="n"/>
+      <c r="G275" s="9" t="n"/>
+      <c r="H275" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I275" s="9" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J275" s="9" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:00</t>
+        </is>
+      </c>
+      <c r="B276" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C276" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D276" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E276" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" s="8" t="n"/>
+      <c r="G276" s="8" t="n"/>
+      <c r="H276" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I276" s="8" t="n">
+        <v>1016.9</v>
+      </c>
+      <c r="J276" s="8" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T15:00</t>
+        </is>
+      </c>
+      <c r="B277" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C277" s="9" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D277" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E277" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F277" s="9" t="n"/>
+      <c r="G277" s="9" t="n"/>
+      <c r="H277" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I277" s="9" t="n">
+        <v>1016.9</v>
+      </c>
+      <c r="J277" s="9" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T16:00</t>
+        </is>
+      </c>
+      <c r="B278" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C278" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D278" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E278" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F278" s="8" t="n"/>
+      <c r="G278" s="8" t="n"/>
+      <c r="H278" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I278" s="8" t="n">
+        <v>1017</v>
+      </c>
+      <c r="J278" s="8" t="n">
+        <v>2634.4</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T17:00</t>
+        </is>
+      </c>
+      <c r="B279" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C279" s="9" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="D279" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E279" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" s="9" t="n"/>
+      <c r="G279" s="9" t="n"/>
+      <c r="H279" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I279" s="9" t="n">
+        <v>1017.1</v>
+      </c>
+      <c r="J279" s="9" t="n">
+        <v>1992.6</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T18:00</t>
+        </is>
+      </c>
+      <c r="B280" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C280" s="8" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D280" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E280" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F280" s="8" t="n"/>
+      <c r="G280" s="8" t="n"/>
+      <c r="H280" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I280" s="8" t="n">
+        <v>1017.1</v>
+      </c>
+      <c r="J280" s="8" t="n">
+        <v>1283.9</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T19:00</t>
+        </is>
+      </c>
+      <c r="B281" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C281" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D281" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="E281" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" s="9" t="n"/>
+      <c r="G281" s="9" t="n"/>
+      <c r="H281" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I281" s="9" t="n">
+        <v>1017.6</v>
+      </c>
+      <c r="J281" s="9" t="n">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T20:00</t>
+        </is>
+      </c>
+      <c r="B282" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C282" s="8" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D282" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E282" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F282" s="8" t="n"/>
+      <c r="G282" s="8" t="n"/>
+      <c r="H282" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I282" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J282" s="8" t="n">
+        <v>83.90000000000001</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T21:00</t>
+        </is>
+      </c>
+      <c r="B283" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C283" s="9" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="D283" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E283" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F283" s="9" t="n"/>
+      <c r="G283" s="9" t="n"/>
+      <c r="H283" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I283" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J283" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-17T22:00</t>
+        </is>
+      </c>
+      <c r="B284" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C284" s="8" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="D284" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E284" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F284" s="8" t="n"/>
+      <c r="G284" s="8" t="n"/>
+      <c r="H284" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I284" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J284" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-17T23:00</t>
+        </is>
+      </c>
+      <c r="B285" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C285" s="9" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="D285" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E285" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F285" s="9" t="n"/>
+      <c r="G285" s="9" t="n"/>
+      <c r="H285" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I285" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J285" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-18 04:21 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J285"/>
+  <dimension ref="A1:J289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -9612,6 +9612,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T00:00</t>
+        </is>
+      </c>
+      <c r="B286" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C286" s="8" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D286" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E286" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F286" s="8" t="n"/>
+      <c r="G286" s="8" t="n"/>
+      <c r="H286" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I286" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J286" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T01:00</t>
+        </is>
+      </c>
+      <c r="B287" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C287" s="9" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D287" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E287" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F287" s="9" t="n"/>
+      <c r="G287" s="9" t="n"/>
+      <c r="H287" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I287" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J287" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T02:00</t>
+        </is>
+      </c>
+      <c r="B288" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C288" s="8" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D288" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E288" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F288" s="8" t="n"/>
+      <c r="G288" s="8" t="n"/>
+      <c r="H288" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I288" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J288" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T03:00</t>
+        </is>
+      </c>
+      <c r="B289" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C289" s="9" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D289" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E289" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F289" s="9" t="n"/>
+      <c r="G289" s="9" t="n"/>
+      <c r="H289" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I289" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J289" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-19 00:01 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J289"/>
+  <dimension ref="A1:J309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -9748,6 +9748,684 @@
         <v>0</v>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T04:00</t>
+        </is>
+      </c>
+      <c r="B290" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C290" s="8" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D290" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E290" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F290" s="8" t="n"/>
+      <c r="G290" s="8" t="n"/>
+      <c r="H290" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I290" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J290" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T05:00</t>
+        </is>
+      </c>
+      <c r="B291" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C291" s="9" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="D291" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="E291" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F291" s="9" t="n"/>
+      <c r="G291" s="9" t="n"/>
+      <c r="H291" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I291" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J291" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T06:00</t>
+        </is>
+      </c>
+      <c r="B292" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C292" s="8" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D292" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E292" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F292" s="8" t="n"/>
+      <c r="G292" s="8" t="n"/>
+      <c r="H292" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I292" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J292" s="8" t="n">
+        <v>60.8</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T07:00</t>
+        </is>
+      </c>
+      <c r="B293" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C293" s="9" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="D293" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E293" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" s="9" t="n"/>
+      <c r="G293" s="9" t="n"/>
+      <c r="H293" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I293" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J293" s="9" t="n">
+        <v>538.2</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T08:00</t>
+        </is>
+      </c>
+      <c r="B294" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C294" s="8" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D294" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E294" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F294" s="8" t="n"/>
+      <c r="G294" s="8" t="n"/>
+      <c r="H294" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I294" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J294" s="8" t="n">
+        <v>1287.4</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T09:00</t>
+        </is>
+      </c>
+      <c r="B295" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C295" s="9" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D295" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="E295" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F295" s="9" t="n"/>
+      <c r="G295" s="9" t="n"/>
+      <c r="H295" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I295" s="9" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J295" s="9" t="n">
+        <v>1465.5</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T10:00</t>
+        </is>
+      </c>
+      <c r="B296" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C296" s="8" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D296" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E296" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F296" s="8" t="n"/>
+      <c r="G296" s="8" t="n"/>
+      <c r="H296" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I296" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J296" s="8" t="n">
+        <v>1205.5</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T11:00</t>
+        </is>
+      </c>
+      <c r="B297" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C297" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D297" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E297" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" s="9" t="n"/>
+      <c r="G297" s="9" t="n"/>
+      <c r="H297" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I297" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J297" s="9" t="n">
+        <v>2016.2</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T12:00</t>
+        </is>
+      </c>
+      <c r="B298" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C298" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D298" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E298" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F298" s="8" t="n"/>
+      <c r="G298" s="8" t="n"/>
+      <c r="H298" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I298" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J298" s="8" t="n">
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T13:00</t>
+        </is>
+      </c>
+      <c r="B299" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C299" s="9" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D299" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E299" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F299" s="9" t="n"/>
+      <c r="G299" s="9" t="n"/>
+      <c r="H299" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I299" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J299" s="9" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T14:00</t>
+        </is>
+      </c>
+      <c r="B300" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C300" s="8" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D300" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E300" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F300" s="8" t="n"/>
+      <c r="G300" s="8" t="n"/>
+      <c r="H300" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I300" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J300" s="8" t="n">
+        <v>3013.4</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T15:00</t>
+        </is>
+      </c>
+      <c r="B301" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C301" s="9" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="D301" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E301" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F301" s="9" t="n"/>
+      <c r="G301" s="9" t="n"/>
+      <c r="H301" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I301" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J301" s="9" t="n">
+        <v>3008.6</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T16:00</t>
+        </is>
+      </c>
+      <c r="B302" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C302" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D302" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="E302" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F302" s="8" t="n"/>
+      <c r="G302" s="8" t="n"/>
+      <c r="H302" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I302" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J302" s="8" t="n">
+        <v>2434.7</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T17:00</t>
+        </is>
+      </c>
+      <c r="B303" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C303" s="9" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D303" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E303" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F303" s="9" t="n"/>
+      <c r="G303" s="9" t="n"/>
+      <c r="H303" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I303" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J303" s="9" t="n">
+        <v>1944.6</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T18:00</t>
+        </is>
+      </c>
+      <c r="B304" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C304" s="8" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D304" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E304" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" s="8" t="n"/>
+      <c r="G304" s="8" t="n"/>
+      <c r="H304" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I304" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J304" s="8" t="n">
+        <v>867.6</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T19:00</t>
+        </is>
+      </c>
+      <c r="B305" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C305" s="9" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D305" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="E305" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F305" s="9" t="n"/>
+      <c r="G305" s="9" t="n"/>
+      <c r="H305" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I305" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J305" s="9" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T20:00</t>
+        </is>
+      </c>
+      <c r="B306" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C306" s="8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D306" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E306" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F306" s="8" t="n"/>
+      <c r="G306" s="8" t="n"/>
+      <c r="H306" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I306" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J306" s="8" t="n">
+        <v>97.7</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T21:00</t>
+        </is>
+      </c>
+      <c r="B307" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C307" s="9" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="D307" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E307" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F307" s="9" t="n"/>
+      <c r="G307" s="9" t="n"/>
+      <c r="H307" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I307" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J307" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-18T22:00</t>
+        </is>
+      </c>
+      <c r="B308" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C308" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D308" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E308" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" s="8" t="n"/>
+      <c r="G308" s="8" t="n"/>
+      <c r="H308" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I308" s="8" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J308" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-18T23:00</t>
+        </is>
+      </c>
+      <c r="B309" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C309" s="9" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="D309" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E309" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F309" s="9" t="n"/>
+      <c r="G309" s="9" t="n"/>
+      <c r="H309" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I309" s="9" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="J309" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-19 04:18 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J309"/>
+  <dimension ref="A1:J313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -10426,6 +10426,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T00:00</t>
+        </is>
+      </c>
+      <c r="B310" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C310" s="8" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D310" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="E310" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" s="8" t="n"/>
+      <c r="G310" s="8" t="n"/>
+      <c r="H310" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I310" s="8" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J310" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T01:00</t>
+        </is>
+      </c>
+      <c r="B311" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C311" s="9" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D311" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E311" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" s="9" t="n"/>
+      <c r="G311" s="9" t="n"/>
+      <c r="H311" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I311" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J311" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T02:00</t>
+        </is>
+      </c>
+      <c r="B312" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C312" s="8" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="D312" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E312" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" s="8" t="n"/>
+      <c r="G312" s="8" t="n"/>
+      <c r="H312" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I312" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J312" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T03:00</t>
+        </is>
+      </c>
+      <c r="B313" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C313" s="9" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="D313" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E313" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" s="9" t="n"/>
+      <c r="G313" s="9" t="n"/>
+      <c r="H313" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I313" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J313" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-19 23:58 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J313"/>
+  <dimension ref="A1:J333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -10562,6 +10562,684 @@
         <v>0</v>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T04:00</t>
+        </is>
+      </c>
+      <c r="B314" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C314" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D314" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E314" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F314" s="8" t="n"/>
+      <c r="G314" s="8" t="n"/>
+      <c r="H314" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I314" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J314" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T05:00</t>
+        </is>
+      </c>
+      <c r="B315" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C315" s="9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D315" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E315" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" s="9" t="n"/>
+      <c r="G315" s="9" t="n"/>
+      <c r="H315" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I315" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J315" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T06:00</t>
+        </is>
+      </c>
+      <c r="B316" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C316" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D316" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E316" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" s="8" t="n"/>
+      <c r="G316" s="8" t="n"/>
+      <c r="H316" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I316" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J316" s="8" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T07:00</t>
+        </is>
+      </c>
+      <c r="B317" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C317" s="9" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D317" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E317" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F317" s="9" t="n"/>
+      <c r="G317" s="9" t="n"/>
+      <c r="H317" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I317" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J317" s="9" t="n">
+        <v>100.1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T08:00</t>
+        </is>
+      </c>
+      <c r="B318" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C318" s="8" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D318" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E318" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F318" s="8" t="n"/>
+      <c r="G318" s="8" t="n"/>
+      <c r="H318" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I318" s="8" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J318" s="8" t="n">
+        <v>353.4</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T09:00</t>
+        </is>
+      </c>
+      <c r="B319" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C319" s="9" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D319" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E319" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F319" s="9" t="n"/>
+      <c r="G319" s="9" t="n"/>
+      <c r="H319" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I319" s="9" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J319" s="9" t="n">
+        <v>577.2</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T10:00</t>
+        </is>
+      </c>
+      <c r="B320" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C320" s="8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D320" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E320" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F320" s="8" t="n"/>
+      <c r="G320" s="8" t="n"/>
+      <c r="H320" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I320" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J320" s="8" t="n">
+        <v>897.2</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T11:00</t>
+        </is>
+      </c>
+      <c r="B321" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C321" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D321" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E321" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F321" s="9" t="n"/>
+      <c r="G321" s="9" t="n"/>
+      <c r="H321" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I321" s="9" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J321" s="9" t="n">
+        <v>514.6</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T12:00</t>
+        </is>
+      </c>
+      <c r="B322" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C322" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D322" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E322" s="8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F322" s="8" t="n"/>
+      <c r="G322" s="8" t="n"/>
+      <c r="H322" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I322" s="8" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J322" s="8" t="n">
+        <v>553.2</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T13:00</t>
+        </is>
+      </c>
+      <c r="B323" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C323" s="9" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D323" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E323" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F323" s="9" t="n"/>
+      <c r="G323" s="9" t="n"/>
+      <c r="H323" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I323" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J323" s="9" t="n">
+        <v>757.1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T14:00</t>
+        </is>
+      </c>
+      <c r="B324" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C324" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D324" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E324" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F324" s="8" t="n"/>
+      <c r="G324" s="8" t="n"/>
+      <c r="H324" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I324" s="8" t="n">
+        <v>1023.3</v>
+      </c>
+      <c r="J324" s="8" t="n">
+        <v>994.4</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T15:00</t>
+        </is>
+      </c>
+      <c r="B325" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C325" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D325" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E325" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" s="9" t="n"/>
+      <c r="G325" s="9" t="n"/>
+      <c r="H325" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I325" s="9" t="n">
+        <v>1023.2</v>
+      </c>
+      <c r="J325" s="9" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T16:00</t>
+        </is>
+      </c>
+      <c r="B326" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C326" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D326" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E326" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F326" s="8" t="n"/>
+      <c r="G326" s="8" t="n"/>
+      <c r="H326" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I326" s="8" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="J326" s="8" t="n">
+        <v>1923.4</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T17:00</t>
+        </is>
+      </c>
+      <c r="B327" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C327" s="9" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="D327" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E327" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" s="9" t="n"/>
+      <c r="G327" s="9" t="n"/>
+      <c r="H327" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I327" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J327" s="9" t="n">
+        <v>1935.1</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T18:00</t>
+        </is>
+      </c>
+      <c r="B328" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C328" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D328" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E328" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" s="8" t="n"/>
+      <c r="G328" s="8" t="n"/>
+      <c r="H328" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I328" s="8" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J328" s="8" t="n">
+        <v>1078.2</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T19:00</t>
+        </is>
+      </c>
+      <c r="B329" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C329" s="9" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D329" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E329" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F329" s="9" t="n"/>
+      <c r="G329" s="9" t="n"/>
+      <c r="H329" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I329" s="9" t="n">
+        <v>1023.5</v>
+      </c>
+      <c r="J329" s="9" t="n">
+        <v>432.6</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T20:00</t>
+        </is>
+      </c>
+      <c r="B330" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C330" s="8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D330" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E330" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" s="8" t="n"/>
+      <c r="G330" s="8" t="n"/>
+      <c r="H330" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I330" s="8" t="n">
+        <v>1024</v>
+      </c>
+      <c r="J330" s="8" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T21:00</t>
+        </is>
+      </c>
+      <c r="B331" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C331" s="9" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D331" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E331" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F331" s="9" t="n"/>
+      <c r="G331" s="9" t="n"/>
+      <c r="H331" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I331" s="9" t="n">
+        <v>1024.5</v>
+      </c>
+      <c r="J331" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-19T22:00</t>
+        </is>
+      </c>
+      <c r="B332" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C332" s="8" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="D332" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E332" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F332" s="8" t="n"/>
+      <c r="G332" s="8" t="n"/>
+      <c r="H332" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I332" s="8" t="n">
+        <v>1024.9</v>
+      </c>
+      <c r="J332" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19T23:00</t>
+        </is>
+      </c>
+      <c r="B333" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C333" s="9" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D333" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E333" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F333" s="9" t="n"/>
+      <c r="G333" s="9" t="n"/>
+      <c r="H333" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I333" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="J333" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-20 04:18 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J333"/>
+  <dimension ref="A1:J337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -11240,6 +11240,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T00:00</t>
+        </is>
+      </c>
+      <c r="B334" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C334" s="8" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="D334" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E334" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F334" s="8" t="n"/>
+      <c r="G334" s="8" t="n"/>
+      <c r="H334" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I334" s="8" t="n">
+        <v>1024.9</v>
+      </c>
+      <c r="J334" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T01:00</t>
+        </is>
+      </c>
+      <c r="B335" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C335" s="9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D335" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="E335" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F335" s="9" t="n"/>
+      <c r="G335" s="9" t="n"/>
+      <c r="H335" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I335" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="J335" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T02:00</t>
+        </is>
+      </c>
+      <c r="B336" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C336" s="8" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="D336" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E336" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F336" s="8" t="n"/>
+      <c r="G336" s="8" t="n"/>
+      <c r="H336" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I336" s="8" t="n">
+        <v>1024.9</v>
+      </c>
+      <c r="J336" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T03:00</t>
+        </is>
+      </c>
+      <c r="B337" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C337" s="9" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D337" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E337" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F337" s="9" t="n"/>
+      <c r="G337" s="9" t="n"/>
+      <c r="H337" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I337" s="9" t="n">
+        <v>1024.9</v>
+      </c>
+      <c r="J337" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-21 00:03 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J337"/>
+  <dimension ref="A1:J357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -11376,6 +11376,682 @@
         <v>0</v>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T04:00</t>
+        </is>
+      </c>
+      <c r="B338" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C338" s="8" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D338" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E338" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" s="8" t="n"/>
+      <c r="G338" s="8" t="n"/>
+      <c r="H338" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I338" s="8" t="n">
+        <v>1024.8</v>
+      </c>
+      <c r="J338" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T05:00</t>
+        </is>
+      </c>
+      <c r="B339" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C339" s="9" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D339" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E339" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F339" s="9" t="n"/>
+      <c r="G339" s="9" t="n"/>
+      <c r="H339" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I339" s="9" t="n">
+        <v>1024.7</v>
+      </c>
+      <c r="J339" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T06:00</t>
+        </is>
+      </c>
+      <c r="B340" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C340" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D340" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E340" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" s="8" t="n"/>
+      <c r="G340" s="8" t="n"/>
+      <c r="H340" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I340" s="8" t="n">
+        <v>1024.8</v>
+      </c>
+      <c r="J340" s="8" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T07:00</t>
+        </is>
+      </c>
+      <c r="B341" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C341" s="9" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D341" s="9" t="n"/>
+      <c r="E341" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F341" s="9" t="n"/>
+      <c r="G341" s="9" t="n"/>
+      <c r="H341" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I341" s="9" t="n">
+        <v>1024.8</v>
+      </c>
+      <c r="J341" s="9" t="n">
+        <v>595.4</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T08:00</t>
+        </is>
+      </c>
+      <c r="B342" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C342" s="8" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D342" s="8" t="n"/>
+      <c r="E342" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F342" s="8" t="n"/>
+      <c r="G342" s="8" t="n"/>
+      <c r="H342" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I342" s="8" t="n">
+        <v>1024.5</v>
+      </c>
+      <c r="J342" s="8" t="n">
+        <v>1365.7</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T09:00</t>
+        </is>
+      </c>
+      <c r="B343" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C343" s="9" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D343" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="E343" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F343" s="9" t="n"/>
+      <c r="G343" s="9" t="n"/>
+      <c r="H343" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I343" s="9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="J343" s="9" t="n">
+        <v>1982.5</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T10:00</t>
+        </is>
+      </c>
+      <c r="B344" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C344" s="8" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="D344" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E344" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" s="8" t="n"/>
+      <c r="G344" s="8" t="n"/>
+      <c r="H344" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I344" s="8" t="n">
+        <v>1023.2</v>
+      </c>
+      <c r="J344" s="8" t="n">
+        <v>2662.8</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T11:00</t>
+        </is>
+      </c>
+      <c r="B345" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C345" s="9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D345" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E345" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" s="9" t="n"/>
+      <c r="G345" s="9" t="n"/>
+      <c r="H345" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I345" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J345" s="9" t="n">
+        <v>3131.8</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T12:00</t>
+        </is>
+      </c>
+      <c r="B346" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C346" s="8" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="D346" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E346" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F346" s="8" t="n"/>
+      <c r="G346" s="8" t="n"/>
+      <c r="H346" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I346" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J346" s="8" t="n">
+        <v>3408.9</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T13:00</t>
+        </is>
+      </c>
+      <c r="B347" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C347" s="9" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="D347" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E347" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F347" s="9" t="n"/>
+      <c r="G347" s="9" t="n"/>
+      <c r="H347" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I347" s="9" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J347" s="9" t="n">
+        <v>3476.7</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T14:00</t>
+        </is>
+      </c>
+      <c r="B348" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C348" s="8" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="D348" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E348" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F348" s="8" t="n"/>
+      <c r="G348" s="8" t="n"/>
+      <c r="H348" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I348" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J348" s="8" t="n">
+        <v>3394.5</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T15:00</t>
+        </is>
+      </c>
+      <c r="B349" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C349" s="9" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D349" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="E349" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F349" s="9" t="n"/>
+      <c r="G349" s="9" t="n"/>
+      <c r="H349" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I349" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J349" s="9" t="n">
+        <v>3078.6</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T16:00</t>
+        </is>
+      </c>
+      <c r="B350" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C350" s="8" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="D350" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="E350" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F350" s="8" t="n"/>
+      <c r="G350" s="8" t="n"/>
+      <c r="H350" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I350" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J350" s="8" t="n">
+        <v>2590.1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T17:00</t>
+        </is>
+      </c>
+      <c r="B351" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C351" s="9" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="D351" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="E351" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F351" s="9" t="n"/>
+      <c r="G351" s="9" t="n"/>
+      <c r="H351" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I351" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J351" s="9" t="n">
+        <v>1921.9</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T18:00</t>
+        </is>
+      </c>
+      <c r="B352" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C352" s="8" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="D352" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="E352" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" s="8" t="n"/>
+      <c r="G352" s="8" t="n"/>
+      <c r="H352" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I352" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J352" s="8" t="n">
+        <v>1280.2</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T19:00</t>
+        </is>
+      </c>
+      <c r="B353" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C353" s="9" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D353" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="E353" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" s="9" t="n"/>
+      <c r="G353" s="9" t="n"/>
+      <c r="H353" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I353" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J353" s="9" t="n">
+        <v>594.5</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T20:00</t>
+        </is>
+      </c>
+      <c r="B354" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C354" s="8" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D354" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="E354" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F354" s="8" t="n"/>
+      <c r="G354" s="8" t="n"/>
+      <c r="H354" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I354" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J354" s="8" t="n">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T21:00</t>
+        </is>
+      </c>
+      <c r="B355" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C355" s="9" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="D355" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E355" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" s="9" t="n"/>
+      <c r="G355" s="9" t="n"/>
+      <c r="H355" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I355" s="9" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J355" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-20T22:00</t>
+        </is>
+      </c>
+      <c r="B356" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C356" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D356" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E356" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F356" s="8" t="n"/>
+      <c r="G356" s="8" t="n"/>
+      <c r="H356" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I356" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J356" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-20T23:00</t>
+        </is>
+      </c>
+      <c r="B357" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C357" s="9" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D357" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="E357" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F357" s="9" t="n"/>
+      <c r="G357" s="9" t="n"/>
+      <c r="H357" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I357" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J357" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-21 04:26 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J357"/>
+  <dimension ref="A1:J361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -12052,6 +12052,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="358">
+      <c r="A358" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T00:00</t>
+        </is>
+      </c>
+      <c r="B358" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C358" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D358" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="E358" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F358" s="8" t="n"/>
+      <c r="G358" s="8" t="n"/>
+      <c r="H358" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I358" s="8" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J358" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T01:00</t>
+        </is>
+      </c>
+      <c r="B359" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C359" s="9" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="D359" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E359" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F359" s="9" t="n"/>
+      <c r="G359" s="9" t="n"/>
+      <c r="H359" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I359" s="9" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J359" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T02:00</t>
+        </is>
+      </c>
+      <c r="B360" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C360" s="8" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D360" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E360" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F360" s="8" t="n"/>
+      <c r="G360" s="8" t="n"/>
+      <c r="H360" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I360" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J360" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T03:00</t>
+        </is>
+      </c>
+      <c r="B361" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C361" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D361" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E361" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F361" s="9" t="n"/>
+      <c r="G361" s="9" t="n"/>
+      <c r="H361" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I361" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J361" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-21 23:57 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J361"/>
+  <dimension ref="A1:J381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -12188,6 +12188,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T04:00</t>
+        </is>
+      </c>
+      <c r="B362" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C362" s="8" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D362" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E362" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F362" s="8" t="n"/>
+      <c r="G362" s="8" t="n"/>
+      <c r="H362" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I362" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J362" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T05:00</t>
+        </is>
+      </c>
+      <c r="B363" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C363" s="9" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D363" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E363" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F363" s="9" t="n"/>
+      <c r="G363" s="9" t="n"/>
+      <c r="H363" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I363" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J363" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T06:00</t>
+        </is>
+      </c>
+      <c r="B364" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C364" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D364" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E364" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F364" s="8" t="n"/>
+      <c r="G364" s="8" t="n"/>
+      <c r="H364" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I364" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J364" s="8" t="n">
+        <v>68.3</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T07:00</t>
+        </is>
+      </c>
+      <c r="B365" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C365" s="9" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D365" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E365" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F365" s="9" t="n"/>
+      <c r="G365" s="9" t="n"/>
+      <c r="H365" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I365" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J365" s="9" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T08:00</t>
+        </is>
+      </c>
+      <c r="B366" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C366" s="8" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D366" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E366" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" s="8" t="n"/>
+      <c r="G366" s="8" t="n"/>
+      <c r="H366" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I366" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J366" s="8" t="n">
+        <v>1265.9</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T09:00</t>
+        </is>
+      </c>
+      <c r="B367" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C367" s="9" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D367" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E367" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" s="9" t="n"/>
+      <c r="G367" s="9" t="n"/>
+      <c r="H367" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I367" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J367" s="9" t="n">
+        <v>1924.4</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T10:00</t>
+        </is>
+      </c>
+      <c r="B368" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C368" s="8" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="D368" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E368" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" s="8" t="n"/>
+      <c r="G368" s="8" t="n"/>
+      <c r="H368" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I368" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J368" s="8" t="n">
+        <v>2358.6</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T11:00</t>
+        </is>
+      </c>
+      <c r="B369" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C369" s="9" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="D369" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="E369" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F369" s="9" t="n"/>
+      <c r="G369" s="9" t="n"/>
+      <c r="H369" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I369" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J369" s="9" t="n">
+        <v>2934</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T12:00</t>
+        </is>
+      </c>
+      <c r="B370" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C370" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D370" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E370" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F370" s="8" t="n"/>
+      <c r="G370" s="8" t="n"/>
+      <c r="H370" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I370" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J370" s="8" t="n">
+        <v>3098.5</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T13:00</t>
+        </is>
+      </c>
+      <c r="B371" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C371" s="9" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D371" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E371" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F371" s="9" t="n"/>
+      <c r="G371" s="9" t="n"/>
+      <c r="H371" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I371" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J371" s="9" t="n">
+        <v>3297.7</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T14:00</t>
+        </is>
+      </c>
+      <c r="B372" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C372" s="8" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D372" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="E372" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F372" s="8" t="n"/>
+      <c r="G372" s="8" t="n"/>
+      <c r="H372" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I372" s="8" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J372" s="8" t="n">
+        <v>3183.9</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T15:00</t>
+        </is>
+      </c>
+      <c r="B373" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C373" s="9" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D373" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E373" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F373" s="9" t="n"/>
+      <c r="G373" s="9" t="n"/>
+      <c r="H373" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I373" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J373" s="9" t="n">
+        <v>2988.9</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T16:00</t>
+        </is>
+      </c>
+      <c r="B374" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C374" s="8" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="D374" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E374" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F374" s="8" t="n"/>
+      <c r="G374" s="8" t="n"/>
+      <c r="H374" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I374" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J374" s="8" t="n">
+        <v>2476</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T17:00</t>
+        </is>
+      </c>
+      <c r="B375" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C375" s="9" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D375" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="E375" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F375" s="9" t="n"/>
+      <c r="G375" s="9" t="n"/>
+      <c r="H375" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I375" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J375" s="9" t="n">
+        <v>1849.2</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T18:00</t>
+        </is>
+      </c>
+      <c r="B376" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C376" s="8" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="D376" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E376" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F376" s="8" t="n"/>
+      <c r="G376" s="8" t="n"/>
+      <c r="H376" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I376" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J376" s="8" t="n">
+        <v>1075.3</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T19:00</t>
+        </is>
+      </c>
+      <c r="B377" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C377" s="9" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="D377" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E377" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F377" s="9" t="n"/>
+      <c r="G377" s="9" t="n"/>
+      <c r="H377" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I377" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J377" s="9" t="n">
+        <v>533.2</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T20:00</t>
+        </is>
+      </c>
+      <c r="B378" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C378" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="D378" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E378" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F378" s="8" t="n"/>
+      <c r="G378" s="8" t="n"/>
+      <c r="H378" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I378" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J378" s="8" t="n">
+        <v>126.2</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T21:00</t>
+        </is>
+      </c>
+      <c r="B379" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C379" s="9" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D379" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E379" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F379" s="9" t="n"/>
+      <c r="G379" s="9" t="n"/>
+      <c r="H379" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I379" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J379" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-21T22:00</t>
+        </is>
+      </c>
+      <c r="B380" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C380" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D380" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E380" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F380" s="8" t="n"/>
+      <c r="G380" s="8" t="n"/>
+      <c r="H380" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I380" s="8" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J380" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-21T23:00</t>
+        </is>
+      </c>
+      <c r="B381" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C381" s="9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D381" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E381" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F381" s="9" t="n"/>
+      <c r="G381" s="9" t="n"/>
+      <c r="H381" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I381" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J381" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-22 04:21 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J381"/>
+  <dimension ref="A1:J385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -12868,6 +12868,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T00:00</t>
+        </is>
+      </c>
+      <c r="B382" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C382" s="8" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D382" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E382" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F382" s="8" t="n"/>
+      <c r="G382" s="8" t="n"/>
+      <c r="H382" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I382" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J382" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T01:00</t>
+        </is>
+      </c>
+      <c r="B383" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C383" s="9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D383" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="E383" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F383" s="9" t="n"/>
+      <c r="G383" s="9" t="n"/>
+      <c r="H383" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I383" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J383" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T02:00</t>
+        </is>
+      </c>
+      <c r="B384" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C384" s="8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D384" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E384" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F384" s="8" t="n"/>
+      <c r="G384" s="8" t="n"/>
+      <c r="H384" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I384" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J384" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T03:00</t>
+        </is>
+      </c>
+      <c r="B385" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C385" s="9" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D385" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E385" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F385" s="9" t="n"/>
+      <c r="G385" s="9" t="n"/>
+      <c r="H385" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I385" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J385" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-23 00:01 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J385"/>
+  <dimension ref="A1:J405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -13004,6 +13004,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T04:00</t>
+        </is>
+      </c>
+      <c r="B386" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C386" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D386" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E386" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F386" s="8" t="n"/>
+      <c r="G386" s="8" t="n"/>
+      <c r="H386" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I386" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J386" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T05:00</t>
+        </is>
+      </c>
+      <c r="B387" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C387" s="9" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D387" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E387" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F387" s="9" t="n"/>
+      <c r="G387" s="9" t="n"/>
+      <c r="H387" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I387" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J387" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T06:00</t>
+        </is>
+      </c>
+      <c r="B388" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C388" s="8" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D388" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E388" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F388" s="8" t="n"/>
+      <c r="G388" s="8" t="n"/>
+      <c r="H388" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I388" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J388" s="8" t="n">
+        <v>84.90000000000001</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T07:00</t>
+        </is>
+      </c>
+      <c r="B389" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C389" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D389" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E389" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F389" s="9" t="n"/>
+      <c r="G389" s="9" t="n"/>
+      <c r="H389" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I389" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J389" s="9" t="n">
+        <v>413.4</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T08:00</t>
+        </is>
+      </c>
+      <c r="B390" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C390" s="8" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="D390" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E390" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F390" s="8" t="n"/>
+      <c r="G390" s="8" t="n"/>
+      <c r="H390" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I390" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J390" s="8" t="n">
+        <v>929.8</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:00</t>
+        </is>
+      </c>
+      <c r="B391" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C391" s="9" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D391" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E391" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F391" s="9" t="n"/>
+      <c r="G391" s="9" t="n"/>
+      <c r="H391" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I391" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J391" s="9" t="n">
+        <v>1780.1</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T10:00</t>
+        </is>
+      </c>
+      <c r="B392" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C392" s="8" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="D392" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E392" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F392" s="8" t="n"/>
+      <c r="G392" s="8" t="n"/>
+      <c r="H392" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I392" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J392" s="8" t="n">
+        <v>2341.1</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T11:00</t>
+        </is>
+      </c>
+      <c r="B393" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C393" s="9" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D393" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E393" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F393" s="9" t="n"/>
+      <c r="G393" s="9" t="n"/>
+      <c r="H393" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I393" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J393" s="9" t="n">
+        <v>2861.5</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T12:00</t>
+        </is>
+      </c>
+      <c r="B394" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C394" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="D394" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E394" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F394" s="8" t="n"/>
+      <c r="G394" s="8" t="n"/>
+      <c r="H394" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I394" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J394" s="8" t="n">
+        <v>3027.4</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T13:00</t>
+        </is>
+      </c>
+      <c r="B395" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C395" s="9" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="D395" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="E395" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F395" s="9" t="n"/>
+      <c r="G395" s="9" t="n"/>
+      <c r="H395" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I395" s="9" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J395" s="9" t="n">
+        <v>1900.4</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T14:00</t>
+        </is>
+      </c>
+      <c r="B396" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C396" s="8" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="D396" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E396" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F396" s="8" t="n"/>
+      <c r="G396" s="8" t="n"/>
+      <c r="H396" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I396" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J396" s="8" t="n">
+        <v>2530.4</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T15:00</t>
+        </is>
+      </c>
+      <c r="B397" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C397" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D397" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E397" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F397" s="9" t="n"/>
+      <c r="G397" s="9" t="n"/>
+      <c r="H397" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I397" s="9" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J397" s="9" t="n">
+        <v>2248.2</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T16:00</t>
+        </is>
+      </c>
+      <c r="B398" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C398" s="8" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="D398" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="E398" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F398" s="8" t="n"/>
+      <c r="G398" s="8" t="n"/>
+      <c r="H398" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I398" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J398" s="8" t="n">
+        <v>1825.4</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T17:00</t>
+        </is>
+      </c>
+      <c r="B399" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C399" s="9" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D399" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E399" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F399" s="9" t="n"/>
+      <c r="G399" s="9" t="n"/>
+      <c r="H399" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I399" s="9" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J399" s="9" t="n">
+        <v>1448.5</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T18:00</t>
+        </is>
+      </c>
+      <c r="B400" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C400" s="8" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="D400" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E400" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F400" s="8" t="n"/>
+      <c r="G400" s="8" t="n"/>
+      <c r="H400" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I400" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J400" s="8" t="n">
+        <v>1069.5</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T19:00</t>
+        </is>
+      </c>
+      <c r="B401" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C401" s="9" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D401" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="E401" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F401" s="9" t="n"/>
+      <c r="G401" s="9" t="n"/>
+      <c r="H401" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I401" s="9" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J401" s="9" t="n">
+        <v>456.2</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T20:00</t>
+        </is>
+      </c>
+      <c r="B402" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C402" s="8" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D402" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E402" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F402" s="8" t="n"/>
+      <c r="G402" s="8" t="n"/>
+      <c r="H402" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I402" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J402" s="8" t="n">
+        <v>63.1</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T21:00</t>
+        </is>
+      </c>
+      <c r="B403" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C403" s="9" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D403" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E403" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F403" s="9" t="n"/>
+      <c r="G403" s="9" t="n"/>
+      <c r="H403" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I403" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J403" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-22T22:00</t>
+        </is>
+      </c>
+      <c r="B404" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C404" s="8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D404" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="E404" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F404" s="8" t="n"/>
+      <c r="G404" s="8" t="n"/>
+      <c r="H404" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I404" s="8" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J404" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-22T23:00</t>
+        </is>
+      </c>
+      <c r="B405" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C405" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D405" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E405" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F405" s="9" t="n"/>
+      <c r="G405" s="9" t="n"/>
+      <c r="H405" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I405" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J405" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-23 03:59 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J405"/>
+  <dimension ref="A1:J409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -13684,6 +13684,140 @@
         <v>0</v>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T00:00</t>
+        </is>
+      </c>
+      <c r="B406" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C406" s="8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D406" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E406" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F406" s="8" t="n"/>
+      <c r="G406" s="8" t="n"/>
+      <c r="H406" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I406" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J406" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T01:00</t>
+        </is>
+      </c>
+      <c r="B407" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C407" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D407" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E407" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F407" s="9" t="n"/>
+      <c r="G407" s="9" t="n"/>
+      <c r="H407" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I407" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J407" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T02:00</t>
+        </is>
+      </c>
+      <c r="B408" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C408" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="D408" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E408" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F408" s="8" t="n"/>
+      <c r="G408" s="8" t="n"/>
+      <c r="H408" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I408" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J408" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T03:00</t>
+        </is>
+      </c>
+      <c r="B409" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C409" s="9" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D409" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E409" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F409" s="9" t="n"/>
+      <c r="G409" s="9" t="n"/>
+      <c r="H409" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I409" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J409" s="9" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-23 23:52 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J409"/>
+  <dimension ref="A1:J429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -13818,6 +13818,682 @@
       </c>
       <c r="J409" s="9" t="n"/>
     </row>
+    <row r="410">
+      <c r="A410" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T04:00</t>
+        </is>
+      </c>
+      <c r="B410" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C410" s="8" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D410" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E410" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F410" s="8" t="n"/>
+      <c r="G410" s="8" t="n"/>
+      <c r="H410" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I410" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J410" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T05:00</t>
+        </is>
+      </c>
+      <c r="B411" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C411" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D411" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E411" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F411" s="9" t="n"/>
+      <c r="G411" s="9" t="n"/>
+      <c r="H411" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I411" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J411" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T06:00</t>
+        </is>
+      </c>
+      <c r="B412" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C412" s="8" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D412" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E412" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F412" s="8" t="n"/>
+      <c r="G412" s="8" t="n"/>
+      <c r="H412" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I412" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J412" s="8" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T07:00</t>
+        </is>
+      </c>
+      <c r="B413" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C413" s="9" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D413" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E413" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F413" s="9" t="n"/>
+      <c r="G413" s="9" t="n"/>
+      <c r="H413" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I413" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J413" s="9" t="n">
+        <v>143.4</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T08:00</t>
+        </is>
+      </c>
+      <c r="B414" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C414" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D414" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E414" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F414" s="8" t="n"/>
+      <c r="G414" s="8" t="n"/>
+      <c r="H414" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I414" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J414" s="8" t="n">
+        <v>337.7</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T09:00</t>
+        </is>
+      </c>
+      <c r="B415" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C415" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D415" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="E415" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F415" s="9" t="n"/>
+      <c r="G415" s="9" t="n"/>
+      <c r="H415" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I415" s="9" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J415" s="9" t="n">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T10:00</t>
+        </is>
+      </c>
+      <c r="B416" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C416" s="8" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D416" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E416" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F416" s="8" t="n"/>
+      <c r="G416" s="8" t="n"/>
+      <c r="H416" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I416" s="8" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J416" s="8" t="n">
+        <v>648.7</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T11:00</t>
+        </is>
+      </c>
+      <c r="B417" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C417" s="9" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="D417" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E417" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F417" s="9" t="n"/>
+      <c r="G417" s="9" t="n"/>
+      <c r="H417" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I417" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J417" s="9" t="n">
+        <v>829.6</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T12:00</t>
+        </is>
+      </c>
+      <c r="B418" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C418" s="8" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D418" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E418" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F418" s="8" t="n"/>
+      <c r="G418" s="8" t="n"/>
+      <c r="H418" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I418" s="8" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="J418" s="8" t="n">
+        <v>203.9</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T13:00</t>
+        </is>
+      </c>
+      <c r="B419" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C419" s="9" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D419" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E419" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F419" s="9" t="n"/>
+      <c r="G419" s="9" t="n"/>
+      <c r="H419" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I419" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J419" s="9" t="n">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T14:00</t>
+        </is>
+      </c>
+      <c r="B420" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C420" s="8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D420" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E420" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F420" s="8" t="n"/>
+      <c r="G420" s="8" t="n"/>
+      <c r="H420" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I420" s="8" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J420" s="8" t="n"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T15:00</t>
+        </is>
+      </c>
+      <c r="B421" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C421" s="9" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D421" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="E421" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F421" s="9" t="n"/>
+      <c r="G421" s="9" t="n"/>
+      <c r="H421" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I421" s="9" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="J421" s="9" t="n"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T16:00</t>
+        </is>
+      </c>
+      <c r="B422" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C422" s="8" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="D422" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E422" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F422" s="8" t="n"/>
+      <c r="G422" s="8" t="n"/>
+      <c r="H422" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I422" s="8" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J422" s="8" t="n">
+        <v>2010.1</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T17:00</t>
+        </is>
+      </c>
+      <c r="B423" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C423" s="9" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="D423" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E423" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F423" s="9" t="n"/>
+      <c r="G423" s="9" t="n"/>
+      <c r="H423" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I423" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J423" s="9" t="n">
+        <v>1996.2</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T18:00</t>
+        </is>
+      </c>
+      <c r="B424" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C424" s="8" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D424" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E424" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F424" s="8" t="n"/>
+      <c r="G424" s="8" t="n"/>
+      <c r="H424" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I424" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J424" s="8" t="n">
+        <v>1242.8</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T19:00</t>
+        </is>
+      </c>
+      <c r="B425" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C425" s="9" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D425" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E425" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F425" s="9" t="n"/>
+      <c r="G425" s="9" t="n"/>
+      <c r="H425" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I425" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J425" s="9" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T20:00</t>
+        </is>
+      </c>
+      <c r="B426" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C426" s="8" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D426" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E426" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F426" s="8" t="n"/>
+      <c r="G426" s="8" t="n"/>
+      <c r="H426" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I426" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J426" s="8" t="n">
+        <v>58.2</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T21:00</t>
+        </is>
+      </c>
+      <c r="B427" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C427" s="9" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="D427" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="E427" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F427" s="9" t="n"/>
+      <c r="G427" s="9" t="n"/>
+      <c r="H427" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I427" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J427" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-23T22:00</t>
+        </is>
+      </c>
+      <c r="B428" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C428" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D428" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E428" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F428" s="8" t="n"/>
+      <c r="G428" s="8" t="n"/>
+      <c r="H428" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I428" s="8" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J428" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-23T23:00</t>
+        </is>
+      </c>
+      <c r="B429" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C429" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D429" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E429" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F429" s="9" t="n"/>
+      <c r="G429" s="9" t="n"/>
+      <c r="H429" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I429" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J429" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-24 04:20 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J429"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -14494,6 +14494,112 @@
         <v>0</v>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T00:00</t>
+        </is>
+      </c>
+      <c r="B430" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C430" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D430" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E430" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F430" s="8" t="n"/>
+      <c r="G430" s="8" t="n"/>
+      <c r="H430" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I430" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J430" s="8" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-24T01:00</t>
+        </is>
+      </c>
+      <c r="B431" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C431" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D431" s="10" t="n"/>
+      <c r="E431" s="10" t="n"/>
+      <c r="F431" s="10" t="n"/>
+      <c r="G431" s="10" t="n"/>
+      <c r="H431" s="10" t="n"/>
+      <c r="I431" s="10" t="n"/>
+      <c r="J431" s="10" t="n"/>
+    </row>
+    <row r="432">
+      <c r="A432" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-24T02:00</t>
+        </is>
+      </c>
+      <c r="B432" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C432" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D432" s="10" t="n"/>
+      <c r="E432" s="10" t="n"/>
+      <c r="F432" s="10" t="n"/>
+      <c r="G432" s="10" t="n"/>
+      <c r="H432" s="10" t="n"/>
+      <c r="I432" s="10" t="n"/>
+      <c r="J432" s="10" t="n"/>
+    </row>
+    <row r="433">
+      <c r="A433" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-24T03:00</t>
+        </is>
+      </c>
+      <c r="B433" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C433" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D433" s="10" t="n"/>
+      <c r="E433" s="10" t="n"/>
+      <c r="F433" s="10" t="n"/>
+      <c r="G433" s="10" t="n"/>
+      <c r="H433" s="10" t="n"/>
+      <c r="I433" s="10" t="n"/>
+      <c r="J433" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-24 23:55 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J433"/>
+  <dimension ref="A1:J453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -14600,6 +14600,686 @@
       <c r="I433" s="10" t="n"/>
       <c r="J433" s="10" t="n"/>
     </row>
+    <row r="434">
+      <c r="A434" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T04:00</t>
+        </is>
+      </c>
+      <c r="B434" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C434" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D434" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E434" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F434" s="8" t="n"/>
+      <c r="G434" s="8" t="n"/>
+      <c r="H434" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I434" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J434" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T05:00</t>
+        </is>
+      </c>
+      <c r="B435" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C435" s="9" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D435" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E435" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F435" s="9" t="n"/>
+      <c r="G435" s="9" t="n"/>
+      <c r="H435" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I435" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J435" s="9" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T06:00</t>
+        </is>
+      </c>
+      <c r="B436" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C436" s="8" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D436" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E436" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F436" s="8" t="n"/>
+      <c r="G436" s="8" t="n"/>
+      <c r="H436" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I436" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J436" s="8" t="n">
+        <v>60.6</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T07:00</t>
+        </is>
+      </c>
+      <c r="B437" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C437" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D437" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E437" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F437" s="9" t="n"/>
+      <c r="G437" s="9" t="n"/>
+      <c r="H437" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I437" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J437" s="9" t="n">
+        <v>536.6</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T08:00</t>
+        </is>
+      </c>
+      <c r="B438" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C438" s="8" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="D438" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E438" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F438" s="8" t="n"/>
+      <c r="G438" s="8" t="n"/>
+      <c r="H438" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I438" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J438" s="8" t="n">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T09:00</t>
+        </is>
+      </c>
+      <c r="B439" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C439" s="9" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D439" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E439" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F439" s="9" t="n"/>
+      <c r="G439" s="9" t="n"/>
+      <c r="H439" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I439" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J439" s="9" t="n">
+        <v>1558.7</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T10:00</t>
+        </is>
+      </c>
+      <c r="B440" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C440" s="8" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D440" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E440" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F440" s="8" t="n"/>
+      <c r="G440" s="8" t="n"/>
+      <c r="H440" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I440" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J440" s="8" t="n">
+        <v>1919.4</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T11:00</t>
+        </is>
+      </c>
+      <c r="B441" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C441" s="9" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="D441" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E441" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F441" s="9" t="n"/>
+      <c r="G441" s="9" t="n"/>
+      <c r="H441" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I441" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J441" s="9" t="n">
+        <v>3042.1</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T12:00</t>
+        </is>
+      </c>
+      <c r="B442" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C442" s="8" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="D442" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E442" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F442" s="8" t="n"/>
+      <c r="G442" s="8" t="n"/>
+      <c r="H442" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I442" s="8" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J442" s="8" t="n">
+        <v>3075.9</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T13:00</t>
+        </is>
+      </c>
+      <c r="B443" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C443" s="9" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D443" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E443" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F443" s="9" t="n"/>
+      <c r="G443" s="9" t="n"/>
+      <c r="H443" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I443" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J443" s="9" t="n">
+        <v>3340.7</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T14:00</t>
+        </is>
+      </c>
+      <c r="B444" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C444" s="8" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="D444" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E444" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F444" s="8" t="n"/>
+      <c r="G444" s="8" t="n"/>
+      <c r="H444" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I444" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J444" s="8" t="n">
+        <v>3202.2</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T15:00</t>
+        </is>
+      </c>
+      <c r="B445" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C445" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="D445" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E445" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F445" s="9" t="n"/>
+      <c r="G445" s="9" t="n"/>
+      <c r="H445" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I445" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J445" s="9" t="n">
+        <v>2902.5</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T16:00</t>
+        </is>
+      </c>
+      <c r="B446" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C446" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D446" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E446" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F446" s="8" t="n"/>
+      <c r="G446" s="8" t="n"/>
+      <c r="H446" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I446" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J446" s="8" t="n">
+        <v>2307.5</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T17:00</t>
+        </is>
+      </c>
+      <c r="B447" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C447" s="9" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D447" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E447" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F447" s="9" t="n"/>
+      <c r="G447" s="9" t="n"/>
+      <c r="H447" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I447" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J447" s="9" t="n">
+        <v>1513.6</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T18:00</t>
+        </is>
+      </c>
+      <c r="B448" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C448" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="D448" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E448" s="8" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F448" s="8" t="n"/>
+      <c r="G448" s="8" t="n"/>
+      <c r="H448" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I448" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J448" s="8" t="n">
+        <v>561.9</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T19:00</t>
+        </is>
+      </c>
+      <c r="B449" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C449" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D449" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E449" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F449" s="9" t="n"/>
+      <c r="G449" s="9" t="n"/>
+      <c r="H449" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I449" s="9" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J449" s="9" t="n">
+        <v>89.40000000000001</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T20:00</t>
+        </is>
+      </c>
+      <c r="B450" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C450" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D450" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E450" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F450" s="8" t="n"/>
+      <c r="G450" s="8" t="n"/>
+      <c r="H450" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I450" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J450" s="8" t="n">
+        <v>38.8</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T21:00</t>
+        </is>
+      </c>
+      <c r="B451" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C451" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D451" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E451" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F451" s="9" t="n"/>
+      <c r="G451" s="9" t="n"/>
+      <c r="H451" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I451" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J451" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-24T22:00</t>
+        </is>
+      </c>
+      <c r="B452" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C452" s="8" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D452" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E452" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F452" s="8" t="n"/>
+      <c r="G452" s="8" t="n"/>
+      <c r="H452" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I452" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J452" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-24T23:00</t>
+        </is>
+      </c>
+      <c r="B453" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C453" s="9" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D453" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E453" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F453" s="9" t="n"/>
+      <c r="G453" s="9" t="n"/>
+      <c r="H453" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I453" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J453" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-25 04:42 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J453"/>
+  <dimension ref="A1:J458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -15280,6 +15280,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="454">
+      <c r="A454" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T00:00</t>
+        </is>
+      </c>
+      <c r="B454" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C454" s="8" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D454" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E454" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F454" s="8" t="n"/>
+      <c r="G454" s="8" t="n"/>
+      <c r="H454" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I454" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J454" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T01:00</t>
+        </is>
+      </c>
+      <c r="B455" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C455" s="9" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D455" s="9" t="n">
+        <v>96</v>
+      </c>
+      <c r="E455" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F455" s="9" t="n"/>
+      <c r="G455" s="9" t="n"/>
+      <c r="H455" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I455" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J455" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T02:00</t>
+        </is>
+      </c>
+      <c r="B456" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C456" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D456" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E456" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F456" s="8" t="n"/>
+      <c r="G456" s="8" t="n"/>
+      <c r="H456" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I456" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J456" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T03:00</t>
+        </is>
+      </c>
+      <c r="B457" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C457" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D457" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="E457" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F457" s="9" t="n"/>
+      <c r="G457" s="9" t="n"/>
+      <c r="H457" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I457" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J457" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T04:00</t>
+        </is>
+      </c>
+      <c r="B458" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C458" s="8" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D458" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="E458" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F458" s="8" t="n"/>
+      <c r="G458" s="8" t="n"/>
+      <c r="H458" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I458" s="8" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J458" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-26 00:01 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J458"/>
+  <dimension ref="A1:J477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -15450,6 +15450,646 @@
         <v>0</v>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T05:00</t>
+        </is>
+      </c>
+      <c r="B459" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C459" s="9" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D459" s="9" t="n">
+        <v>99</v>
+      </c>
+      <c r="E459" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F459" s="9" t="n"/>
+      <c r="G459" s="9" t="n"/>
+      <c r="H459" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I459" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J459" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T06:00</t>
+        </is>
+      </c>
+      <c r="B460" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C460" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D460" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E460" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F460" s="8" t="n"/>
+      <c r="G460" s="8" t="n"/>
+      <c r="H460" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I460" s="8" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J460" s="8" t="n">
+        <v>82.59999999999999</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T07:00</t>
+        </is>
+      </c>
+      <c r="B461" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C461" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D461" s="9" t="n"/>
+      <c r="E461" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F461" s="9" t="n"/>
+      <c r="G461" s="9" t="n"/>
+      <c r="H461" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I461" s="9" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J461" s="9" t="n">
+        <v>313.5</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T08:00</t>
+        </is>
+      </c>
+      <c r="B462" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C462" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D462" s="8" t="n"/>
+      <c r="E462" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F462" s="8" t="n"/>
+      <c r="G462" s="8" t="n"/>
+      <c r="H462" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I462" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J462" s="8" t="n">
+        <v>661.8</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T09:00</t>
+        </is>
+      </c>
+      <c r="B463" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C463" s="9" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D463" s="9" t="n"/>
+      <c r="E463" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F463" s="9" t="n"/>
+      <c r="G463" s="9" t="n"/>
+      <c r="H463" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I463" s="9" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J463" s="9" t="n">
+        <v>1609.5</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T10:00</t>
+        </is>
+      </c>
+      <c r="B464" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C464" s="8" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="D464" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E464" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F464" s="8" t="n"/>
+      <c r="G464" s="8" t="n"/>
+      <c r="H464" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I464" s="8" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J464" s="8" t="n">
+        <v>2121.5</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T11:00</t>
+        </is>
+      </c>
+      <c r="B465" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C465" s="9" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="D465" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="E465" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F465" s="9" t="n"/>
+      <c r="G465" s="9" t="n"/>
+      <c r="H465" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I465" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J465" s="9" t="n">
+        <v>2580.6</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T12:00</t>
+        </is>
+      </c>
+      <c r="B466" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C466" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D466" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E466" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F466" s="8" t="n"/>
+      <c r="G466" s="8" t="n"/>
+      <c r="H466" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I466" s="8" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J466" s="8" t="n">
+        <v>3053.3</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T13:00</t>
+        </is>
+      </c>
+      <c r="B467" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C467" s="9" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="D467" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E467" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F467" s="9" t="n"/>
+      <c r="G467" s="9" t="n"/>
+      <c r="H467" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I467" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J467" s="9" t="n">
+        <v>3319.7</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T14:00</t>
+        </is>
+      </c>
+      <c r="B468" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C468" s="8" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="D468" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E468" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F468" s="8" t="n"/>
+      <c r="G468" s="8" t="n"/>
+      <c r="H468" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I468" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J468" s="8" t="n">
+        <v>3314</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T15:00</t>
+        </is>
+      </c>
+      <c r="B469" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C469" s="9" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="D469" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="E469" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F469" s="9" t="n"/>
+      <c r="G469" s="9" t="n"/>
+      <c r="H469" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I469" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J469" s="9" t="n">
+        <v>3014.8</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T16:00</t>
+        </is>
+      </c>
+      <c r="B470" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C470" s="8" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D470" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="E470" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F470" s="8" t="n"/>
+      <c r="G470" s="8" t="n"/>
+      <c r="H470" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I470" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J470" s="8" t="n">
+        <v>2526.6</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T17:00</t>
+        </is>
+      </c>
+      <c r="B471" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C471" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="D471" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E471" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F471" s="9" t="n"/>
+      <c r="G471" s="9" t="n"/>
+      <c r="H471" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I471" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J471" s="9" t="n">
+        <v>1961.7</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T18:00</t>
+        </is>
+      </c>
+      <c r="B472" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C472" s="8" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="D472" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E472" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F472" s="8" t="n"/>
+      <c r="G472" s="8" t="n"/>
+      <c r="H472" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I472" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J472" s="8" t="n">
+        <v>1254.7</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T19:00</t>
+        </is>
+      </c>
+      <c r="B473" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C473" s="9" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="D473" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E473" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F473" s="9" t="n"/>
+      <c r="G473" s="9" t="n"/>
+      <c r="H473" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I473" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J473" s="9" t="n">
+        <v>530.4</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T20:00</t>
+        </is>
+      </c>
+      <c r="B474" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C474" s="8" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="D474" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E474" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F474" s="8" t="n"/>
+      <c r="G474" s="8" t="n"/>
+      <c r="H474" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I474" s="8" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J474" s="8" t="n">
+        <v>94.3</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T21:00</t>
+        </is>
+      </c>
+      <c r="B475" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C475" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="D475" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="E475" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F475" s="9" t="n"/>
+      <c r="G475" s="9" t="n"/>
+      <c r="H475" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I475" s="9" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J475" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:00</t>
+        </is>
+      </c>
+      <c r="B476" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C476" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="D476" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E476" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F476" s="8" t="n"/>
+      <c r="G476" s="8" t="n"/>
+      <c r="H476" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I476" s="8" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J476" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-25T23:00</t>
+        </is>
+      </c>
+      <c r="B477" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C477" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D477" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E477" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F477" s="9" t="n"/>
+      <c r="G477" s="9" t="n"/>
+      <c r="H477" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I477" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J477" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-26 04:17 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J477"/>
+  <dimension ref="A1:J481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -16090,6 +16090,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="478">
+      <c r="A478" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T00:00</t>
+        </is>
+      </c>
+      <c r="B478" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C478" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D478" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E478" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F478" s="8" t="n"/>
+      <c r="G478" s="8" t="n"/>
+      <c r="H478" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I478" s="8" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J478" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T01:00</t>
+        </is>
+      </c>
+      <c r="B479" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C479" s="9" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D479" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="E479" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F479" s="9" t="n"/>
+      <c r="G479" s="9" t="n"/>
+      <c r="H479" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I479" s="9" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J479" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T02:00</t>
+        </is>
+      </c>
+      <c r="B480" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C480" s="8" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D480" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E480" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F480" s="8" t="n"/>
+      <c r="G480" s="8" t="n"/>
+      <c r="H480" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I480" s="8" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="J480" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T03:00</t>
+        </is>
+      </c>
+      <c r="B481" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C481" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D481" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E481" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F481" s="9" t="n"/>
+      <c r="G481" s="9" t="n"/>
+      <c r="H481" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I481" s="9" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="J481" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-26 23:59 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J481"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -16226,6 +16226,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T04:00</t>
+        </is>
+      </c>
+      <c r="B482" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C482" s="8" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D482" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E482" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F482" s="8" t="n"/>
+      <c r="G482" s="8" t="n"/>
+      <c r="H482" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I482" s="8" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J482" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T05:00</t>
+        </is>
+      </c>
+      <c r="B483" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C483" s="9" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D483" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E483" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F483" s="9" t="n"/>
+      <c r="G483" s="9" t="n"/>
+      <c r="H483" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I483" s="9" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J483" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T06:00</t>
+        </is>
+      </c>
+      <c r="B484" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C484" s="8" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D484" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E484" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F484" s="8" t="n"/>
+      <c r="G484" s="8" t="n"/>
+      <c r="H484" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I484" s="8" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="J484" s="8" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T07:00</t>
+        </is>
+      </c>
+      <c r="B485" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C485" s="9" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D485" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E485" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F485" s="9" t="n"/>
+      <c r="G485" s="9" t="n"/>
+      <c r="H485" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I485" s="9" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J485" s="9" t="n">
+        <v>576.2</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T08:00</t>
+        </is>
+      </c>
+      <c r="B486" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C486" s="8" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D486" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E486" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F486" s="8" t="n"/>
+      <c r="G486" s="8" t="n"/>
+      <c r="H486" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I486" s="8" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J486" s="8" t="n">
+        <v>1272.8</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T09:00</t>
+        </is>
+      </c>
+      <c r="B487" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C487" s="9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D487" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="E487" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F487" s="9" t="n"/>
+      <c r="G487" s="9" t="n"/>
+      <c r="H487" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I487" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J487" s="9" t="n">
+        <v>1893</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T10:00</t>
+        </is>
+      </c>
+      <c r="B488" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C488" s="8" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D488" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E488" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F488" s="8" t="n"/>
+      <c r="G488" s="8" t="n"/>
+      <c r="H488" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I488" s="8" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="J488" s="8" t="n">
+        <v>2477.9</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T11:00</t>
+        </is>
+      </c>
+      <c r="B489" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C489" s="9" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D489" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="E489" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F489" s="9" t="n"/>
+      <c r="G489" s="9" t="n"/>
+      <c r="H489" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I489" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J489" s="9" t="n">
+        <v>2990.5</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T12:00</t>
+        </is>
+      </c>
+      <c r="B490" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C490" s="8" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="D490" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E490" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F490" s="8" t="n"/>
+      <c r="G490" s="8" t="n"/>
+      <c r="H490" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I490" s="8" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J490" s="8" t="n">
+        <v>3291.2</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T13:00</t>
+        </is>
+      </c>
+      <c r="B491" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C491" s="9" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="D491" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E491" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F491" s="9" t="n"/>
+      <c r="G491" s="9" t="n"/>
+      <c r="H491" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I491" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J491" s="9" t="n">
+        <v>3393.7</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T14:00</t>
+        </is>
+      </c>
+      <c r="B492" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C492" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="D492" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E492" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F492" s="8" t="n"/>
+      <c r="G492" s="8" t="n"/>
+      <c r="H492" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I492" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J492" s="8" t="n">
+        <v>3282.6</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T15:00</t>
+        </is>
+      </c>
+      <c r="B493" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C493" s="9" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="D493" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E493" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F493" s="9" t="n"/>
+      <c r="G493" s="9" t="n"/>
+      <c r="H493" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I493" s="9" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J493" s="9" t="n">
+        <v>2977.1</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T16:00</t>
+        </is>
+      </c>
+      <c r="B494" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C494" s="8" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="D494" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="E494" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F494" s="8" t="n"/>
+      <c r="G494" s="8" t="n"/>
+      <c r="H494" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I494" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J494" s="8" t="n">
+        <v>2475.5</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T17:00</t>
+        </is>
+      </c>
+      <c r="B495" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C495" s="9" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="D495" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E495" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F495" s="9" t="n"/>
+      <c r="G495" s="9" t="n"/>
+      <c r="H495" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I495" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J495" s="9" t="n">
+        <v>1919.1</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T18:00</t>
+        </is>
+      </c>
+      <c r="B496" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C496" s="8" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="D496" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E496" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F496" s="8" t="n"/>
+      <c r="G496" s="8" t="n"/>
+      <c r="H496" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I496" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J496" s="8" t="n">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T19:00</t>
+        </is>
+      </c>
+      <c r="B497" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C497" s="9" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="D497" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E497" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F497" s="9" t="n"/>
+      <c r="G497" s="9" t="n"/>
+      <c r="H497" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I497" s="9" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J497" s="9" t="n">
+        <v>308.7</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T20:00</t>
+        </is>
+      </c>
+      <c r="B498" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C498" s="8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D498" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E498" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F498" s="8" t="n"/>
+      <c r="G498" s="8" t="n"/>
+      <c r="H498" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I498" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J498" s="8" t="n">
+        <v>78.2</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T21:00</t>
+        </is>
+      </c>
+      <c r="B499" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C499" s="9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D499" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E499" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F499" s="9" t="n"/>
+      <c r="G499" s="9" t="n"/>
+      <c r="H499" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I499" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J499" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-26T22:00</t>
+        </is>
+      </c>
+      <c r="B500" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C500" s="8" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="D500" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E500" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F500" s="8" t="n"/>
+      <c r="G500" s="8" t="n"/>
+      <c r="H500" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I500" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J500" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-26T23:00</t>
+        </is>
+      </c>
+      <c r="B501" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C501" s="9" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D501" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E501" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F501" s="9" t="n"/>
+      <c r="G501" s="9" t="n"/>
+      <c r="H501" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I501" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J501" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-27 04:40 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J501"/>
+  <dimension ref="A1:J506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -16906,6 +16906,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="502">
+      <c r="A502" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T00:00</t>
+        </is>
+      </c>
+      <c r="B502" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C502" s="8" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D502" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E502" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F502" s="8" t="n"/>
+      <c r="G502" s="8" t="n"/>
+      <c r="H502" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I502" s="8" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J502" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T01:00</t>
+        </is>
+      </c>
+      <c r="B503" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C503" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D503" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="E503" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F503" s="9" t="n"/>
+      <c r="G503" s="9" t="n"/>
+      <c r="H503" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I503" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J503" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T02:00</t>
+        </is>
+      </c>
+      <c r="B504" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C504" s="8" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D504" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E504" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F504" s="8" t="n"/>
+      <c r="G504" s="8" t="n"/>
+      <c r="H504" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I504" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J504" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T03:00</t>
+        </is>
+      </c>
+      <c r="B505" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C505" s="9" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D505" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E505" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F505" s="9" t="n"/>
+      <c r="G505" s="9" t="n"/>
+      <c r="H505" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I505" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J505" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T04:00</t>
+        </is>
+      </c>
+      <c r="B506" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C506" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D506" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E506" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F506" s="8" t="n"/>
+      <c r="G506" s="8" t="n"/>
+      <c r="H506" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I506" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J506" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-27 23:57 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J506"/>
+  <dimension ref="A1:J525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -17076,6 +17076,652 @@
         <v>0</v>
       </c>
     </row>
+    <row r="507">
+      <c r="A507" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T05:00</t>
+        </is>
+      </c>
+      <c r="B507" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C507" s="9" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="D507" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E507" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F507" s="9" t="n"/>
+      <c r="G507" s="9" t="n"/>
+      <c r="H507" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I507" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J507" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T06:00</t>
+        </is>
+      </c>
+      <c r="B508" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C508" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D508" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E508" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F508" s="8" t="n"/>
+      <c r="G508" s="8" t="n"/>
+      <c r="H508" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I508" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J508" s="8" t="n">
+        <v>92.59999999999999</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T07:00</t>
+        </is>
+      </c>
+      <c r="B509" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C509" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D509" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E509" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F509" s="9" t="n"/>
+      <c r="G509" s="9" t="n"/>
+      <c r="H509" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I509" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J509" s="9" t="n">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T08:00</t>
+        </is>
+      </c>
+      <c r="B510" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C510" s="8" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D510" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E510" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F510" s="8" t="n"/>
+      <c r="G510" s="8" t="n"/>
+      <c r="H510" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I510" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J510" s="8" t="n">
+        <v>1134.4</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T09:00</t>
+        </is>
+      </c>
+      <c r="B511" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C511" s="9" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D511" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E511" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F511" s="9" t="n"/>
+      <c r="G511" s="9" t="n"/>
+      <c r="H511" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I511" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J511" s="9" t="n">
+        <v>1762.9</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T10:00</t>
+        </is>
+      </c>
+      <c r="B512" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C512" s="8" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="D512" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E512" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F512" s="8" t="n"/>
+      <c r="G512" s="8" t="n"/>
+      <c r="H512" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I512" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J512" s="8" t="n">
+        <v>2387.1</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T11:00</t>
+        </is>
+      </c>
+      <c r="B513" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C513" s="9" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="D513" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E513" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F513" s="9" t="n"/>
+      <c r="G513" s="9" t="n"/>
+      <c r="H513" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I513" s="9" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J513" s="9" t="n">
+        <v>2933.7</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T12:00</t>
+        </is>
+      </c>
+      <c r="B514" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C514" s="8" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="D514" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="E514" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F514" s="8" t="n"/>
+      <c r="G514" s="8" t="n"/>
+      <c r="H514" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I514" s="8" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J514" s="8" t="n">
+        <v>3235.2</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T13:00</t>
+        </is>
+      </c>
+      <c r="B515" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C515" s="9" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="D515" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E515" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F515" s="9" t="n"/>
+      <c r="G515" s="9" t="n"/>
+      <c r="H515" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I515" s="9" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J515" s="9" t="n">
+        <v>3322</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T14:00</t>
+        </is>
+      </c>
+      <c r="B516" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C516" s="8" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="D516" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="E516" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F516" s="8" t="n"/>
+      <c r="G516" s="8" t="n"/>
+      <c r="H516" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I516" s="8" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J516" s="8" t="n">
+        <v>3215.3</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T15:00</t>
+        </is>
+      </c>
+      <c r="B517" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C517" s="9" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="D517" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E517" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F517" s="9" t="n"/>
+      <c r="G517" s="9" t="n"/>
+      <c r="H517" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I517" s="9" t="n">
+        <v>1017.8</v>
+      </c>
+      <c r="J517" s="9" t="n">
+        <v>2952.7</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T16:00</t>
+        </is>
+      </c>
+      <c r="B518" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C518" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="D518" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E518" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F518" s="8" t="n"/>
+      <c r="G518" s="8" t="n"/>
+      <c r="H518" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I518" s="8" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J518" s="8" t="n">
+        <v>2455.2</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T17:00</t>
+        </is>
+      </c>
+      <c r="B519" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C519" s="9" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D519" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E519" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F519" s="9" t="n"/>
+      <c r="G519" s="9" t="n"/>
+      <c r="H519" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I519" s="9" t="n">
+        <v>1017</v>
+      </c>
+      <c r="J519" s="9" t="n">
+        <v>1843.4</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T18:00</t>
+        </is>
+      </c>
+      <c r="B520" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C520" s="8" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="D520" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E520" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F520" s="8" t="n"/>
+      <c r="G520" s="8" t="n"/>
+      <c r="H520" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I520" s="8" t="n">
+        <v>1016.9</v>
+      </c>
+      <c r="J520" s="8" t="n">
+        <v>1152.1</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T19:00</t>
+        </is>
+      </c>
+      <c r="B521" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C521" s="9" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="D521" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="E521" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F521" s="9" t="n"/>
+      <c r="G521" s="9" t="n"/>
+      <c r="H521" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I521" s="9" t="n">
+        <v>1017.2</v>
+      </c>
+      <c r="J521" s="9" t="n">
+        <v>462.8</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T20:00</t>
+        </is>
+      </c>
+      <c r="B522" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C522" s="8" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D522" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E522" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F522" s="8" t="n"/>
+      <c r="G522" s="8" t="n"/>
+      <c r="H522" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I522" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J522" s="8" t="n">
+        <v>89.7</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T21:00</t>
+        </is>
+      </c>
+      <c r="B523" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C523" s="9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D523" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E523" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F523" s="9" t="n"/>
+      <c r="G523" s="9" t="n"/>
+      <c r="H523" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I523" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J523" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27T22:00</t>
+        </is>
+      </c>
+      <c r="B524" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C524" s="8" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D524" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E524" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F524" s="8" t="n"/>
+      <c r="G524" s="8" t="n"/>
+      <c r="H524" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I524" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J524" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-27T23:00</t>
+        </is>
+      </c>
+      <c r="B525" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C525" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D525" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E525" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F525" s="9" t="n"/>
+      <c r="G525" s="9" t="n"/>
+      <c r="H525" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I525" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J525" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-28 04:20 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J525"/>
+  <dimension ref="A1:J529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -17722,6 +17722,112 @@
         <v>0</v>
       </c>
     </row>
+    <row r="526">
+      <c r="A526" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T00:00</t>
+        </is>
+      </c>
+      <c r="B526" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C526" s="8" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D526" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E526" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F526" s="8" t="n"/>
+      <c r="G526" s="8" t="n"/>
+      <c r="H526" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I526" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J526" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28T01:00</t>
+        </is>
+      </c>
+      <c r="B527" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C527" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D527" s="10" t="n"/>
+      <c r="E527" s="10" t="n"/>
+      <c r="F527" s="10" t="n"/>
+      <c r="G527" s="10" t="n"/>
+      <c r="H527" s="10" t="n"/>
+      <c r="I527" s="10" t="n"/>
+      <c r="J527" s="10" t="n"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28T02:00</t>
+        </is>
+      </c>
+      <c r="B528" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C528" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D528" s="10" t="n"/>
+      <c r="E528" s="10" t="n"/>
+      <c r="F528" s="10" t="n"/>
+      <c r="G528" s="10" t="n"/>
+      <c r="H528" s="10" t="n"/>
+      <c r="I528" s="10" t="n"/>
+      <c r="J528" s="10" t="n"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28T03:00</t>
+        </is>
+      </c>
+      <c r="B529" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C529" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D529" s="10" t="n"/>
+      <c r="E529" s="10" t="n"/>
+      <c r="F529" s="10" t="n"/>
+      <c r="G529" s="10" t="n"/>
+      <c r="H529" s="10" t="n"/>
+      <c r="I529" s="10" t="n"/>
+      <c r="J529" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-29 00:06 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J529"/>
+  <dimension ref="A1:J549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -17828,6 +17828,686 @@
       <c r="I529" s="10" t="n"/>
       <c r="J529" s="10" t="n"/>
     </row>
+    <row r="530">
+      <c r="A530" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T04:00</t>
+        </is>
+      </c>
+      <c r="B530" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C530" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D530" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E530" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F530" s="8" t="n"/>
+      <c r="G530" s="8" t="n"/>
+      <c r="H530" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I530" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J530" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T05:00</t>
+        </is>
+      </c>
+      <c r="B531" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C531" s="9" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D531" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E531" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F531" s="9" t="n"/>
+      <c r="G531" s="9" t="n"/>
+      <c r="H531" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I531" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J531" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T06:00</t>
+        </is>
+      </c>
+      <c r="B532" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C532" s="8" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D532" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E532" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F532" s="8" t="n"/>
+      <c r="G532" s="8" t="n"/>
+      <c r="H532" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I532" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J532" s="8" t="n">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T07:00</t>
+        </is>
+      </c>
+      <c r="B533" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C533" s="9" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D533" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E533" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F533" s="9" t="n"/>
+      <c r="G533" s="9" t="n"/>
+      <c r="H533" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I533" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J533" s="9" t="n">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T08:00</t>
+        </is>
+      </c>
+      <c r="B534" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C534" s="8" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D534" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E534" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F534" s="8" t="n"/>
+      <c r="G534" s="8" t="n"/>
+      <c r="H534" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I534" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J534" s="8" t="n">
+        <v>1256.3</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T09:00</t>
+        </is>
+      </c>
+      <c r="B535" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C535" s="9" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="D535" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="E535" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F535" s="9" t="n"/>
+      <c r="G535" s="9" t="n"/>
+      <c r="H535" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I535" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J535" s="9" t="n">
+        <v>1922.5</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T10:00</t>
+        </is>
+      </c>
+      <c r="B536" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C536" s="8" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="D536" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E536" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F536" s="8" t="n"/>
+      <c r="G536" s="8" t="n"/>
+      <c r="H536" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I536" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J536" s="8" t="n">
+        <v>2553.8</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:00</t>
+        </is>
+      </c>
+      <c r="B537" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C537" s="9" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D537" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E537" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F537" s="9" t="n"/>
+      <c r="G537" s="9" t="n"/>
+      <c r="H537" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I537" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J537" s="9" t="n">
+        <v>2900.5</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T12:00</t>
+        </is>
+      </c>
+      <c r="B538" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C538" s="8" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="D538" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E538" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F538" s="8" t="n"/>
+      <c r="G538" s="8" t="n"/>
+      <c r="H538" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I538" s="8" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J538" s="8" t="n">
+        <v>3253.3</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T13:00</t>
+        </is>
+      </c>
+      <c r="B539" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C539" s="9" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="D539" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="E539" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F539" s="9" t="n"/>
+      <c r="G539" s="9" t="n"/>
+      <c r="H539" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I539" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J539" s="9" t="n">
+        <v>3386.6</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T14:00</t>
+        </is>
+      </c>
+      <c r="B540" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C540" s="8" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D540" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E540" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F540" s="8" t="n"/>
+      <c r="G540" s="8" t="n"/>
+      <c r="H540" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I540" s="8" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J540" s="8" t="n">
+        <v>3298.8</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T15:00</t>
+        </is>
+      </c>
+      <c r="B541" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C541" s="9" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="D541" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E541" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F541" s="9" t="n"/>
+      <c r="G541" s="9" t="n"/>
+      <c r="H541" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I541" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J541" s="9" t="n">
+        <v>3013.2</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T16:00</t>
+        </is>
+      </c>
+      <c r="B542" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C542" s="8" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="D542" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E542" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F542" s="8" t="n"/>
+      <c r="G542" s="8" t="n"/>
+      <c r="H542" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I542" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J542" s="8" t="n">
+        <v>2574.8</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T17:00</t>
+        </is>
+      </c>
+      <c r="B543" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C543" s="9" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="D543" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E543" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F543" s="9" t="n"/>
+      <c r="G543" s="9" t="n"/>
+      <c r="H543" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I543" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J543" s="9" t="n">
+        <v>1964.5</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T18:00</t>
+        </is>
+      </c>
+      <c r="B544" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C544" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D544" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="E544" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F544" s="8" t="n"/>
+      <c r="G544" s="8" t="n"/>
+      <c r="H544" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I544" s="8" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J544" s="8" t="n">
+        <v>1274.1</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T19:00</t>
+        </is>
+      </c>
+      <c r="B545" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C545" s="9" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="D545" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="E545" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F545" s="9" t="n"/>
+      <c r="G545" s="9" t="n"/>
+      <c r="H545" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I545" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J545" s="9" t="n">
+        <v>564.8</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T20:00</t>
+        </is>
+      </c>
+      <c r="B546" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C546" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D546" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E546" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F546" s="8" t="n"/>
+      <c r="G546" s="8" t="n"/>
+      <c r="H546" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I546" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J546" s="8" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T21:00</t>
+        </is>
+      </c>
+      <c r="B547" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C547" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D547" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E547" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F547" s="9" t="n"/>
+      <c r="G547" s="9" t="n"/>
+      <c r="H547" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I547" s="9" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J547" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-28T22:00</t>
+        </is>
+      </c>
+      <c r="B548" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C548" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D548" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E548" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F548" s="8" t="n"/>
+      <c r="G548" s="8" t="n"/>
+      <c r="H548" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I548" s="8" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J548" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-28T23:00</t>
+        </is>
+      </c>
+      <c r="B549" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C549" s="9" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D549" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E549" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F549" s="9" t="n"/>
+      <c r="G549" s="9" t="n"/>
+      <c r="H549" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I549" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J549" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-29 04:23 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J549"/>
+  <dimension ref="A1:J553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -18508,6 +18508,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="550">
+      <c r="A550" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T00:00</t>
+        </is>
+      </c>
+      <c r="B550" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C550" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D550" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E550" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F550" s="8" t="n"/>
+      <c r="G550" s="8" t="n"/>
+      <c r="H550" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I550" s="8" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J550" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T01:00</t>
+        </is>
+      </c>
+      <c r="B551" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C551" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D551" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E551" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F551" s="9" t="n"/>
+      <c r="G551" s="9" t="n"/>
+      <c r="H551" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I551" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J551" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T02:00</t>
+        </is>
+      </c>
+      <c r="B552" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C552" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D552" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E552" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F552" s="8" t="n"/>
+      <c r="G552" s="8" t="n"/>
+      <c r="H552" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I552" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J552" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T03:00</t>
+        </is>
+      </c>
+      <c r="B553" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C553" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D553" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E553" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F553" s="9" t="n"/>
+      <c r="G553" s="9" t="n"/>
+      <c r="H553" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I553" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J553" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-30 00:04 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J553"/>
+  <dimension ref="A1:J573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -18644,6 +18644,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="554">
+      <c r="A554" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T04:00</t>
+        </is>
+      </c>
+      <c r="B554" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C554" s="8" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D554" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E554" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F554" s="8" t="n"/>
+      <c r="G554" s="8" t="n"/>
+      <c r="H554" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I554" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J554" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T05:00</t>
+        </is>
+      </c>
+      <c r="B555" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C555" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D555" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E555" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F555" s="9" t="n"/>
+      <c r="G555" s="9" t="n"/>
+      <c r="H555" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I555" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J555" s="9" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:00</t>
+        </is>
+      </c>
+      <c r="B556" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C556" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D556" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E556" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F556" s="8" t="n"/>
+      <c r="G556" s="8" t="n"/>
+      <c r="H556" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I556" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J556" s="8" t="n">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T07:00</t>
+        </is>
+      </c>
+      <c r="B557" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C557" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D557" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E557" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F557" s="9" t="n"/>
+      <c r="G557" s="9" t="n"/>
+      <c r="H557" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I557" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J557" s="9" t="n">
+        <v>210.1</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T08:00</t>
+        </is>
+      </c>
+      <c r="B558" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C558" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D558" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E558" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F558" s="8" t="n"/>
+      <c r="G558" s="8" t="n"/>
+      <c r="H558" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I558" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J558" s="8" t="n">
+        <v>1099.6</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T09:00</t>
+        </is>
+      </c>
+      <c r="B559" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C559" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D559" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="E559" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F559" s="9" t="n"/>
+      <c r="G559" s="9" t="n"/>
+      <c r="H559" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I559" s="9" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J559" s="9" t="n">
+        <v>1935</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T10:00</t>
+        </is>
+      </c>
+      <c r="B560" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C560" s="8" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D560" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E560" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F560" s="8" t="n"/>
+      <c r="G560" s="8" t="n"/>
+      <c r="H560" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I560" s="8" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J560" s="8" t="n">
+        <v>2593</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T11:00</t>
+        </is>
+      </c>
+      <c r="B561" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C561" s="9" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D561" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="E561" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F561" s="9" t="n"/>
+      <c r="G561" s="9" t="n"/>
+      <c r="H561" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I561" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J561" s="9" t="n">
+        <v>2734.5</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T12:00</t>
+        </is>
+      </c>
+      <c r="B562" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C562" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D562" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E562" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F562" s="8" t="n"/>
+      <c r="G562" s="8" t="n"/>
+      <c r="H562" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I562" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J562" s="8" t="n">
+        <v>3193.4</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T13:00</t>
+        </is>
+      </c>
+      <c r="B563" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C563" s="9" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="D563" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E563" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F563" s="9" t="n"/>
+      <c r="G563" s="9" t="n"/>
+      <c r="H563" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I563" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J563" s="9" t="n">
+        <v>3134.1</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T14:00</t>
+        </is>
+      </c>
+      <c r="B564" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C564" s="8" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D564" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E564" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F564" s="8" t="n"/>
+      <c r="G564" s="8" t="n"/>
+      <c r="H564" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I564" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J564" s="8" t="n">
+        <v>3307.5</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T15:00</t>
+        </is>
+      </c>
+      <c r="B565" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C565" s="9" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D565" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E565" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F565" s="9" t="n"/>
+      <c r="G565" s="9" t="n"/>
+      <c r="H565" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I565" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J565" s="9" t="n">
+        <v>3037.3</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T16:00</t>
+        </is>
+      </c>
+      <c r="B566" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C566" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="D566" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="E566" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F566" s="8" t="n"/>
+      <c r="G566" s="8" t="n"/>
+      <c r="H566" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I566" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J566" s="8" t="n">
+        <v>2590.7</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T17:00</t>
+        </is>
+      </c>
+      <c r="B567" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C567" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="D567" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="E567" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F567" s="9" t="n"/>
+      <c r="G567" s="9" t="n"/>
+      <c r="H567" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I567" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J567" s="9" t="n">
+        <v>1947.3</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T18:00</t>
+        </is>
+      </c>
+      <c r="B568" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C568" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D568" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E568" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F568" s="8" t="n"/>
+      <c r="G568" s="8" t="n"/>
+      <c r="H568" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I568" s="8" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J568" s="8" t="n">
+        <v>1317.4</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T19:00</t>
+        </is>
+      </c>
+      <c r="B569" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C569" s="9" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D569" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E569" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F569" s="9" t="n"/>
+      <c r="G569" s="9" t="n"/>
+      <c r="H569" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I569" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J569" s="9" t="n">
+        <v>578.5</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T20:00</t>
+        </is>
+      </c>
+      <c r="B570" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C570" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D570" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E570" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F570" s="8" t="n"/>
+      <c r="G570" s="8" t="n"/>
+      <c r="H570" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I570" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J570" s="8" t="n">
+        <v>133.3</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T21:00</t>
+        </is>
+      </c>
+      <c r="B571" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C571" s="9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D571" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E571" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F571" s="9" t="n"/>
+      <c r="G571" s="9" t="n"/>
+      <c r="H571" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I571" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J571" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-29T22:00</t>
+        </is>
+      </c>
+      <c r="B572" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C572" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D572" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E572" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F572" s="8" t="n"/>
+      <c r="G572" s="8" t="n"/>
+      <c r="H572" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I572" s="8" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J572" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-29T23:00</t>
+        </is>
+      </c>
+      <c r="B573" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C573" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D573" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E573" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F573" s="9" t="n"/>
+      <c r="G573" s="9" t="n"/>
+      <c r="H573" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I573" s="9" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J573" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-30 04:08 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J573"/>
+  <dimension ref="A1:J577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -19324,6 +19324,112 @@
         <v>0</v>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T00:00</t>
+        </is>
+      </c>
+      <c r="B574" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C574" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D574" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E574" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F574" s="8" t="n"/>
+      <c r="G574" s="8" t="n"/>
+      <c r="H574" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I574" s="8" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J574" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-30T01:00</t>
+        </is>
+      </c>
+      <c r="B575" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C575" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D575" s="10" t="n"/>
+      <c r="E575" s="10" t="n"/>
+      <c r="F575" s="10" t="n"/>
+      <c r="G575" s="10" t="n"/>
+      <c r="H575" s="10" t="n"/>
+      <c r="I575" s="10" t="n"/>
+      <c r="J575" s="10" t="n"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-30T02:00</t>
+        </is>
+      </c>
+      <c r="B576" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C576" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D576" s="10" t="n"/>
+      <c r="E576" s="10" t="n"/>
+      <c r="F576" s="10" t="n"/>
+      <c r="G576" s="10" t="n"/>
+      <c r="H576" s="10" t="n"/>
+      <c r="I576" s="10" t="n"/>
+      <c r="J576" s="10" t="n"/>
+    </row>
+    <row r="577">
+      <c r="A577" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-30T03:00</t>
+        </is>
+      </c>
+      <c r="B577" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C577" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D577" s="10" t="n"/>
+      <c r="E577" s="10" t="n"/>
+      <c r="F577" s="10" t="n"/>
+      <c r="G577" s="10" t="n"/>
+      <c r="H577" s="10" t="n"/>
+      <c r="I577" s="10" t="n"/>
+      <c r="J577" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-30 23:57 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J577"/>
+  <dimension ref="A1:J597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -19430,6 +19430,682 @@
       <c r="I577" s="10" t="n"/>
       <c r="J577" s="10" t="n"/>
     </row>
+    <row r="578">
+      <c r="A578" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T04:00</t>
+        </is>
+      </c>
+      <c r="B578" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C578" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D578" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E578" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F578" s="8" t="n"/>
+      <c r="G578" s="8" t="n"/>
+      <c r="H578" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I578" s="8" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J578" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T05:00</t>
+        </is>
+      </c>
+      <c r="B579" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C579" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D579" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E579" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F579" s="9" t="n"/>
+      <c r="G579" s="9" t="n"/>
+      <c r="H579" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I579" s="9" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J579" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T06:00</t>
+        </is>
+      </c>
+      <c r="B580" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C580" s="8" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D580" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E580" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F580" s="8" t="n"/>
+      <c r="G580" s="8" t="n"/>
+      <c r="H580" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I580" s="8" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="J580" s="8" t="n">
+        <v>25.1</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T07:00</t>
+        </is>
+      </c>
+      <c r="B581" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C581" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D581" s="9" t="n">
+        <v>97</v>
+      </c>
+      <c r="E581" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F581" s="9" t="n"/>
+      <c r="G581" s="9" t="n"/>
+      <c r="H581" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I581" s="9" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J581" s="9" t="n">
+        <v>163.2</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T08:00</t>
+        </is>
+      </c>
+      <c r="B582" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C582" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="D582" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E582" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F582" s="8" t="n"/>
+      <c r="G582" s="8" t="n"/>
+      <c r="H582" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I582" s="8" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J582" s="8" t="n">
+        <v>373.6</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T09:00</t>
+        </is>
+      </c>
+      <c r="B583" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C583" s="9" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E583" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F583" s="9" t="n"/>
+      <c r="G583" s="9" t="n"/>
+      <c r="H583" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I583" s="9" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="J583" s="9" t="n">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T10:00</t>
+        </is>
+      </c>
+      <c r="B584" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C584" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D584" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E584" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F584" s="8" t="n"/>
+      <c r="G584" s="8" t="n"/>
+      <c r="H584" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I584" s="8" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J584" s="8" t="n">
+        <v>887.8</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T11:00</t>
+        </is>
+      </c>
+      <c r="B585" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C585" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D585" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E585" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F585" s="9" t="n"/>
+      <c r="G585" s="9" t="n"/>
+      <c r="H585" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I585" s="9" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J585" s="9" t="n">
+        <v>1021.7</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T12:00</t>
+        </is>
+      </c>
+      <c r="B586" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C586" s="8" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D586" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="E586" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F586" s="8" t="n"/>
+      <c r="G586" s="8" t="n"/>
+      <c r="H586" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I586" s="8" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J586" s="8" t="n">
+        <v>1099.1</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T13:00</t>
+        </is>
+      </c>
+      <c r="B587" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C587" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D587" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E587" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F587" s="9" t="n"/>
+      <c r="G587" s="9" t="n"/>
+      <c r="H587" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I587" s="9" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="J587" s="9" t="n"/>
+    </row>
+    <row r="588">
+      <c r="A588" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T14:00</t>
+        </is>
+      </c>
+      <c r="B588" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C588" s="8" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D588" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E588" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F588" s="8" t="n"/>
+      <c r="G588" s="8" t="n"/>
+      <c r="H588" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I588" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J588" s="8" t="n"/>
+    </row>
+    <row r="589">
+      <c r="A589" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T15:00</t>
+        </is>
+      </c>
+      <c r="B589" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C589" s="9" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D589" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="E589" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F589" s="9" t="n"/>
+      <c r="G589" s="9" t="n"/>
+      <c r="H589" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I589" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J589" s="9" t="n">
+        <v>3058.7</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T16:00</t>
+        </is>
+      </c>
+      <c r="B590" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C590" s="8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D590" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E590" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F590" s="8" t="n"/>
+      <c r="G590" s="8" t="n"/>
+      <c r="H590" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I590" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J590" s="8" t="n">
+        <v>2587.8</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T17:00</t>
+        </is>
+      </c>
+      <c r="B591" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C591" s="9" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="D591" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E591" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F591" s="9" t="n"/>
+      <c r="G591" s="9" t="n"/>
+      <c r="H591" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I591" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J591" s="9" t="n">
+        <v>1997.5</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T18:00</t>
+        </is>
+      </c>
+      <c r="B592" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C592" s="8" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D592" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E592" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F592" s="8" t="n"/>
+      <c r="G592" s="8" t="n"/>
+      <c r="H592" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I592" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J592" s="8" t="n">
+        <v>1319.6</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T19:00</t>
+        </is>
+      </c>
+      <c r="B593" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C593" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D593" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E593" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F593" s="9" t="n"/>
+      <c r="G593" s="9" t="n"/>
+      <c r="H593" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I593" s="9" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J593" s="9" t="n">
+        <v>607.2</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T20:00</t>
+        </is>
+      </c>
+      <c r="B594" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C594" s="8" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="D594" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E594" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F594" s="8" t="n"/>
+      <c r="G594" s="8" t="n"/>
+      <c r="H594" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I594" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J594" s="8" t="n">
+        <v>125.3</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T21:00</t>
+        </is>
+      </c>
+      <c r="B595" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C595" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D595" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E595" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F595" s="9" t="n"/>
+      <c r="G595" s="9" t="n"/>
+      <c r="H595" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I595" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J595" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-30T22:00</t>
+        </is>
+      </c>
+      <c r="B596" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C596" s="8" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D596" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E596" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F596" s="8" t="n"/>
+      <c r="G596" s="8" t="n"/>
+      <c r="H596" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I596" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J596" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-30T23:00</t>
+        </is>
+      </c>
+      <c r="B597" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C597" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D597" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E597" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F597" s="9" t="n"/>
+      <c r="G597" s="9" t="n"/>
+      <c r="H597" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I597" s="9" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J597" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-05-31 04:43 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J597"/>
+  <dimension ref="A1:J602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -20106,6 +20106,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="598">
+      <c r="A598" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T00:00</t>
+        </is>
+      </c>
+      <c r="B598" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C598" s="8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D598" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E598" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F598" s="8" t="n"/>
+      <c r="G598" s="8" t="n"/>
+      <c r="H598" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I598" s="8" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J598" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T01:00</t>
+        </is>
+      </c>
+      <c r="B599" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C599" s="9" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D599" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E599" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F599" s="9" t="n"/>
+      <c r="G599" s="9" t="n"/>
+      <c r="H599" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I599" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J599" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T02:00</t>
+        </is>
+      </c>
+      <c r="B600" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C600" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D600" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E600" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F600" s="8" t="n"/>
+      <c r="G600" s="8" t="n"/>
+      <c r="H600" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I600" s="8" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J600" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T03:00</t>
+        </is>
+      </c>
+      <c r="B601" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C601" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D601" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="E601" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F601" s="9" t="n"/>
+      <c r="G601" s="9" t="n"/>
+      <c r="H601" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I601" s="9" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J601" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T04:00</t>
+        </is>
+      </c>
+      <c r="B602" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C602" s="8" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D602" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="E602" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F602" s="8" t="n"/>
+      <c r="G602" s="8" t="n"/>
+      <c r="H602" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I602" s="8" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J602" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-01 00:02 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J602"/>
+  <dimension ref="A1:J621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -20274,6 +20274,572 @@
       </c>
       <c r="J602" s="8" t="n"/>
     </row>
+    <row r="603">
+      <c r="A603" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T13:00</t>
+        </is>
+      </c>
+      <c r="B603" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C603" s="9" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="D603" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E603" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F603" s="9" t="n"/>
+      <c r="G603" s="9" t="n"/>
+      <c r="H603" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I603" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J603" s="9" t="n">
+        <v>3442.4</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T14:00</t>
+        </is>
+      </c>
+      <c r="B604" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C604" s="8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D604" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E604" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F604" s="8" t="n"/>
+      <c r="G604" s="8" t="n"/>
+      <c r="H604" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I604" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J604" s="8" t="n">
+        <v>3340.1</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T15:00</t>
+        </is>
+      </c>
+      <c r="B605" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C605" s="9" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D605" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E605" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F605" s="9" t="n"/>
+      <c r="G605" s="9" t="n"/>
+      <c r="H605" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I605" s="9" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J605" s="9" t="n">
+        <v>2986.7</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T16:00</t>
+        </is>
+      </c>
+      <c r="B606" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C606" s="8" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="D606" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E606" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F606" s="8" t="n"/>
+      <c r="G606" s="8" t="n"/>
+      <c r="H606" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I606" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J606" s="8" t="n">
+        <v>2430.2</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T17:00</t>
+        </is>
+      </c>
+      <c r="B607" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C607" s="9" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="D607" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="E607" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F607" s="9" t="n"/>
+      <c r="G607" s="9" t="n"/>
+      <c r="H607" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I607" s="9" t="n">
+        <v>1018.3</v>
+      </c>
+      <c r="J607" s="9" t="n">
+        <v>2019.2</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T18:00</t>
+        </is>
+      </c>
+      <c r="B608" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C608" s="8" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="D608" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E608" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F608" s="8" t="n"/>
+      <c r="G608" s="8" t="n"/>
+      <c r="H608" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I608" s="8" t="n">
+        <v>1018.3</v>
+      </c>
+      <c r="J608" s="8" t="n">
+        <v>1292.4</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T19:00</t>
+        </is>
+      </c>
+      <c r="B609" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C609" s="9" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D609" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E609" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F609" s="9" t="n"/>
+      <c r="G609" s="9" t="n"/>
+      <c r="H609" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I609" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J609" s="9" t="n">
+        <v>669.1</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T20:00</t>
+        </is>
+      </c>
+      <c r="B610" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C610" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="D610" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E610" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F610" s="8" t="n"/>
+      <c r="G610" s="8" t="n"/>
+      <c r="H610" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I610" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J610" s="8" t="n">
+        <v>141.9</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T21:00</t>
+        </is>
+      </c>
+      <c r="B611" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C611" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D611" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E611" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F611" s="9" t="n"/>
+      <c r="G611" s="9" t="n"/>
+      <c r="H611" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I611" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J611" s="9" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-31T22:00</t>
+        </is>
+      </c>
+      <c r="B612" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C612" s="8" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D612" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="E612" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F612" s="8" t="n"/>
+      <c r="G612" s="8" t="n"/>
+      <c r="H612" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I612" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J612" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-31T23:00</t>
+        </is>
+      </c>
+      <c r="B613" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C613" s="9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D613" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E613" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F613" s="9" t="n"/>
+      <c r="G613" s="9" t="n"/>
+      <c r="H613" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I613" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J613" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T05:00</t>
+        </is>
+      </c>
+      <c r="B614" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C614" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D614" s="10" t="n"/>
+      <c r="E614" s="10" t="n"/>
+      <c r="F614" s="10" t="n"/>
+      <c r="G614" s="10" t="n"/>
+      <c r="H614" s="10" t="n"/>
+      <c r="I614" s="10" t="n"/>
+      <c r="J614" s="10" t="n"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T06:00</t>
+        </is>
+      </c>
+      <c r="B615" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C615" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D615" s="10" t="n"/>
+      <c r="E615" s="10" t="n"/>
+      <c r="F615" s="10" t="n"/>
+      <c r="G615" s="10" t="n"/>
+      <c r="H615" s="10" t="n"/>
+      <c r="I615" s="10" t="n"/>
+      <c r="J615" s="10" t="n"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T07:00</t>
+        </is>
+      </c>
+      <c r="B616" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C616" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D616" s="10" t="n"/>
+      <c r="E616" s="10" t="n"/>
+      <c r="F616" s="10" t="n"/>
+      <c r="G616" s="10" t="n"/>
+      <c r="H616" s="10" t="n"/>
+      <c r="I616" s="10" t="n"/>
+      <c r="J616" s="10" t="n"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T08:00</t>
+        </is>
+      </c>
+      <c r="B617" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C617" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D617" s="10" t="n"/>
+      <c r="E617" s="10" t="n"/>
+      <c r="F617" s="10" t="n"/>
+      <c r="G617" s="10" t="n"/>
+      <c r="H617" s="10" t="n"/>
+      <c r="I617" s="10" t="n"/>
+      <c r="J617" s="10" t="n"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T09:00</t>
+        </is>
+      </c>
+      <c r="B618" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C618" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D618" s="10" t="n"/>
+      <c r="E618" s="10" t="n"/>
+      <c r="F618" s="10" t="n"/>
+      <c r="G618" s="10" t="n"/>
+      <c r="H618" s="10" t="n"/>
+      <c r="I618" s="10" t="n"/>
+      <c r="J618" s="10" t="n"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T10:00</t>
+        </is>
+      </c>
+      <c r="B619" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C619" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D619" s="10" t="n"/>
+      <c r="E619" s="10" t="n"/>
+      <c r="F619" s="10" t="n"/>
+      <c r="G619" s="10" t="n"/>
+      <c r="H619" s="10" t="n"/>
+      <c r="I619" s="10" t="n"/>
+      <c r="J619" s="10" t="n"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T11:00</t>
+        </is>
+      </c>
+      <c r="B620" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C620" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D620" s="10" t="n"/>
+      <c r="E620" s="10" t="n"/>
+      <c r="F620" s="10" t="n"/>
+      <c r="G620" s="10" t="n"/>
+      <c r="H620" s="10" t="n"/>
+      <c r="I620" s="10" t="n"/>
+      <c r="J620" s="10" t="n"/>
+    </row>
+    <row r="621">
+      <c r="A621" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-31T12:00</t>
+        </is>
+      </c>
+      <c r="B621" s="10" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C621" s="10" t="inlineStr">
+        <is>
+          <t>NO DATA</t>
+        </is>
+      </c>
+      <c r="D621" s="10" t="n"/>
+      <c r="E621" s="10" t="n"/>
+      <c r="F621" s="10" t="n"/>
+      <c r="G621" s="10" t="n"/>
+      <c r="H621" s="10" t="n"/>
+      <c r="I621" s="10" t="n"/>
+      <c r="J621" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-01 05:05 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J621"/>
+  <dimension ref="A1:J626"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -20840,6 +20840,176 @@
       <c r="I621" s="10" t="n"/>
       <c r="J621" s="10" t="n"/>
     </row>
+    <row r="622">
+      <c r="A622" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T00:00</t>
+        </is>
+      </c>
+      <c r="B622" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C622" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D622" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E622" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F622" s="8" t="n"/>
+      <c r="G622" s="8" t="n"/>
+      <c r="H622" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I622" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J622" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T01:00</t>
+        </is>
+      </c>
+      <c r="B623" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C623" s="9" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D623" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E623" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F623" s="9" t="n"/>
+      <c r="G623" s="9" t="n"/>
+      <c r="H623" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I623" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J623" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T02:00</t>
+        </is>
+      </c>
+      <c r="B624" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C624" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D624" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E624" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F624" s="8" t="n"/>
+      <c r="G624" s="8" t="n"/>
+      <c r="H624" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I624" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J624" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T03:00</t>
+        </is>
+      </c>
+      <c r="B625" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C625" s="9" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D625" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E625" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F625" s="9" t="n"/>
+      <c r="G625" s="9" t="n"/>
+      <c r="H625" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I625" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J625" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T04:00</t>
+        </is>
+      </c>
+      <c r="B626" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C626" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D626" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E626" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F626" s="8" t="n"/>
+      <c r="G626" s="8" t="n"/>
+      <c r="H626" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I626" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J626" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-02 00:09 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J626"/>
+  <dimension ref="A1:J645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -21010,6 +21010,652 @@
         <v>0</v>
       </c>
     </row>
+    <row r="627">
+      <c r="A627" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T05:00</t>
+        </is>
+      </c>
+      <c r="B627" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C627" s="9" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D627" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E627" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F627" s="9" t="n"/>
+      <c r="G627" s="9" t="n"/>
+      <c r="H627" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I627" s="9" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J627" s="9" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T06:00</t>
+        </is>
+      </c>
+      <c r="B628" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C628" s="8" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D628" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="E628" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F628" s="8" t="n"/>
+      <c r="G628" s="8" t="n"/>
+      <c r="H628" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I628" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J628" s="8" t="n">
+        <v>86.09999999999999</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T07:00</t>
+        </is>
+      </c>
+      <c r="B629" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C629" s="9" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D629" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E629" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F629" s="9" t="n"/>
+      <c r="G629" s="9" t="n"/>
+      <c r="H629" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I629" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J629" s="9" t="n">
+        <v>601.5</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T08:00</t>
+        </is>
+      </c>
+      <c r="B630" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C630" s="8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D630" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E630" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F630" s="8" t="n"/>
+      <c r="G630" s="8" t="n"/>
+      <c r="H630" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I630" s="8" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J630" s="8" t="n">
+        <v>1305.3</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T09:00</t>
+        </is>
+      </c>
+      <c r="B631" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C631" s="9" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D631" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E631" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F631" s="9" t="n"/>
+      <c r="G631" s="9" t="n"/>
+      <c r="H631" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I631" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J631" s="9" t="n">
+        <v>1894.2</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T10:00</t>
+        </is>
+      </c>
+      <c r="B632" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C632" s="8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D632" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E632" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F632" s="8" t="n"/>
+      <c r="G632" s="8" t="n"/>
+      <c r="H632" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I632" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J632" s="8" t="n">
+        <v>2509.7</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T11:00</t>
+        </is>
+      </c>
+      <c r="B633" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C633" s="9" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D633" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E633" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F633" s="9" t="n"/>
+      <c r="G633" s="9" t="n"/>
+      <c r="H633" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I633" s="9" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J633" s="9" t="n">
+        <v>2945</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T12:00</t>
+        </is>
+      </c>
+      <c r="B634" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C634" s="8" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D634" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E634" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F634" s="8" t="n"/>
+      <c r="G634" s="8" t="n"/>
+      <c r="H634" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I634" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J634" s="8" t="n">
+        <v>3333.2</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T13:00</t>
+        </is>
+      </c>
+      <c r="B635" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C635" s="9" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D635" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E635" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F635" s="9" t="n"/>
+      <c r="G635" s="9" t="n"/>
+      <c r="H635" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I635" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J635" s="9" t="n">
+        <v>3439.9</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T14:00</t>
+        </is>
+      </c>
+      <c r="B636" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C636" s="8" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="D636" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E636" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F636" s="8" t="n"/>
+      <c r="G636" s="8" t="n"/>
+      <c r="H636" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I636" s="8" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J636" s="8" t="n">
+        <v>3364.4</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T15:00</t>
+        </is>
+      </c>
+      <c r="B637" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C637" s="9" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="D637" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E637" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F637" s="9" t="n"/>
+      <c r="G637" s="9" t="n"/>
+      <c r="H637" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I637" s="9" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J637" s="9" t="n">
+        <v>3096</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T16:00</t>
+        </is>
+      </c>
+      <c r="B638" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C638" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="D638" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E638" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F638" s="8" t="n"/>
+      <c r="G638" s="8" t="n"/>
+      <c r="H638" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I638" s="8" t="n">
+        <v>1017.7</v>
+      </c>
+      <c r="J638" s="8" t="n">
+        <v>2649.2</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T17:00</t>
+        </is>
+      </c>
+      <c r="B639" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C639" s="9" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="D639" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E639" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F639" s="9" t="n"/>
+      <c r="G639" s="9" t="n"/>
+      <c r="H639" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I639" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J639" s="9" t="n">
+        <v>2061.6</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T18:00</t>
+        </is>
+      </c>
+      <c r="B640" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C640" s="8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D640" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E640" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F640" s="8" t="n"/>
+      <c r="G640" s="8" t="n"/>
+      <c r="H640" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I640" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J640" s="8" t="n">
+        <v>1360.1</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T19:00</t>
+        </is>
+      </c>
+      <c r="B641" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C641" s="9" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="D641" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="E641" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F641" s="9" t="n"/>
+      <c r="G641" s="9" t="n"/>
+      <c r="H641" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I641" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J641" s="9" t="n">
+        <v>683.8</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T20:00</t>
+        </is>
+      </c>
+      <c r="B642" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C642" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D642" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E642" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F642" s="8" t="n"/>
+      <c r="G642" s="8" t="n"/>
+      <c r="H642" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I642" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J642" s="8" t="n">
+        <v>119.2</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T21:00</t>
+        </is>
+      </c>
+      <c r="B643" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C643" s="9" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D643" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="E643" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F643" s="9" t="n"/>
+      <c r="G643" s="9" t="n"/>
+      <c r="H643" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I643" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J643" s="9" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-01T22:00</t>
+        </is>
+      </c>
+      <c r="B644" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C644" s="8" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="D644" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="E644" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F644" s="8" t="n"/>
+      <c r="G644" s="8" t="n"/>
+      <c r="H644" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I644" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J644" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-01T23:00</t>
+        </is>
+      </c>
+      <c r="B645" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C645" s="9" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="D645" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E645" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F645" s="9" t="n"/>
+      <c r="G645" s="9" t="n"/>
+      <c r="H645" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I645" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J645" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-02 04:51 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J645"/>
+  <dimension ref="A1:J650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -21656,6 +21656,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="646">
+      <c r="A646" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T00:00</t>
+        </is>
+      </c>
+      <c r="B646" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C646" s="8" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="D646" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E646" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F646" s="8" t="n"/>
+      <c r="G646" s="8" t="n"/>
+      <c r="H646" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I646" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J646" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T01:00</t>
+        </is>
+      </c>
+      <c r="B647" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C647" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D647" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E647" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F647" s="9" t="n"/>
+      <c r="G647" s="9" t="n"/>
+      <c r="H647" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I647" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J647" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T02:00</t>
+        </is>
+      </c>
+      <c r="B648" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C648" s="8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D648" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E648" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F648" s="8" t="n"/>
+      <c r="G648" s="8" t="n"/>
+      <c r="H648" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I648" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J648" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T03:00</t>
+        </is>
+      </c>
+      <c r="B649" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C649" s="9" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D649" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E649" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F649" s="9" t="n"/>
+      <c r="G649" s="9" t="n"/>
+      <c r="H649" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I649" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J649" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T04:00</t>
+        </is>
+      </c>
+      <c r="B650" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C650" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D650" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E650" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F650" s="8" t="n"/>
+      <c r="G650" s="8" t="n"/>
+      <c r="H650" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I650" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J650" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-03 00:24 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J650"/>
+  <dimension ref="A1:J669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -21826,6 +21826,644 @@
         <v>0</v>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T05:00</t>
+        </is>
+      </c>
+      <c r="B651" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C651" s="9" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D651" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E651" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F651" s="9" t="n"/>
+      <c r="G651" s="9" t="n"/>
+      <c r="H651" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I651" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J651" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T06:00</t>
+        </is>
+      </c>
+      <c r="B652" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C652" s="8" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="D652" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E652" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F652" s="8" t="n"/>
+      <c r="G652" s="8" t="n"/>
+      <c r="H652" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I652" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J652" s="8" t="n">
+        <v>47.9</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T07:00</t>
+        </is>
+      </c>
+      <c r="B653" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C653" s="9" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D653" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E653" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F653" s="9" t="n"/>
+      <c r="G653" s="9" t="n"/>
+      <c r="H653" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I653" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J653" s="9" t="n">
+        <v>377.5</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T08:00</t>
+        </is>
+      </c>
+      <c r="B654" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C654" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D654" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="E654" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F654" s="8" t="n"/>
+      <c r="G654" s="8" t="n"/>
+      <c r="H654" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I654" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J654" s="8" t="n">
+        <v>1010.7</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T09:00</t>
+        </is>
+      </c>
+      <c r="B655" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C655" s="9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D655" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E655" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F655" s="9" t="n"/>
+      <c r="G655" s="9" t="n"/>
+      <c r="H655" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I655" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J655" s="9" t="n">
+        <v>1666.4</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T10:00</t>
+        </is>
+      </c>
+      <c r="B656" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C656" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D656" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E656" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F656" s="8" t="n"/>
+      <c r="G656" s="8" t="n"/>
+      <c r="H656" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I656" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J656" s="8" t="n">
+        <v>1880.7</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T11:00</t>
+        </is>
+      </c>
+      <c r="B657" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C657" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D657" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E657" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F657" s="9" t="n"/>
+      <c r="G657" s="9" t="n"/>
+      <c r="H657" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I657" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J657" s="9" t="n">
+        <v>1914.4</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T12:00</t>
+        </is>
+      </c>
+      <c r="B658" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C658" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D658" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E658" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F658" s="8" t="n"/>
+      <c r="G658" s="8" t="n"/>
+      <c r="H658" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I658" s="8" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J658" s="8" t="n"/>
+    </row>
+    <row r="659">
+      <c r="A659" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T13:00</t>
+        </is>
+      </c>
+      <c r="B659" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C659" s="9" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="D659" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E659" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F659" s="9" t="n"/>
+      <c r="G659" s="9" t="n"/>
+      <c r="H659" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I659" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J659" s="9" t="n"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T14:00</t>
+        </is>
+      </c>
+      <c r="B660" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C660" s="8" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="D660" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="E660" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F660" s="8" t="n"/>
+      <c r="G660" s="8" t="n"/>
+      <c r="H660" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I660" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J660" s="8" t="n"/>
+    </row>
+    <row r="661">
+      <c r="A661" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T15:00</t>
+        </is>
+      </c>
+      <c r="B661" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C661" s="9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D661" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E661" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F661" s="9" t="n"/>
+      <c r="G661" s="9" t="n"/>
+      <c r="H661" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I661" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J661" s="9" t="n"/>
+    </row>
+    <row r="662">
+      <c r="A662" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T16:00</t>
+        </is>
+      </c>
+      <c r="B662" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C662" s="8" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D662" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E662" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F662" s="8" t="n"/>
+      <c r="G662" s="8" t="n"/>
+      <c r="H662" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I662" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J662" s="8" t="n">
+        <v>2610.1</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T17:00</t>
+        </is>
+      </c>
+      <c r="B663" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C663" s="9" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D663" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E663" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F663" s="9" t="n"/>
+      <c r="G663" s="9" t="n"/>
+      <c r="H663" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I663" s="9" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J663" s="9" t="n">
+        <v>2088.6</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T18:00</t>
+        </is>
+      </c>
+      <c r="B664" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C664" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D664" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="E664" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F664" s="8" t="n"/>
+      <c r="G664" s="8" t="n"/>
+      <c r="H664" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I664" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J664" s="8" t="n">
+        <v>1309.4</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T19:00</t>
+        </is>
+      </c>
+      <c r="B665" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C665" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D665" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E665" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F665" s="9" t="n"/>
+      <c r="G665" s="9" t="n"/>
+      <c r="H665" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I665" s="9" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J665" s="9" t="n">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T20:00</t>
+        </is>
+      </c>
+      <c r="B666" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C666" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D666" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E666" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F666" s="8" t="n"/>
+      <c r="G666" s="8" t="n"/>
+      <c r="H666" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I666" s="8" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J666" s="8" t="n">
+        <v>159.5</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T21:00</t>
+        </is>
+      </c>
+      <c r="B667" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C667" s="9" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D667" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E667" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F667" s="9" t="n"/>
+      <c r="G667" s="9" t="n"/>
+      <c r="H667" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I667" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J667" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-02T22:00</t>
+        </is>
+      </c>
+      <c r="B668" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C668" s="8" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D668" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="E668" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F668" s="8" t="n"/>
+      <c r="G668" s="8" t="n"/>
+      <c r="H668" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I668" s="8" t="n">
+        <v>1023.5</v>
+      </c>
+      <c r="J668" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-02T23:00</t>
+        </is>
+      </c>
+      <c r="B669" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C669" s="9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D669" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E669" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F669" s="9" t="n"/>
+      <c r="G669" s="9" t="n"/>
+      <c r="H669" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I669" s="9" t="n">
+        <v>1023.7</v>
+      </c>
+      <c r="J669" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-03 05:02 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J669"/>
+  <dimension ref="A1:J674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -22464,6 +22464,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="670">
+      <c r="A670" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T00:00</t>
+        </is>
+      </c>
+      <c r="B670" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C670" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D670" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E670" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F670" s="8" t="n"/>
+      <c r="G670" s="8" t="n"/>
+      <c r="H670" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I670" s="8" t="n">
+        <v>1023.9</v>
+      </c>
+      <c r="J670" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T01:00</t>
+        </is>
+      </c>
+      <c r="B671" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C671" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D671" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E671" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F671" s="9" t="n"/>
+      <c r="G671" s="9" t="n"/>
+      <c r="H671" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I671" s="9" t="n">
+        <v>1024.1</v>
+      </c>
+      <c r="J671" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T02:00</t>
+        </is>
+      </c>
+      <c r="B672" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C672" s="8" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D672" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E672" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F672" s="8" t="n"/>
+      <c r="G672" s="8" t="n"/>
+      <c r="H672" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I672" s="8" t="n">
+        <v>1023.7</v>
+      </c>
+      <c r="J672" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T03:00</t>
+        </is>
+      </c>
+      <c r="B673" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C673" s="9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D673" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E673" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F673" s="9" t="n"/>
+      <c r="G673" s="9" t="n"/>
+      <c r="H673" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I673" s="9" t="n">
+        <v>1023.5</v>
+      </c>
+      <c r="J673" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T04:00</t>
+        </is>
+      </c>
+      <c r="B674" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C674" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D674" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E674" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F674" s="8" t="n"/>
+      <c r="G674" s="8" t="n"/>
+      <c r="H674" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I674" s="8" t="n">
+        <v>1023.7</v>
+      </c>
+      <c r="J674" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-04 00:27 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J674"/>
+  <dimension ref="A1:J693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -22634,6 +22634,642 @@
         <v>0</v>
       </c>
     </row>
+    <row r="675">
+      <c r="A675" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T05:00</t>
+        </is>
+      </c>
+      <c r="B675" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C675" s="9" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D675" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E675" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F675" s="9" t="n"/>
+      <c r="G675" s="9" t="n"/>
+      <c r="H675" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I675" s="9" t="n">
+        <v>1023.6</v>
+      </c>
+      <c r="J675" s="9" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T06:00</t>
+        </is>
+      </c>
+      <c r="B676" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C676" s="8" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D676" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E676" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F676" s="8" t="n"/>
+      <c r="G676" s="8" t="n"/>
+      <c r="H676" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I676" s="8" t="n">
+        <v>1023.6</v>
+      </c>
+      <c r="J676" s="8" t="n">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T07:00</t>
+        </is>
+      </c>
+      <c r="B677" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C677" s="9" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="D677" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E677" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F677" s="9" t="n"/>
+      <c r="G677" s="9" t="n"/>
+      <c r="H677" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I677" s="9" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J677" s="9" t="n">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:00</t>
+        </is>
+      </c>
+      <c r="B678" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C678" s="8" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="D678" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E678" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F678" s="8" t="n"/>
+      <c r="G678" s="8" t="n"/>
+      <c r="H678" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I678" s="8" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J678" s="8" t="n">
+        <v>1315.4</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T09:00</t>
+        </is>
+      </c>
+      <c r="B679" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C679" s="9" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D679" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E679" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F679" s="9" t="n"/>
+      <c r="G679" s="9" t="n"/>
+      <c r="H679" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I679" s="9" t="n">
+        <v>1022.8</v>
+      </c>
+      <c r="J679" s="9" t="n">
+        <v>1860.2</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T10:00</t>
+        </is>
+      </c>
+      <c r="B680" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C680" s="8" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D680" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="E680" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F680" s="8" t="n"/>
+      <c r="G680" s="8" t="n"/>
+      <c r="H680" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I680" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J680" s="8" t="n">
+        <v>2591.2</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T11:00</t>
+        </is>
+      </c>
+      <c r="B681" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C681" s="9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D681" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E681" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F681" s="9" t="n"/>
+      <c r="G681" s="9" t="n"/>
+      <c r="H681" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I681" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J681" s="9" t="n"/>
+    </row>
+    <row r="682">
+      <c r="A682" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T12:00</t>
+        </is>
+      </c>
+      <c r="B682" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C682" s="8" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D682" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="E682" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F682" s="8" t="n"/>
+      <c r="G682" s="8" t="n"/>
+      <c r="H682" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I682" s="8" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J682" s="8" t="n"/>
+    </row>
+    <row r="683">
+      <c r="A683" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T13:00</t>
+        </is>
+      </c>
+      <c r="B683" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C683" s="9" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D683" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E683" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F683" s="9" t="n"/>
+      <c r="G683" s="9" t="n"/>
+      <c r="H683" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I683" s="9" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J683" s="9" t="n"/>
+    </row>
+    <row r="684">
+      <c r="A684" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T14:00</t>
+        </is>
+      </c>
+      <c r="B684" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C684" s="8" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D684" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E684" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F684" s="8" t="n"/>
+      <c r="G684" s="8" t="n"/>
+      <c r="H684" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I684" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J684" s="8" t="n"/>
+    </row>
+    <row r="685">
+      <c r="A685" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T15:00</t>
+        </is>
+      </c>
+      <c r="B685" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C685" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D685" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E685" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F685" s="9" t="n"/>
+      <c r="G685" s="9" t="n"/>
+      <c r="H685" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I685" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J685" s="9" t="n"/>
+    </row>
+    <row r="686">
+      <c r="A686" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T16:00</t>
+        </is>
+      </c>
+      <c r="B686" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C686" s="8" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D686" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E686" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F686" s="8" t="n"/>
+      <c r="G686" s="8" t="n"/>
+      <c r="H686" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I686" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J686" s="8" t="n">
+        <v>763.9</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T17:00</t>
+        </is>
+      </c>
+      <c r="B687" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C687" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D687" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="E687" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F687" s="9" t="n"/>
+      <c r="G687" s="9" t="n"/>
+      <c r="H687" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I687" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J687" s="9" t="n">
+        <v>519.1</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T18:00</t>
+        </is>
+      </c>
+      <c r="B688" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C688" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D688" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E688" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F688" s="8" t="n"/>
+      <c r="G688" s="8" t="n"/>
+      <c r="H688" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I688" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J688" s="8" t="n">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T19:00</t>
+        </is>
+      </c>
+      <c r="B689" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C689" s="9" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="D689" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="E689" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F689" s="9" t="n"/>
+      <c r="G689" s="9" t="n"/>
+      <c r="H689" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I689" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J689" s="9" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T20:00</t>
+        </is>
+      </c>
+      <c r="B690" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C690" s="8" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D690" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E690" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F690" s="8" t="n"/>
+      <c r="G690" s="8" t="n"/>
+      <c r="H690" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I690" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J690" s="8" t="n">
+        <v>47.4</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T21:00</t>
+        </is>
+      </c>
+      <c r="B691" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C691" s="9" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="D691" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E691" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F691" s="9" t="n"/>
+      <c r="G691" s="9" t="n"/>
+      <c r="H691" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I691" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J691" s="9" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03T22:00</t>
+        </is>
+      </c>
+      <c r="B692" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C692" s="8" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="D692" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E692" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F692" s="8" t="n"/>
+      <c r="G692" s="8" t="n"/>
+      <c r="H692" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I692" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J692" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-03T23:00</t>
+        </is>
+      </c>
+      <c r="B693" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C693" s="9" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D693" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E693" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F693" s="9" t="n"/>
+      <c r="G693" s="9" t="n"/>
+      <c r="H693" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I693" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J693" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-04 04:54 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J693"/>
+  <dimension ref="A1:J698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -23270,6 +23270,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="694">
+      <c r="A694" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T00:00</t>
+        </is>
+      </c>
+      <c r="B694" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C694" s="8" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D694" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E694" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F694" s="8" t="n"/>
+      <c r="G694" s="8" t="n"/>
+      <c r="H694" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I694" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J694" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T01:00</t>
+        </is>
+      </c>
+      <c r="B695" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C695" s="9" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D695" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E695" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F695" s="9" t="n"/>
+      <c r="G695" s="9" t="n"/>
+      <c r="H695" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I695" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J695" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T02:00</t>
+        </is>
+      </c>
+      <c r="B696" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C696" s="8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D696" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E696" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F696" s="8" t="n"/>
+      <c r="G696" s="8" t="n"/>
+      <c r="H696" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I696" s="8" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J696" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T03:00</t>
+        </is>
+      </c>
+      <c r="B697" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C697" s="9" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="D697" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E697" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F697" s="9" t="n"/>
+      <c r="G697" s="9" t="n"/>
+      <c r="H697" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I697" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J697" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T04:00</t>
+        </is>
+      </c>
+      <c r="B698" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C698" s="8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D698" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E698" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F698" s="8" t="n"/>
+      <c r="G698" s="8" t="n"/>
+      <c r="H698" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I698" s="8" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J698" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-05 00:01 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J698"/>
+  <dimension ref="A1:J717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -23440,6 +23440,648 @@
         <v>0</v>
       </c>
     </row>
+    <row r="699">
+      <c r="A699" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T05:00</t>
+        </is>
+      </c>
+      <c r="B699" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C699" s="9" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D699" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E699" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F699" s="9" t="n"/>
+      <c r="G699" s="9" t="n"/>
+      <c r="H699" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I699" s="9" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J699" s="9" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T06:00</t>
+        </is>
+      </c>
+      <c r="B700" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C700" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D700" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E700" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F700" s="8" t="n"/>
+      <c r="G700" s="8" t="n"/>
+      <c r="H700" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I700" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J700" s="8" t="n">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T07:00</t>
+        </is>
+      </c>
+      <c r="B701" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C701" s="9" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D701" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E701" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F701" s="9" t="n"/>
+      <c r="G701" s="9" t="n"/>
+      <c r="H701" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I701" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J701" s="9" t="n">
+        <v>416.5</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T08:00</t>
+        </is>
+      </c>
+      <c r="B702" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C702" s="8" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D702" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="E702" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F702" s="8" t="n"/>
+      <c r="G702" s="8" t="n"/>
+      <c r="H702" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I702" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J702" s="8" t="n">
+        <v>852.2</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T09:00</t>
+        </is>
+      </c>
+      <c r="B703" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C703" s="9" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="D703" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E703" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F703" s="9" t="n"/>
+      <c r="G703" s="9" t="n"/>
+      <c r="H703" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I703" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J703" s="9" t="n">
+        <v>1256.4</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T10:00</t>
+        </is>
+      </c>
+      <c r="B704" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C704" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D704" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E704" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F704" s="8" t="n"/>
+      <c r="G704" s="8" t="n"/>
+      <c r="H704" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I704" s="8" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J704" s="8" t="n">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T11:00</t>
+        </is>
+      </c>
+      <c r="B705" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C705" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D705" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E705" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F705" s="9" t="n"/>
+      <c r="G705" s="9" t="n"/>
+      <c r="H705" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I705" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J705" s="9" t="n">
+        <v>534.5</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T12:00</t>
+        </is>
+      </c>
+      <c r="B706" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C706" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D706" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="E706" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F706" s="8" t="n"/>
+      <c r="G706" s="8" t="n"/>
+      <c r="H706" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I706" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J706" s="8" t="n">
+        <v>1186.9</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T13:00</t>
+        </is>
+      </c>
+      <c r="B707" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C707" s="9" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="D707" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E707" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F707" s="9" t="n"/>
+      <c r="G707" s="9" t="n"/>
+      <c r="H707" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I707" s="9" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J707" s="9" t="n">
+        <v>1566.4</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T14:00</t>
+        </is>
+      </c>
+      <c r="B708" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C708" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D708" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E708" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F708" s="8" t="n"/>
+      <c r="G708" s="8" t="n"/>
+      <c r="H708" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I708" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J708" s="8" t="n"/>
+    </row>
+    <row r="709">
+      <c r="A709" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T15:00</t>
+        </is>
+      </c>
+      <c r="B709" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C709" s="9" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D709" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E709" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F709" s="9" t="n"/>
+      <c r="G709" s="9" t="n"/>
+      <c r="H709" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I709" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J709" s="9" t="n"/>
+    </row>
+    <row r="710">
+      <c r="A710" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T16:00</t>
+        </is>
+      </c>
+      <c r="B710" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C710" s="8" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="D710" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E710" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F710" s="8" t="n"/>
+      <c r="G710" s="8" t="n"/>
+      <c r="H710" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I710" s="8" t="n">
+        <v>1018.1</v>
+      </c>
+      <c r="J710" s="8" t="n">
+        <v>2769.3</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T17:00</t>
+        </is>
+      </c>
+      <c r="B711" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C711" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D711" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E711" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F711" s="9" t="n"/>
+      <c r="G711" s="9" t="n"/>
+      <c r="H711" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I711" s="9" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J711" s="9" t="n">
+        <v>2151.5</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T18:00</t>
+        </is>
+      </c>
+      <c r="B712" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C712" s="8" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D712" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E712" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F712" s="8" t="n"/>
+      <c r="G712" s="8" t="n"/>
+      <c r="H712" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I712" s="8" t="n">
+        <v>1018</v>
+      </c>
+      <c r="J712" s="8" t="n">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T19:00</t>
+        </is>
+      </c>
+      <c r="B713" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C713" s="9" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D713" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E713" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F713" s="9" t="n"/>
+      <c r="G713" s="9" t="n"/>
+      <c r="H713" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I713" s="9" t="n">
+        <v>1018.5</v>
+      </c>
+      <c r="J713" s="9" t="n">
+        <v>740.9</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T20:00</t>
+        </is>
+      </c>
+      <c r="B714" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C714" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D714" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E714" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F714" s="8" t="n"/>
+      <c r="G714" s="8" t="n"/>
+      <c r="H714" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I714" s="8" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J714" s="8" t="n">
+        <v>172.7</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T21:00</t>
+        </is>
+      </c>
+      <c r="B715" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C715" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D715" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E715" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F715" s="9" t="n"/>
+      <c r="G715" s="9" t="n"/>
+      <c r="H715" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I715" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J715" s="9" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04T22:00</t>
+        </is>
+      </c>
+      <c r="B716" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C716" s="8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D716" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E716" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F716" s="8" t="n"/>
+      <c r="G716" s="8" t="n"/>
+      <c r="H716" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I716" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J716" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-04T23:00</t>
+        </is>
+      </c>
+      <c r="B717" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C717" s="9" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D717" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E717" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F717" s="9" t="n"/>
+      <c r="G717" s="9" t="n"/>
+      <c r="H717" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I717" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J717" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-05 04:39 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J717"/>
+  <dimension ref="A1:J722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -24082,6 +24082,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="718">
+      <c r="A718" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:00</t>
+        </is>
+      </c>
+      <c r="B718" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C718" s="8" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D718" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="E718" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F718" s="8" t="n"/>
+      <c r="G718" s="8" t="n"/>
+      <c r="H718" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I718" s="8" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J718" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T01:00</t>
+        </is>
+      </c>
+      <c r="B719" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C719" s="9" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="D719" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E719" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F719" s="9" t="n"/>
+      <c r="G719" s="9" t="n"/>
+      <c r="H719" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I719" s="9" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J719" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T02:00</t>
+        </is>
+      </c>
+      <c r="B720" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C720" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D720" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E720" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F720" s="8" t="n"/>
+      <c r="G720" s="8" t="n"/>
+      <c r="H720" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I720" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J720" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T03:00</t>
+        </is>
+      </c>
+      <c r="B721" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C721" s="9" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D721" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E721" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F721" s="9" t="n"/>
+      <c r="G721" s="9" t="n"/>
+      <c r="H721" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I721" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J721" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T04:00</t>
+        </is>
+      </c>
+      <c r="B722" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C722" s="8" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="D722" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E722" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F722" s="8" t="n"/>
+      <c r="G722" s="8" t="n"/>
+      <c r="H722" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I722" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J722" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-06 00:01 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J722"/>
+  <dimension ref="A1:J741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -24252,6 +24252,646 @@
         <v>0</v>
       </c>
     </row>
+    <row r="723">
+      <c r="A723" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T05:00</t>
+        </is>
+      </c>
+      <c r="B723" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C723" s="9" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D723" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E723" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F723" s="9" t="n"/>
+      <c r="G723" s="9" t="n"/>
+      <c r="H723" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I723" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J723" s="9" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T06:00</t>
+        </is>
+      </c>
+      <c r="B724" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C724" s="8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D724" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E724" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F724" s="8" t="n"/>
+      <c r="G724" s="8" t="n"/>
+      <c r="H724" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I724" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J724" s="8" t="n">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T07:00</t>
+        </is>
+      </c>
+      <c r="B725" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C725" s="9" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D725" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="E725" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F725" s="9" t="n"/>
+      <c r="G725" s="9" t="n"/>
+      <c r="H725" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I725" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J725" s="9" t="n">
+        <v>623.7</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T08:00</t>
+        </is>
+      </c>
+      <c r="B726" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C726" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D726" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E726" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F726" s="8" t="n"/>
+      <c r="G726" s="8" t="n"/>
+      <c r="H726" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I726" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J726" s="8" t="n">
+        <v>1362.9</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T09:00</t>
+        </is>
+      </c>
+      <c r="B727" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C727" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D727" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E727" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F727" s="9" t="n"/>
+      <c r="G727" s="9" t="n"/>
+      <c r="H727" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I727" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J727" s="9" t="n">
+        <v>1994.1</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T10:00</t>
+        </is>
+      </c>
+      <c r="B728" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C728" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="D728" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E728" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F728" s="8" t="n"/>
+      <c r="G728" s="8" t="n"/>
+      <c r="H728" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I728" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J728" s="8" t="n">
+        <v>2569.6</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T11:00</t>
+        </is>
+      </c>
+      <c r="B729" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C729" s="9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="D729" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E729" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F729" s="9" t="n"/>
+      <c r="G729" s="9" t="n"/>
+      <c r="H729" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I729" s="9" t="n">
+        <v>1017.6</v>
+      </c>
+      <c r="J729" s="9" t="n"/>
+    </row>
+    <row r="730">
+      <c r="A730" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T12:00</t>
+        </is>
+      </c>
+      <c r="B730" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C730" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D730" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E730" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F730" s="8" t="n"/>
+      <c r="G730" s="8" t="n"/>
+      <c r="H730" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I730" s="8" t="n">
+        <v>1017.7</v>
+      </c>
+      <c r="J730" s="8" t="n">
+        <v>2185.3</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T13:00</t>
+        </is>
+      </c>
+      <c r="B731" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C731" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="D731" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E731" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F731" s="9" t="n"/>
+      <c r="G731" s="9" t="n"/>
+      <c r="H731" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I731" s="9" t="n">
+        <v>1017.5</v>
+      </c>
+      <c r="J731" s="9" t="n"/>
+    </row>
+    <row r="732">
+      <c r="A732" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T14:00</t>
+        </is>
+      </c>
+      <c r="B732" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C732" s="8" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="D732" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E732" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F732" s="8" t="n"/>
+      <c r="G732" s="8" t="n"/>
+      <c r="H732" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I732" s="8" t="n">
+        <v>1017.5</v>
+      </c>
+      <c r="J732" s="8" t="n"/>
+    </row>
+    <row r="733">
+      <c r="A733" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T15:00</t>
+        </is>
+      </c>
+      <c r="B733" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C733" s="9" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="D733" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E733" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F733" s="9" t="n"/>
+      <c r="G733" s="9" t="n"/>
+      <c r="H733" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I733" s="9" t="n">
+        <v>1017.3</v>
+      </c>
+      <c r="J733" s="9" t="n">
+        <v>3114.8</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:00</t>
+        </is>
+      </c>
+      <c r="B734" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C734" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="D734" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="E734" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F734" s="8" t="n"/>
+      <c r="G734" s="8" t="n"/>
+      <c r="H734" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I734" s="8" t="n">
+        <v>1017.2</v>
+      </c>
+      <c r="J734" s="8" t="n">
+        <v>2201.7</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T17:00</t>
+        </is>
+      </c>
+      <c r="B735" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C735" s="9" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="D735" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="E735" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F735" s="9" t="n"/>
+      <c r="G735" s="9" t="n"/>
+      <c r="H735" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I735" s="9" t="n">
+        <v>1016.9</v>
+      </c>
+      <c r="J735" s="9" t="n">
+        <v>1945.1</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T18:00</t>
+        </is>
+      </c>
+      <c r="B736" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C736" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D736" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="E736" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F736" s="8" t="n"/>
+      <c r="G736" s="8" t="n"/>
+      <c r="H736" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I736" s="8" t="n">
+        <v>1017.2</v>
+      </c>
+      <c r="J736" s="8" t="n">
+        <v>1376.6</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:00</t>
+        </is>
+      </c>
+      <c r="B737" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C737" s="9" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="D737" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="E737" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F737" s="9" t="n"/>
+      <c r="G737" s="9" t="n"/>
+      <c r="H737" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I737" s="9" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J737" s="9" t="n">
+        <v>511.6</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T20:00</t>
+        </is>
+      </c>
+      <c r="B738" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C738" s="8" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D738" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="E738" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F738" s="8" t="n"/>
+      <c r="G738" s="8" t="n"/>
+      <c r="H738" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I738" s="8" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J738" s="8" t="n">
+        <v>73.7</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T21:00</t>
+        </is>
+      </c>
+      <c r="B739" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C739" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D739" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E739" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F739" s="9" t="n"/>
+      <c r="G739" s="9" t="n"/>
+      <c r="H739" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I739" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J739" s="9" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05T22:00</t>
+        </is>
+      </c>
+      <c r="B740" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C740" s="8" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="D740" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E740" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F740" s="8" t="n"/>
+      <c r="G740" s="8" t="n"/>
+      <c r="H740" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I740" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J740" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-05T23:00</t>
+        </is>
+      </c>
+      <c r="B741" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C741" s="9" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D741" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="E741" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F741" s="9" t="n"/>
+      <c r="G741" s="9" t="n"/>
+      <c r="H741" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I741" s="9" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J741" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-06 04:12 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J741"/>
+  <dimension ref="A1:J745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -24892,6 +24892,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="742">
+      <c r="A742" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T00:00</t>
+        </is>
+      </c>
+      <c r="B742" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C742" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D742" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E742" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F742" s="8" t="n"/>
+      <c r="G742" s="8" t="n"/>
+      <c r="H742" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I742" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J742" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T01:00</t>
+        </is>
+      </c>
+      <c r="B743" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C743" s="9" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D743" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="E743" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F743" s="9" t="n"/>
+      <c r="G743" s="9" t="n"/>
+      <c r="H743" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I743" s="9" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J743" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T02:00</t>
+        </is>
+      </c>
+      <c r="B744" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C744" s="8" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D744" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="E744" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F744" s="8" t="n"/>
+      <c r="G744" s="8" t="n"/>
+      <c r="H744" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I744" s="8" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J744" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T03:00</t>
+        </is>
+      </c>
+      <c r="B745" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C745" s="9" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D745" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E745" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F745" s="9" t="n"/>
+      <c r="G745" s="9" t="n"/>
+      <c r="H745" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I745" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J745" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-06 23:59 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J745"/>
+  <dimension ref="A1:J765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -25028,6 +25028,678 @@
         <v>0</v>
       </c>
     </row>
+    <row r="746">
+      <c r="A746" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T04:00</t>
+        </is>
+      </c>
+      <c r="B746" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C746" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D746" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E746" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F746" s="8" t="n"/>
+      <c r="G746" s="8" t="n"/>
+      <c r="H746" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I746" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J746" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T05:00</t>
+        </is>
+      </c>
+      <c r="B747" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C747" s="9" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D747" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="E747" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F747" s="9" t="n"/>
+      <c r="G747" s="9" t="n"/>
+      <c r="H747" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I747" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J747" s="9" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T06:00</t>
+        </is>
+      </c>
+      <c r="B748" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C748" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D748" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E748" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F748" s="8" t="n"/>
+      <c r="G748" s="8" t="n"/>
+      <c r="H748" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I748" s="8" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J748" s="8" t="n">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T07:00</t>
+        </is>
+      </c>
+      <c r="B749" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C749" s="9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D749" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E749" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F749" s="9" t="n"/>
+      <c r="G749" s="9" t="n"/>
+      <c r="H749" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I749" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J749" s="9" t="n">
+        <v>191.5</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T08:00</t>
+        </is>
+      </c>
+      <c r="B750" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C750" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D750" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E750" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F750" s="8" t="n"/>
+      <c r="G750" s="8" t="n"/>
+      <c r="H750" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I750" s="8" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="J750" s="8" t="n">
+        <v>454.2</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T09:00</t>
+        </is>
+      </c>
+      <c r="B751" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C751" s="9" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="D751" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="E751" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F751" s="9" t="n"/>
+      <c r="G751" s="9" t="n"/>
+      <c r="H751" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I751" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J751" s="9" t="n">
+        <v>1143.1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T10:00</t>
+        </is>
+      </c>
+      <c r="B752" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C752" s="8" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="D752" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E752" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F752" s="8" t="n"/>
+      <c r="G752" s="8" t="n"/>
+      <c r="H752" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I752" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J752" s="8" t="n">
+        <v>1373.7</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T11:00</t>
+        </is>
+      </c>
+      <c r="B753" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C753" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="D753" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E753" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F753" s="9" t="n"/>
+      <c r="G753" s="9" t="n"/>
+      <c r="H753" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I753" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J753" s="9" t="n"/>
+    </row>
+    <row r="754">
+      <c r="A754" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T12:00</t>
+        </is>
+      </c>
+      <c r="B754" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C754" s="8" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="D754" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E754" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F754" s="8" t="n"/>
+      <c r="G754" s="8" t="n"/>
+      <c r="H754" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I754" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J754" s="8" t="n"/>
+    </row>
+    <row r="755">
+      <c r="A755" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T13:00</t>
+        </is>
+      </c>
+      <c r="B755" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C755" s="9" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="D755" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="E755" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F755" s="9" t="n"/>
+      <c r="G755" s="9" t="n"/>
+      <c r="H755" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I755" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J755" s="9" t="n"/>
+    </row>
+    <row r="756">
+      <c r="A756" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T14:00</t>
+        </is>
+      </c>
+      <c r="B756" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C756" s="8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D756" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E756" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F756" s="8" t="n"/>
+      <c r="G756" s="8" t="n"/>
+      <c r="H756" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I756" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J756" s="8" t="n"/>
+    </row>
+    <row r="757">
+      <c r="A757" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T15:00</t>
+        </is>
+      </c>
+      <c r="B757" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C757" s="9" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D757" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="E757" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F757" s="9" t="n"/>
+      <c r="G757" s="9" t="n"/>
+      <c r="H757" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I757" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J757" s="9" t="n">
+        <v>3111.6</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T16:00</t>
+        </is>
+      </c>
+      <c r="B758" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C758" s="8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D758" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E758" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F758" s="8" t="n"/>
+      <c r="G758" s="8" t="n"/>
+      <c r="H758" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I758" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J758" s="8" t="n">
+        <v>2721.7</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T17:00</t>
+        </is>
+      </c>
+      <c r="B759" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C759" s="9" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D759" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E759" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F759" s="9" t="n"/>
+      <c r="G759" s="9" t="n"/>
+      <c r="H759" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I759" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J759" s="9" t="n">
+        <v>1396.8</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T18:00</t>
+        </is>
+      </c>
+      <c r="B760" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C760" s="8" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D760" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E760" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F760" s="8" t="n"/>
+      <c r="G760" s="8" t="n"/>
+      <c r="H760" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I760" s="8" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J760" s="8" t="n">
+        <v>946.4</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T19:00</t>
+        </is>
+      </c>
+      <c r="B761" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C761" s="9" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D761" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="E761" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F761" s="9" t="n"/>
+      <c r="G761" s="9" t="n"/>
+      <c r="H761" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I761" s="9" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="J761" s="9" t="n">
+        <v>648.2</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T20:00</t>
+        </is>
+      </c>
+      <c r="B762" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C762" s="8" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D762" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E762" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F762" s="8" t="n"/>
+      <c r="G762" s="8" t="n"/>
+      <c r="H762" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I762" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J762" s="8" t="n">
+        <v>238.3</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T21:00</t>
+        </is>
+      </c>
+      <c r="B763" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C763" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D763" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="E763" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F763" s="9" t="n"/>
+      <c r="G763" s="9" t="n"/>
+      <c r="H763" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I763" s="9" t="n">
+        <v>1020</v>
+      </c>
+      <c r="J763" s="9" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06T22:00</t>
+        </is>
+      </c>
+      <c r="B764" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C764" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D764" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E764" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F764" s="8" t="n"/>
+      <c r="G764" s="8" t="n"/>
+      <c r="H764" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I764" s="8" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J764" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-06T23:00</t>
+        </is>
+      </c>
+      <c r="B765" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C765" s="9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D765" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E765" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F765" s="9" t="n"/>
+      <c r="G765" s="9" t="n"/>
+      <c r="H765" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I765" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J765" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-07 04:48 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J765"/>
+  <dimension ref="A1:J770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -25700,6 +25700,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="766">
+      <c r="A766" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T00:00</t>
+        </is>
+      </c>
+      <c r="B766" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C766" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D766" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E766" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F766" s="8" t="n"/>
+      <c r="G766" s="8" t="n"/>
+      <c r="H766" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I766" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J766" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T01:00</t>
+        </is>
+      </c>
+      <c r="B767" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C767" s="9" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D767" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E767" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F767" s="9" t="n"/>
+      <c r="G767" s="9" t="n"/>
+      <c r="H767" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I767" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J767" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T02:00</t>
+        </is>
+      </c>
+      <c r="B768" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C768" s="8" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="D768" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E768" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F768" s="8" t="n"/>
+      <c r="G768" s="8" t="n"/>
+      <c r="H768" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I768" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J768" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T03:00</t>
+        </is>
+      </c>
+      <c r="B769" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C769" s="9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D769" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E769" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F769" s="9" t="n"/>
+      <c r="G769" s="9" t="n"/>
+      <c r="H769" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I769" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J769" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T04:00</t>
+        </is>
+      </c>
+      <c r="B770" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C770" s="8" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D770" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E770" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F770" s="8" t="n"/>
+      <c r="G770" s="8" t="n"/>
+      <c r="H770" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I770" s="8" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J770" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-08 00:02 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J770"/>
+  <dimension ref="A1:J789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -25870,6 +25870,652 @@
         <v>0</v>
       </c>
     </row>
+    <row r="771">
+      <c r="A771" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T05:00</t>
+        </is>
+      </c>
+      <c r="B771" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C771" s="9" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D771" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="E771" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F771" s="9" t="n"/>
+      <c r="G771" s="9" t="n"/>
+      <c r="H771" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I771" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J771" s="9" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00</t>
+        </is>
+      </c>
+      <c r="B772" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C772" s="8" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D772" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E772" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F772" s="8" t="n"/>
+      <c r="G772" s="8" t="n"/>
+      <c r="H772" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I772" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J772" s="8" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T07:00</t>
+        </is>
+      </c>
+      <c r="B773" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C773" s="9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D773" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="E773" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F773" s="9" t="n"/>
+      <c r="G773" s="9" t="n"/>
+      <c r="H773" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I773" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J773" s="9" t="n">
+        <v>506.8</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T08:00</t>
+        </is>
+      </c>
+      <c r="B774" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C774" s="8" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D774" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="E774" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F774" s="8" t="n"/>
+      <c r="G774" s="8" t="n"/>
+      <c r="H774" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I774" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J774" s="8" t="n">
+        <v>1519.4</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T09:00</t>
+        </is>
+      </c>
+      <c r="B775" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C775" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D775" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E775" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F775" s="9" t="n"/>
+      <c r="G775" s="9" t="n"/>
+      <c r="H775" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I775" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J775" s="9" t="n">
+        <v>1916.2</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T10:00</t>
+        </is>
+      </c>
+      <c r="B776" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C776" s="8" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="D776" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E776" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F776" s="8" t="n"/>
+      <c r="G776" s="8" t="n"/>
+      <c r="H776" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I776" s="8" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J776" s="8" t="n">
+        <v>2609.2</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T11:00</t>
+        </is>
+      </c>
+      <c r="B777" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C777" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D777" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E777" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F777" s="9" t="n"/>
+      <c r="G777" s="9" t="n"/>
+      <c r="H777" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I777" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J777" s="9" t="n">
+        <v>3118</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T12:00</t>
+        </is>
+      </c>
+      <c r="B778" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C778" s="8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D778" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E778" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F778" s="8" t="n"/>
+      <c r="G778" s="8" t="n"/>
+      <c r="H778" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I778" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J778" s="8" t="n">
+        <v>3412.3</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T13:00</t>
+        </is>
+      </c>
+      <c r="B779" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C779" s="9" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D779" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="E779" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F779" s="9" t="n"/>
+      <c r="G779" s="9" t="n"/>
+      <c r="H779" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I779" s="9" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J779" s="9" t="n">
+        <v>3514.6</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T14:00</t>
+        </is>
+      </c>
+      <c r="B780" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C780" s="8" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D780" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E780" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F780" s="8" t="n"/>
+      <c r="G780" s="8" t="n"/>
+      <c r="H780" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I780" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J780" s="8" t="n">
+        <v>3390.7</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T15:00</t>
+        </is>
+      </c>
+      <c r="B781" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C781" s="9" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="D781" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E781" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F781" s="9" t="n"/>
+      <c r="G781" s="9" t="n"/>
+      <c r="H781" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I781" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J781" s="9" t="n">
+        <v>3146.8</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T16:00</t>
+        </is>
+      </c>
+      <c r="B782" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C782" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="D782" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E782" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F782" s="8" t="n"/>
+      <c r="G782" s="8" t="n"/>
+      <c r="H782" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I782" s="8" t="n">
+        <v>1019.6</v>
+      </c>
+      <c r="J782" s="8" t="n">
+        <v>2724.8</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T17:00</t>
+        </is>
+      </c>
+      <c r="B783" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C783" s="9" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="D783" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="E783" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F783" s="9" t="n"/>
+      <c r="G783" s="9" t="n"/>
+      <c r="H783" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I783" s="9" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J783" s="9" t="n">
+        <v>2100.2</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T18:00</t>
+        </is>
+      </c>
+      <c r="B784" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C784" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D784" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="E784" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F784" s="8" t="n"/>
+      <c r="G784" s="8" t="n"/>
+      <c r="H784" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I784" s="8" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J784" s="8" t="n">
+        <v>1435.2</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T19:00</t>
+        </is>
+      </c>
+      <c r="B785" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C785" s="9" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="D785" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E785" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F785" s="9" t="n"/>
+      <c r="G785" s="9" t="n"/>
+      <c r="H785" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I785" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J785" s="9" t="n">
+        <v>746.3</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T20:00</t>
+        </is>
+      </c>
+      <c r="B786" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C786" s="8" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="D786" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="E786" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F786" s="8" t="n"/>
+      <c r="G786" s="8" t="n"/>
+      <c r="H786" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I786" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J786" s="8" t="n">
+        <v>176.1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T21:00</t>
+        </is>
+      </c>
+      <c r="B787" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C787" s="9" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D787" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="E787" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F787" s="9" t="n"/>
+      <c r="G787" s="9" t="n"/>
+      <c r="H787" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I787" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J787" s="9" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-07T22:00</t>
+        </is>
+      </c>
+      <c r="B788" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C788" s="8" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D788" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E788" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F788" s="8" t="n"/>
+      <c r="G788" s="8" t="n"/>
+      <c r="H788" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I788" s="8" t="n">
+        <v>1022.7</v>
+      </c>
+      <c r="J788" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07T23:00</t>
+        </is>
+      </c>
+      <c r="B789" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C789" s="9" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D789" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E789" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F789" s="9" t="n"/>
+      <c r="G789" s="9" t="n"/>
+      <c r="H789" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I789" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J789" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-08 04:53 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J789"/>
+  <dimension ref="A1:J794"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -26516,6 +26516,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="790">
+      <c r="A790" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T00:00</t>
+        </is>
+      </c>
+      <c r="B790" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C790" s="8" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="D790" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="E790" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F790" s="8" t="n"/>
+      <c r="G790" s="8" t="n"/>
+      <c r="H790" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I790" s="8" t="n">
+        <v>1023.2</v>
+      </c>
+      <c r="J790" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T01:00</t>
+        </is>
+      </c>
+      <c r="B791" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C791" s="9" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D791" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="E791" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F791" s="9" t="n"/>
+      <c r="G791" s="9" t="n"/>
+      <c r="H791" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I791" s="9" t="n">
+        <v>1023.3</v>
+      </c>
+      <c r="J791" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T02:00</t>
+        </is>
+      </c>
+      <c r="B792" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C792" s="8" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D792" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="E792" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F792" s="8" t="n"/>
+      <c r="G792" s="8" t="n"/>
+      <c r="H792" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I792" s="8" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J792" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T03:00</t>
+        </is>
+      </c>
+      <c r="B793" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C793" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D793" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="E793" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F793" s="9" t="n"/>
+      <c r="G793" s="9" t="n"/>
+      <c r="H793" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I793" s="9" t="n">
+        <v>1023</v>
+      </c>
+      <c r="J793" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T04:00</t>
+        </is>
+      </c>
+      <c r="B794" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C794" s="8" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D794" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="E794" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F794" s="8" t="n"/>
+      <c r="G794" s="8" t="n"/>
+      <c r="H794" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I794" s="8" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J794" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-09 00:00 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J794"/>
+  <dimension ref="A1:J813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -26686,6 +26686,648 @@
         <v>0</v>
       </c>
     </row>
+    <row r="795">
+      <c r="A795" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T05:00</t>
+        </is>
+      </c>
+      <c r="B795" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C795" s="9" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D795" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E795" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F795" s="9" t="n"/>
+      <c r="G795" s="9" t="n"/>
+      <c r="H795" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I795" s="9" t="n">
+        <v>1023.3</v>
+      </c>
+      <c r="J795" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:00</t>
+        </is>
+      </c>
+      <c r="B796" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C796" s="8" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D796" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E796" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F796" s="8" t="n"/>
+      <c r="G796" s="8" t="n"/>
+      <c r="H796" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I796" s="8" t="n">
+        <v>1023.6</v>
+      </c>
+      <c r="J796" s="8" t="n">
+        <v>95.40000000000001</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T07:00</t>
+        </is>
+      </c>
+      <c r="B797" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C797" s="9" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D797" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E797" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F797" s="9" t="n"/>
+      <c r="G797" s="9" t="n"/>
+      <c r="H797" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I797" s="9" t="n">
+        <v>1023.6</v>
+      </c>
+      <c r="J797" s="9" t="n">
+        <v>672.3</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T08:00</t>
+        </is>
+      </c>
+      <c r="B798" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C798" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D798" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E798" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F798" s="8" t="n"/>
+      <c r="G798" s="8" t="n"/>
+      <c r="H798" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I798" s="8" t="n">
+        <v>1023.6</v>
+      </c>
+      <c r="J798" s="8" t="n">
+        <v>1326.7</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T09:00</t>
+        </is>
+      </c>
+      <c r="B799" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C799" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="D799" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="E799" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F799" s="9" t="n"/>
+      <c r="G799" s="9" t="n"/>
+      <c r="H799" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I799" s="9" t="n">
+        <v>1023.9</v>
+      </c>
+      <c r="J799" s="9" t="n">
+        <v>2007.2</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T10:00</t>
+        </is>
+      </c>
+      <c r="B800" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C800" s="8" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D800" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E800" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F800" s="8" t="n"/>
+      <c r="G800" s="8" t="n"/>
+      <c r="H800" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I800" s="8" t="n">
+        <v>1023.8</v>
+      </c>
+      <c r="J800" s="8" t="n">
+        <v>2613.6</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T11:00</t>
+        </is>
+      </c>
+      <c r="B801" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C801" s="9" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D801" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E801" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F801" s="9" t="n"/>
+      <c r="G801" s="9" t="n"/>
+      <c r="H801" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I801" s="9" t="n">
+        <v>1023.4</v>
+      </c>
+      <c r="J801" s="9" t="n">
+        <v>3100.9</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T12:00</t>
+        </is>
+      </c>
+      <c r="B802" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C802" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="D802" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="E802" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F802" s="8" t="n"/>
+      <c r="G802" s="8" t="n"/>
+      <c r="H802" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I802" s="8" t="n">
+        <v>1023.1</v>
+      </c>
+      <c r="J802" s="8" t="n">
+        <v>3380.3</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T13:00</t>
+        </is>
+      </c>
+      <c r="B803" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C803" s="9" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D803" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E803" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F803" s="9" t="n"/>
+      <c r="G803" s="9" t="n"/>
+      <c r="H803" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I803" s="9" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J803" s="9" t="n">
+        <v>3441.7</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T14:00</t>
+        </is>
+      </c>
+      <c r="B804" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C804" s="8" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D804" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E804" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F804" s="8" t="n"/>
+      <c r="G804" s="8" t="n"/>
+      <c r="H804" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I804" s="8" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J804" s="8" t="n"/>
+    </row>
+    <row r="805">
+      <c r="A805" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T15:00</t>
+        </is>
+      </c>
+      <c r="B805" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C805" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D805" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E805" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F805" s="9" t="n"/>
+      <c r="G805" s="9" t="n"/>
+      <c r="H805" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I805" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J805" s="9" t="n"/>
+    </row>
+    <row r="806">
+      <c r="A806" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T16:00</t>
+        </is>
+      </c>
+      <c r="B806" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C806" s="8" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D806" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E806" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F806" s="8" t="n"/>
+      <c r="G806" s="8" t="n"/>
+      <c r="H806" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I806" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J806" s="8" t="n">
+        <v>2054.6</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T17:00</t>
+        </is>
+      </c>
+      <c r="B807" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C807" s="9" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D807" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E807" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F807" s="9" t="n"/>
+      <c r="G807" s="9" t="n"/>
+      <c r="H807" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I807" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J807" s="9" t="n">
+        <v>1511.5</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T18:00</t>
+        </is>
+      </c>
+      <c r="B808" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C808" s="8" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D808" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E808" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F808" s="8" t="n"/>
+      <c r="G808" s="8" t="n"/>
+      <c r="H808" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I808" s="8" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J808" s="8" t="n">
+        <v>853.2</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T19:00</t>
+        </is>
+      </c>
+      <c r="B809" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C809" s="9" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D809" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E809" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F809" s="9" t="n"/>
+      <c r="G809" s="9" t="n"/>
+      <c r="H809" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I809" s="9" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J809" s="9" t="n">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T20:00</t>
+        </is>
+      </c>
+      <c r="B810" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C810" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D810" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="E810" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F810" s="8" t="n"/>
+      <c r="G810" s="8" t="n"/>
+      <c r="H810" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I810" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J810" s="8" t="n">
+        <v>141.3</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T21:00</t>
+        </is>
+      </c>
+      <c r="B811" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C811" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D811" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="E811" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F811" s="9" t="n"/>
+      <c r="G811" s="9" t="n"/>
+      <c r="H811" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I811" s="9" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="J811" s="9" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-08T22:00</t>
+        </is>
+      </c>
+      <c r="B812" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C812" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D812" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E812" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F812" s="8" t="n"/>
+      <c r="G812" s="8" t="n"/>
+      <c r="H812" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I812" s="8" t="n">
+        <v>1022.5</v>
+      </c>
+      <c r="J812" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08T23:00</t>
+        </is>
+      </c>
+      <c r="B813" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C813" s="9" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="D813" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E813" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F813" s="9" t="n"/>
+      <c r="G813" s="9" t="n"/>
+      <c r="H813" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I813" s="9" t="n">
+        <v>1022.6</v>
+      </c>
+      <c r="J813" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-09 04:15 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J813"/>
+  <dimension ref="A1:J817"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -27328,6 +27328,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="814">
+      <c r="A814" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T00:00</t>
+        </is>
+      </c>
+      <c r="B814" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C814" s="8" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D814" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E814" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F814" s="8" t="n"/>
+      <c r="G814" s="8" t="n"/>
+      <c r="H814" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I814" s="8" t="n">
+        <v>1022.4</v>
+      </c>
+      <c r="J814" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T01:00</t>
+        </is>
+      </c>
+      <c r="B815" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C815" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D815" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="E815" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F815" s="9" t="n"/>
+      <c r="G815" s="9" t="n"/>
+      <c r="H815" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I815" s="9" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J815" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T02:00</t>
+        </is>
+      </c>
+      <c r="B816" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C816" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D816" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E816" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F816" s="8" t="n"/>
+      <c r="G816" s="8" t="n"/>
+      <c r="H816" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I816" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J816" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T03:00</t>
+        </is>
+      </c>
+      <c r="B817" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C817" s="9" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D817" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="E817" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F817" s="9" t="n"/>
+      <c r="G817" s="9" t="n"/>
+      <c r="H817" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I817" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J817" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-10 00:07 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J817"/>
+  <dimension ref="A1:J837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -27464,6 +27464,686 @@
         <v>0</v>
       </c>
     </row>
+    <row r="818">
+      <c r="A818" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T04:00</t>
+        </is>
+      </c>
+      <c r="B818" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C818" s="8" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D818" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E818" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F818" s="8" t="n"/>
+      <c r="G818" s="8" t="n"/>
+      <c r="H818" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I818" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J818" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T05:00</t>
+        </is>
+      </c>
+      <c r="B819" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C819" s="9" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="D819" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E819" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F819" s="9" t="n"/>
+      <c r="G819" s="9" t="n"/>
+      <c r="H819" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I819" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J819" s="9" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T06:00</t>
+        </is>
+      </c>
+      <c r="B820" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C820" s="8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D820" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E820" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F820" s="8" t="n"/>
+      <c r="G820" s="8" t="n"/>
+      <c r="H820" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I820" s="8" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J820" s="8" t="n">
+        <v>38.3</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T07:00</t>
+        </is>
+      </c>
+      <c r="B821" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C821" s="9" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D821" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E821" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F821" s="9" t="n"/>
+      <c r="G821" s="9" t="n"/>
+      <c r="H821" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I821" s="9" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J821" s="9" t="n">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T08:00</t>
+        </is>
+      </c>
+      <c r="B822" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C822" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="D822" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E822" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F822" s="8" t="n"/>
+      <c r="G822" s="8" t="n"/>
+      <c r="H822" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I822" s="8" t="n">
+        <v>1022</v>
+      </c>
+      <c r="J822" s="8" t="n">
+        <v>1444.6</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T09:00</t>
+        </is>
+      </c>
+      <c r="B823" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C823" s="9" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D823" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E823" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F823" s="9" t="n"/>
+      <c r="G823" s="9" t="n"/>
+      <c r="H823" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I823" s="9" t="n">
+        <v>1021.9</v>
+      </c>
+      <c r="J823" s="9" t="n">
+        <v>2052.8</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T10:00</t>
+        </is>
+      </c>
+      <c r="B824" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C824" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D824" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E824" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F824" s="8" t="n"/>
+      <c r="G824" s="8" t="n"/>
+      <c r="H824" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I824" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J824" s="8" t="n">
+        <v>2677.4</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T11:00</t>
+        </is>
+      </c>
+      <c r="B825" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C825" s="9" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D825" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E825" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F825" s="9" t="n"/>
+      <c r="G825" s="9" t="n"/>
+      <c r="H825" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I825" s="9" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J825" s="9" t="n">
+        <v>3118.9</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T12:00</t>
+        </is>
+      </c>
+      <c r="B826" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C826" s="8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D826" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E826" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F826" s="8" t="n"/>
+      <c r="G826" s="8" t="n"/>
+      <c r="H826" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I826" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J826" s="8" t="n">
+        <v>3403.2</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T13:00</t>
+        </is>
+      </c>
+      <c r="B827" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C827" s="9" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="D827" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E827" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F827" s="9" t="n"/>
+      <c r="G827" s="9" t="n"/>
+      <c r="H827" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I827" s="9" t="n">
+        <v>1019.9</v>
+      </c>
+      <c r="J827" s="9" t="n">
+        <v>3510</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T14:00</t>
+        </is>
+      </c>
+      <c r="B828" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C828" s="8" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="D828" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="E828" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F828" s="8" t="n"/>
+      <c r="G828" s="8" t="n"/>
+      <c r="H828" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I828" s="8" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J828" s="8" t="n">
+        <v>3421.8</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T15:00</t>
+        </is>
+      </c>
+      <c r="B829" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C829" s="9" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D829" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E829" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F829" s="9" t="n"/>
+      <c r="G829" s="9" t="n"/>
+      <c r="H829" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I829" s="9" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J829" s="9" t="n">
+        <v>3182.1</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T16:00</t>
+        </is>
+      </c>
+      <c r="B830" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C830" s="8" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D830" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E830" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F830" s="8" t="n"/>
+      <c r="G830" s="8" t="n"/>
+      <c r="H830" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I830" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J830" s="8" t="n">
+        <v>2735.3</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T17:00</t>
+        </is>
+      </c>
+      <c r="B831" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C831" s="9" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D831" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E831" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F831" s="9" t="n"/>
+      <c r="G831" s="9" t="n"/>
+      <c r="H831" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I831" s="9" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J831" s="9" t="n">
+        <v>2114.8</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T18:00</t>
+        </is>
+      </c>
+      <c r="B832" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C832" s="8" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D832" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="E832" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F832" s="8" t="n"/>
+      <c r="G832" s="8" t="n"/>
+      <c r="H832" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I832" s="8" t="n">
+        <v>1018.7</v>
+      </c>
+      <c r="J832" s="8" t="n">
+        <v>1443.5</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T19:00</t>
+        </is>
+      </c>
+      <c r="B833" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C833" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="D833" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="E833" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F833" s="9" t="n"/>
+      <c r="G833" s="9" t="n"/>
+      <c r="H833" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I833" s="9" t="n">
+        <v>1019</v>
+      </c>
+      <c r="J833" s="9" t="n">
+        <v>749.7</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T20:00</t>
+        </is>
+      </c>
+      <c r="B834" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C834" s="8" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="D834" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E834" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F834" s="8" t="n"/>
+      <c r="G834" s="8" t="n"/>
+      <c r="H834" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I834" s="8" t="n">
+        <v>1019.7</v>
+      </c>
+      <c r="J834" s="8" t="n">
+        <v>175.4</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T21:00</t>
+        </is>
+      </c>
+      <c r="B835" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C835" s="9" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D835" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E835" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F835" s="9" t="n"/>
+      <c r="G835" s="9" t="n"/>
+      <c r="H835" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I835" s="9" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J835" s="9" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-09T22:00</t>
+        </is>
+      </c>
+      <c r="B836" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C836" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D836" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E836" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F836" s="8" t="n"/>
+      <c r="G836" s="8" t="n"/>
+      <c r="H836" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I836" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J836" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-09T23:00</t>
+        </is>
+      </c>
+      <c r="B837" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C837" s="9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D837" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E837" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F837" s="9" t="n"/>
+      <c r="G837" s="9" t="n"/>
+      <c r="H837" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I837" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J837" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-10 04:26 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J837"/>
+  <dimension ref="A1:J841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -28144,6 +28144,142 @@
         <v>0</v>
       </c>
     </row>
+    <row r="838">
+      <c r="A838" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T00:00</t>
+        </is>
+      </c>
+      <c r="B838" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C838" s="8" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D838" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E838" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F838" s="8" t="n"/>
+      <c r="G838" s="8" t="n"/>
+      <c r="H838" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I838" s="8" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J838" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T01:00</t>
+        </is>
+      </c>
+      <c r="B839" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C839" s="9" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D839" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E839" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F839" s="9" t="n"/>
+      <c r="G839" s="9" t="n"/>
+      <c r="H839" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I839" s="9" t="n">
+        <v>1021.5</v>
+      </c>
+      <c r="J839" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T02:00</t>
+        </is>
+      </c>
+      <c r="B840" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C840" s="8" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="D840" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E840" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F840" s="8" t="n"/>
+      <c r="G840" s="8" t="n"/>
+      <c r="H840" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I840" s="8" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J840" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T03:00</t>
+        </is>
+      </c>
+      <c r="B841" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C841" s="9" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="D841" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="E841" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F841" s="9" t="n"/>
+      <c r="G841" s="9" t="n"/>
+      <c r="H841" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I841" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J841" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-11 00:11 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J841"/>
+  <dimension ref="A1:J861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -28280,6 +28280,682 @@
         <v>0</v>
       </c>
     </row>
+    <row r="842">
+      <c r="A842" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T04:00</t>
+        </is>
+      </c>
+      <c r="B842" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C842" s="8" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="D842" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E842" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F842" s="8" t="n"/>
+      <c r="G842" s="8" t="n"/>
+      <c r="H842" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I842" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J842" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T05:00</t>
+        </is>
+      </c>
+      <c r="B843" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C843" s="9" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D843" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E843" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F843" s="9" t="n"/>
+      <c r="G843" s="9" t="n"/>
+      <c r="H843" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I843" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J843" s="9" t="n"/>
+    </row>
+    <row r="844">
+      <c r="A844" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T06:00</t>
+        </is>
+      </c>
+      <c r="B844" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C844" s="8" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D844" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="E844" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F844" s="8" t="n"/>
+      <c r="G844" s="8" t="n"/>
+      <c r="H844" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I844" s="8" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J844" s="8" t="n">
+        <v>89.90000000000001</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T07:00</t>
+        </is>
+      </c>
+      <c r="B845" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C845" s="9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="D845" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E845" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F845" s="9" t="n"/>
+      <c r="G845" s="9" t="n"/>
+      <c r="H845" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I845" s="9" t="n">
+        <v>1021.6</v>
+      </c>
+      <c r="J845" s="9" t="n">
+        <v>710.2</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T08:00</t>
+        </is>
+      </c>
+      <c r="B846" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C846" s="8" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D846" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E846" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F846" s="8" t="n"/>
+      <c r="G846" s="8" t="n"/>
+      <c r="H846" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I846" s="8" t="n">
+        <v>1021.7</v>
+      </c>
+      <c r="J846" s="8" t="n"/>
+    </row>
+    <row r="847">
+      <c r="A847" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T09:00</t>
+        </is>
+      </c>
+      <c r="B847" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C847" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="D847" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="E847" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F847" s="9" t="n"/>
+      <c r="G847" s="9" t="n"/>
+      <c r="H847" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I847" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J847" s="9" t="n">
+        <v>2027.4</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T10:00</t>
+        </is>
+      </c>
+      <c r="B848" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C848" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D848" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E848" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F848" s="8" t="n"/>
+      <c r="G848" s="8" t="n"/>
+      <c r="H848" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I848" s="8" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="J848" s="8" t="n">
+        <v>2598.4</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T11:00</t>
+        </is>
+      </c>
+      <c r="B849" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C849" s="9" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D849" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="E849" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F849" s="9" t="n"/>
+      <c r="G849" s="9" t="n"/>
+      <c r="H849" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I849" s="9" t="n">
+        <v>1020.7</v>
+      </c>
+      <c r="J849" s="9" t="n">
+        <v>3149.3</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T12:00</t>
+        </is>
+      </c>
+      <c r="B850" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C850" s="8" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="D850" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E850" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F850" s="8" t="n"/>
+      <c r="G850" s="8" t="n"/>
+      <c r="H850" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I850" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J850" s="8" t="n">
+        <v>3433.6</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T13:00</t>
+        </is>
+      </c>
+      <c r="B851" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C851" s="9" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="D851" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="E851" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F851" s="9" t="n"/>
+      <c r="G851" s="9" t="n"/>
+      <c r="H851" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I851" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J851" s="9" t="n">
+        <v>3536.1</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T14:00</t>
+        </is>
+      </c>
+      <c r="B852" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C852" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="D852" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="E852" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F852" s="8" t="n"/>
+      <c r="G852" s="8" t="n"/>
+      <c r="H852" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I852" s="8" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J852" s="8" t="n">
+        <v>3411.8</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T15:00</t>
+        </is>
+      </c>
+      <c r="B853" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C853" s="9" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="D853" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="E853" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F853" s="9" t="n"/>
+      <c r="G853" s="9" t="n"/>
+      <c r="H853" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I853" s="9" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J853" s="9" t="n">
+        <v>3167.4</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T16:00</t>
+        </is>
+      </c>
+      <c r="B854" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C854" s="8" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="D854" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E854" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F854" s="8" t="n"/>
+      <c r="G854" s="8" t="n"/>
+      <c r="H854" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I854" s="8" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J854" s="8" t="n">
+        <v>2724.8</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T17:00</t>
+        </is>
+      </c>
+      <c r="B855" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C855" s="9" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="D855" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="E855" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F855" s="9" t="n"/>
+      <c r="G855" s="9" t="n"/>
+      <c r="H855" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I855" s="9" t="n">
+        <v>1018</v>
+      </c>
+      <c r="J855" s="9" t="n">
+        <v>2109.8</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T18:00</t>
+        </is>
+      </c>
+      <c r="B856" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C856" s="8" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="D856" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E856" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F856" s="8" t="n"/>
+      <c r="G856" s="8" t="n"/>
+      <c r="H856" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I856" s="8" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="J856" s="8" t="n">
+        <v>1449.8</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T19:00</t>
+        </is>
+      </c>
+      <c r="B857" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C857" s="9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="D857" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="E857" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F857" s="9" t="n"/>
+      <c r="G857" s="9" t="n"/>
+      <c r="H857" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I857" s="9" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="J857" s="9" t="n">
+        <v>751.7</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T20:00</t>
+        </is>
+      </c>
+      <c r="B858" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C858" s="8" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D858" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="E858" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F858" s="8" t="n"/>
+      <c r="G858" s="8" t="n"/>
+      <c r="H858" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I858" s="8" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="J858" s="8" t="n">
+        <v>189.3</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T21:00</t>
+        </is>
+      </c>
+      <c r="B859" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C859" s="9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D859" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="E859" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F859" s="9" t="n"/>
+      <c r="G859" s="9" t="n"/>
+      <c r="H859" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I859" s="9" t="n">
+        <v>1019.5</v>
+      </c>
+      <c r="J859" s="9" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-10T22:00</t>
+        </is>
+      </c>
+      <c r="B860" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C860" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D860" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="E860" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F860" s="8" t="n"/>
+      <c r="G860" s="8" t="n"/>
+      <c r="H860" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I860" s="8" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J860" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10T23:00</t>
+        </is>
+      </c>
+      <c r="B861" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C861" s="9" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D861" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E861" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F861" s="9" t="n"/>
+      <c r="G861" s="9" t="n"/>
+      <c r="H861" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I861" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J861" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-11 04:49 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J861"/>
+  <dimension ref="A1:J866"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -28956,6 +28956,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="862">
+      <c r="A862" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T00:00</t>
+        </is>
+      </c>
+      <c r="B862" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C862" s="8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D862" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="E862" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F862" s="8" t="n"/>
+      <c r="G862" s="8" t="n"/>
+      <c r="H862" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I862" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J862" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T01:00</t>
+        </is>
+      </c>
+      <c r="B863" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C863" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D863" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E863" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F863" s="9" t="n"/>
+      <c r="G863" s="9" t="n"/>
+      <c r="H863" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I863" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J863" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T02:00</t>
+        </is>
+      </c>
+      <c r="B864" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C864" s="8" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="D864" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E864" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F864" s="8" t="n"/>
+      <c r="G864" s="8" t="n"/>
+      <c r="H864" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I864" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J864" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T03:00</t>
+        </is>
+      </c>
+      <c r="B865" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C865" s="9" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D865" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E865" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F865" s="9" t="n"/>
+      <c r="G865" s="9" t="n"/>
+      <c r="H865" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I865" s="9" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J865" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T04:00</t>
+        </is>
+      </c>
+      <c r="B866" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C866" s="8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="D866" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="E866" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F866" s="8" t="n"/>
+      <c r="G866" s="8" t="n"/>
+      <c r="H866" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I866" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J866" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-12 00:16 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J866"/>
+  <dimension ref="A1:J885"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -29126,6 +29126,652 @@
         <v>0</v>
       </c>
     </row>
+    <row r="867">
+      <c r="A867" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T05:00</t>
+        </is>
+      </c>
+      <c r="B867" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C867" s="9" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D867" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E867" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F867" s="9" t="n"/>
+      <c r="G867" s="9" t="n"/>
+      <c r="H867" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I867" s="9" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J867" s="9" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T06:00</t>
+        </is>
+      </c>
+      <c r="B868" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C868" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D868" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E868" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F868" s="8" t="n"/>
+      <c r="G868" s="8" t="n"/>
+      <c r="H868" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I868" s="8" t="n">
+        <v>1020.9</v>
+      </c>
+      <c r="J868" s="8" t="n">
+        <v>96.09999999999999</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T07:00</t>
+        </is>
+      </c>
+      <c r="B869" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C869" s="9" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D869" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E869" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F869" s="9" t="n"/>
+      <c r="G869" s="9" t="n"/>
+      <c r="H869" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I869" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J869" s="9" t="n">
+        <v>653.7</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T08:00</t>
+        </is>
+      </c>
+      <c r="B870" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C870" s="8" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="D870" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E870" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F870" s="8" t="n"/>
+      <c r="G870" s="8" t="n"/>
+      <c r="H870" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I870" s="8" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J870" s="8" t="n">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T09:00</t>
+        </is>
+      </c>
+      <c r="B871" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C871" s="9" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="D871" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E871" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F871" s="9" t="n"/>
+      <c r="G871" s="9" t="n"/>
+      <c r="H871" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I871" s="9" t="n">
+        <v>1021.4</v>
+      </c>
+      <c r="J871" s="9" t="n">
+        <v>2059.6</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T10:00</t>
+        </is>
+      </c>
+      <c r="B872" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C872" s="8" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="D872" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="E872" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F872" s="8" t="n"/>
+      <c r="G872" s="8" t="n"/>
+      <c r="H872" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I872" s="8" t="n">
+        <v>1021.3</v>
+      </c>
+      <c r="J872" s="8" t="n">
+        <v>2648.1</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T11:00</t>
+        </is>
+      </c>
+      <c r="B873" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C873" s="9" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="D873" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="E873" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F873" s="9" t="n"/>
+      <c r="G873" s="9" t="n"/>
+      <c r="H873" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I873" s="9" t="n">
+        <v>1021.2</v>
+      </c>
+      <c r="J873" s="9" t="n">
+        <v>3134.2</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T12:00</t>
+        </is>
+      </c>
+      <c r="B874" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C874" s="8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D874" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E874" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F874" s="8" t="n"/>
+      <c r="G874" s="8" t="n"/>
+      <c r="H874" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I874" s="8" t="n">
+        <v>1021</v>
+      </c>
+      <c r="J874" s="8" t="n">
+        <v>3383.7</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T13:00</t>
+        </is>
+      </c>
+      <c r="B875" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C875" s="9" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="D875" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="E875" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F875" s="9" t="n"/>
+      <c r="G875" s="9" t="n"/>
+      <c r="H875" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I875" s="9" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J875" s="9" t="n">
+        <v>3521.7</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T14:00</t>
+        </is>
+      </c>
+      <c r="B876" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C876" s="8" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="D876" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E876" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F876" s="8" t="n"/>
+      <c r="G876" s="8" t="n"/>
+      <c r="H876" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I876" s="8" t="n">
+        <v>1020.1</v>
+      </c>
+      <c r="J876" s="8" t="n">
+        <v>3418.8</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T15:00</t>
+        </is>
+      </c>
+      <c r="B877" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C877" s="9" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="D877" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="E877" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F877" s="9" t="n"/>
+      <c r="G877" s="9" t="n"/>
+      <c r="H877" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I877" s="9" t="n">
+        <v>1019.4</v>
+      </c>
+      <c r="J877" s="9" t="n">
+        <v>3174.2</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T16:00</t>
+        </is>
+      </c>
+      <c r="B878" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C878" s="8" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="D878" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="E878" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F878" s="8" t="n"/>
+      <c r="G878" s="8" t="n"/>
+      <c r="H878" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I878" s="8" t="n">
+        <v>1018.9</v>
+      </c>
+      <c r="J878" s="8" t="n">
+        <v>2722.9</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T17:00</t>
+        </is>
+      </c>
+      <c r="B879" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C879" s="9" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="D879" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="E879" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F879" s="9" t="n"/>
+      <c r="G879" s="9" t="n"/>
+      <c r="H879" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I879" s="9" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J879" s="9" t="n">
+        <v>2015.4</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T18:00</t>
+        </is>
+      </c>
+      <c r="B880" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C880" s="8" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="D880" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E880" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F880" s="8" t="n"/>
+      <c r="G880" s="8" t="n"/>
+      <c r="H880" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I880" s="8" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="J880" s="8" t="n">
+        <v>1455.3</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T19:00</t>
+        </is>
+      </c>
+      <c r="B881" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C881" s="9" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="D881" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="E881" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F881" s="9" t="n"/>
+      <c r="G881" s="9" t="n"/>
+      <c r="H881" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I881" s="9" t="n">
+        <v>1018.6</v>
+      </c>
+      <c r="J881" s="9" t="n">
+        <v>764.6</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T20:00</t>
+        </is>
+      </c>
+      <c r="B882" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C882" s="8" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="D882" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E882" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F882" s="8" t="n"/>
+      <c r="G882" s="8" t="n"/>
+      <c r="H882" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I882" s="8" t="n">
+        <v>1019.1</v>
+      </c>
+      <c r="J882" s="8" t="n">
+        <v>191.8</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T21:00</t>
+        </is>
+      </c>
+      <c r="B883" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C883" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D883" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="E883" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F883" s="9" t="n"/>
+      <c r="G883" s="9" t="n"/>
+      <c r="H883" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I883" s="9" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J883" s="9" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-11T22:00</t>
+        </is>
+      </c>
+      <c r="B884" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C884" s="8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D884" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="E884" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F884" s="8" t="n"/>
+      <c r="G884" s="8" t="n"/>
+      <c r="H884" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I884" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J884" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11T23:00</t>
+        </is>
+      </c>
+      <c r="B885" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C885" s="9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D885" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="E885" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F885" s="9" t="n"/>
+      <c r="G885" s="9" t="n"/>
+      <c r="H885" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I885" s="9" t="n">
+        <v>1020.6</v>
+      </c>
+      <c r="J885" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
climate data: 2026-06-12 04:52 UTC
</commit_message>
<xml_diff>
--- a/data/climate_guimaraes.xlsx
+++ b/data/climate_guimaraes.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J885"/>
+  <dimension ref="A1:J890"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="6" min="1" max="1"/>
@@ -29772,6 +29772,176 @@
         <v>0</v>
       </c>
     </row>
+    <row r="886">
+      <c r="A886" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-12T00:00</t>
+        </is>
+      </c>
+      <c r="B886" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C886" s="8" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D886" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="E886" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F886" s="8" t="n"/>
+      <c r="G886" s="8" t="n"/>
+      <c r="H886" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I886" s="8" t="n">
+        <v>1020.5</v>
+      </c>
+      <c r="J886" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12T01:00</t>
+        </is>
+      </c>
+      <c r="B887" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C887" s="9" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="D887" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E887" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F887" s="9" t="n"/>
+      <c r="G887" s="9" t="n"/>
+      <c r="H887" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I887" s="9" t="n">
+        <v>1020.3</v>
+      </c>
+      <c r="J887" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-12T02:00</t>
+        </is>
+      </c>
+      <c r="B888" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C888" s="8" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="D888" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E888" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F888" s="8" t="n"/>
+      <c r="G888" s="8" t="n"/>
+      <c r="H888" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I888" s="8" t="n">
+        <v>1019.8</v>
+      </c>
+      <c r="J888" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12T03:00</t>
+        </is>
+      </c>
+      <c r="B889" s="9" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C889" s="9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="D889" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="E889" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F889" s="9" t="n"/>
+      <c r="G889" s="9" t="n"/>
+      <c r="H889" s="9" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I889" s="9" t="n">
+        <v>1020.2</v>
+      </c>
+      <c r="J889" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-12T04:00</t>
+        </is>
+      </c>
+      <c r="B890" s="8" t="inlineStr">
+        <is>
+          <t>Guimarães</t>
+        </is>
+      </c>
+      <c r="C890" s="8" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="D890" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="E890" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F890" s="8" t="n"/>
+      <c r="G890" s="8" t="n"/>
+      <c r="H890" s="8" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+      <c r="I890" s="8" t="n">
+        <v>1020.4</v>
+      </c>
+      <c r="J890" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>